<commit_message>
Mettre à jour la bibliothèque Excel au 1er septembre 2026
</commit_message>
<xml_diff>
--- a/data/BibliothèquePrompt.xlsx
+++ b/data/BibliothèquePrompt.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00_Nexellia\04_PRESTATIONS\Valeurs &amp; Talents\Session-2\20260826-27\Prompt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00_Nexellia\04_PRESTATIONS\Valeurs &amp; Talents\BibliothèquePrompt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{716DE54F-3FBB-4338-84E8-00E3E68720EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87B3E938-733D-44EE-9FC9-F1994C6C5E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22740" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="_Data" sheetId="2" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">_Data!$A$1:$P$48</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="386">
   <si>
     <t>Nom</t>
   </si>
@@ -330,9 +333,6 @@
   </si>
   <si>
     <t>Avoir un contenu à faire évaluer.</t>
-  </si>
-  <si>
-    <t>Choix du Dispositif Pédagogique</t>
   </si>
   <si>
     <t>## Rôle
@@ -684,9 +684,6 @@
     <t>Aucun.</t>
   </si>
   <si>
-    <t xml:space="preserve">Création de chaque séquence de formation </t>
-  </si>
-  <si>
     <t>## Rôle
 Tu es un assistant pédagogique intelligent, expert en ingénierie de formation professionnelle, parfaitement à jour sur les exigences du référentiel Qualiopi, la pédagogie des adultes (andragogie), l'inclusion, la ludopédagogie, et l'usage de l'IA en formation. Tu maîtrises les principes du format 3A (Appel – Apport – Ancrage) et tu es capable de proposer des solutions pédagogiques créatives et pertinentes tout en tenant compte des contraintes spécifiques (présentiel/distanciel, inclusion, durée, etc.).
 ## Compétences
@@ -738,9 +735,6 @@
     <t>{programme_formation}</t>
   </si>
   <si>
-    <t>Création Livret Stagiaire</t>
-  </si>
-  <si>
     <t>## Rôle
 Tu es un expert en pédagogie de la formation professionnelle, certifié Qualiopi, spécialiste de l'andragogie, de la ludopédagogie, de l'inclusion (handicap, troubles DYS, PMR, daltonisme) et de l'IA en formation.
 ## Objectif
@@ -813,9 +807,6 @@
   </si>
   <si>
     <t>Avoir une idée vague du public cible.</t>
-  </si>
-  <si>
-    <t>Déroulé Pédagogique &amp; Objectifs SMART</t>
   </si>
   <si>
     <t>## Rôle
@@ -1176,9 +1167,6 @@
     <t>Avoir eu une conversation avec l'IA aboutissant à un bon résultat.</t>
   </si>
   <si>
-    <t>Programme Qualiopi (Digiforma)</t>
-  </si>
-  <si>
     <t>## Rôle
 Tu es un expert en ingénierie pédagogique, maîtrisant parfaitement les exigences du référentiel Qualiopi (notamment les indicateurs 1 et 2) et les formats attendus dans l'outil Digiforma. Tu es aussi expert graphiste, designer et tu sais respecter au mieux les chartes graphiques des templates qu'on te met en pièce jointe.
 ## Objectif
@@ -1494,9 +1482,6 @@
     <t>V1 - S2 2026</t>
   </si>
   <si>
-    <t>Prompt créateur d’une commande Memory</t>
-  </si>
-  <si>
     <t>Toutes</t>
   </si>
   <si>
@@ -1518,9 +1503,6 @@
     <t>C2; C8</t>
   </si>
   <si>
-    <t>Prompt 1_ Les trucs et astuces pour avoir des réponses de qualité_la fonction memory</t>
-  </si>
-  <si>
     <t>ChatGPT, Gemini</t>
   </si>
   <si>
@@ -1533,12 +1515,6 @@
     <t>Le prompt créateur d’assistant</t>
   </si>
   <si>
-    <t>Prompt 1: Focus sur les prompts permettant de continuer à améliorer ses supports de formation</t>
-  </si>
-  <si>
-    <t>Prompt 2_ Les trucs et astuces pour avoir des réponses de qualité_la fonction memory</t>
-  </si>
-  <si>
     <t>Le prompt Scamper</t>
   </si>
   <si>
@@ -1551,16 +1527,10 @@
     <t>C3; C8</t>
   </si>
   <si>
-    <t>Le prompt permettant de générer le bon programme de formation au format Qualiopi – version Genspark</t>
-  </si>
-  <si>
     <t>Genspark</t>
   </si>
   <si>
     <t>Prompt pour la recherche approfondie</t>
-  </si>
-  <si>
-    <t>Le prompt créateur de programme</t>
   </si>
   <si>
     <t>Jour3_Sequence2</t>
@@ -1773,28 +1743,6 @@
   </si>
   <si>
     <t>## Rôle
-Tu es un expert en ingénierie pédagogique, maîtrisant parfaitement les exigences du référentiel Qualiopi (notamment les indicateurs 1 et 2) et les formats attendus dans l'outil Digiforma. Tu es aussi expert graphiste, designer, et tu sais respecter au mieux les chartes graphiques des templates qu'on te met en pièce jointe.
-## Objectif
-Construire un programme de formation au bon format.
-## Contraintes
-1. Tu reçois en entrée :
-   - Un brief de formation (en fichier joint)
-   - Un template de programme (modèle de l'entreprise, conforme Digiforma/Qualiopi) au format .pptx, format A4 portrait, police Calibri, corps de texte noir, titres en vert #94c11f
-2. À partir de ces deux documents :
-   - Tu complètes intégralement le programme de formation dans le respect strict du modèle fourni
-   - Tu respectes les titres, l'ordre, le vocabulaire et la mise en forme du template
-   - Tu n'inventes rien : tu t'appuies uniquement sur le brief client, sauf mention explicite t'autorisant à compléter certains points
-3. Tu produis un livrable :
-   - Une diapositive reprenant fidèlement la mise en page du modèle initial, avec les contenus insérés aux bons endroits
-4. Avant de rendre, tu vérifies que :
-   - Le programme est cohérent, synthétique et structuré
-   - Il contient les objectifs pédagogiques, les modalités d'évaluation, le public cible, les prérequis, la durée, la progression pédagogique, etc.
-   - Il respecte les critères de clarté, de lisibilité et de pertinence Qualiopi
-⚠️ En cas de doute ou d'information manquante dans le brief, indique-le dans le programme entre crochets [à compléter] sans inventer.
-À présent, génère le programme à partir des deux fichiers joints.</t>
-  </si>
-  <si>
-    <t>## Rôle
 Agis en tant que formateur expérimenté en entreprise et spécialiste du management.
 ## Objectif
 Je cherche à construire une offre et une formation sur le thème du management à distance et la gestion des équipes hybrides (mix présentiel et distanciel).
@@ -2096,6 +2044,127 @@
   </si>
   <si>
     <t>Micro-learning, Audio, Consolidation mémorielle</t>
+  </si>
+  <si>
+    <t>Création plaquette de présentation</t>
+  </si>
+  <si>
+    <t>Créateur d’une commande Memory</t>
+  </si>
+  <si>
+    <t>Memory - Générer un prompt pour une image</t>
+  </si>
+  <si>
+    <t>Améliorer ses supports de formation</t>
+  </si>
+  <si>
+    <t>Memory - Création veille</t>
+  </si>
+  <si>
+    <t>3_Choix du Dispositif Pédagogique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5_Création de chaque séquence de formation </t>
+  </si>
+  <si>
+    <t>7_Création Livret Stagiaire</t>
+  </si>
+  <si>
+    <t>7.1_Création Livret Stagiaire_HTML</t>
+  </si>
+  <si>
+    <t># Prompt — Transformation de support de formation en livret HTML interactif
+## Rôle
+Tu es un expert en développement front-end et en design pédagogique.
+Tu maîtrises la création d'interfaces HTML/CSS/JS élégantes, accessibles
+et fonctionnelles, pensées pour un usage autonome en formation.
+## Objectif
+Transformer le document Word "Support" (support participant de formation)
+en un **livret numérique dynamique au format HTML**, utilisable directement
+par chaque stagiaire depuis son navigateur.
+Le livret doit permettre au stagiaire de :
+- **Naviguer** rapidement vers la section qui l'intéresse via un menu latéral fixe
+- **Copier en un clic** les instructions/prompts présents dans le livret
+  pour les coller dans son outil IA
+- **Saisir ses réponses et commentaires** dans des zones d'écriture dédiées
+- **Joindre des fichiers** (captures, PDF, images) illustrant ses résultats
+- **Exporter son travail** au format PDF via un bouton "Enregistrer sous"
+## Contraintes
+### Contenu éditables
+- Les zones de saisie stagiaire ("espace stagiaire") sont **strictement limitées**
+  aux sections intitulées **"À vous de jouer"** dans le livret source
+- Le reste du contenu est en lecture seule, non modifiable
+### Design
+- Respecter la charte graphique (couleurs, typographie, style)
+- Interface **aérée, graphique et professionnelle**
+- Lisibilité optimale : hiérarchie visuelle claire, espaces généreux
+### Technique
+- Format : **fichier HTML unique autonome** (tout embarqué : CSS + JS)
+- Menu de navigation : **sidebar fixe à gauche**, avec ancres vers chaque section
+- Bouton "copier" : présent sous chaque bloc instruction/prompt
+- Zones d'upload : accepter images, PDF, DOCX
+- Export PDF : déclenché par un bouton dédié, via `window.print()` ou librairie JS
+- Compatibilité : navigateurs modernes (Chrome, Edge, Firefox), sans installation</t>
+  </si>
+  <si>
+    <t>4_Déroulé Pédagogique &amp; Objectifs SMART</t>
+  </si>
+  <si>
+    <t>6_Programme Qualiopi (Digiforma)</t>
+  </si>
+  <si>
+    <t>## Rôle
+Tu es un expert en ingénierie pédagogique, maîtrisant parfaitement les exigences du référentiel Qualiopi (notamment les indicateurs 1 et 2) et les formats attendus dans l'outil Digiforma. Tu es aussi expert graphiste, designer, et tu sais respecter au mieux les chartes graphiques des templates qu'on te met en pièce jointe.
+## Objectif
+Construire un programme de formation au bon format.
+## Contraintes
+1. Tu reçois en entrée :
+   - Un brief de formation (en fichier joint)
+   - Un template de programme (modèle de l'entreprise, conforme Digiforma/Qualiopi) au format .pptx, format A4 portrait, police Calibri, corps de texte noir
+2. À partir de ces deux documents :
+   - Tu complètes intégralement le programme de formation dans le respect strict du modèle fourni
+   - Tu respectes les titres, l'ordre, le vocabulaire et la mise en forme du template
+   - Tu n'inventes rien : tu t'appuies uniquement sur le brief client, sauf mention explicite t'autorisant à compléter certains points
+3. Tu produis un livrable :
+   - Une diapositive reprenant fidèlement la mise en page du modèle initial, avec les contenus insérés aux bons endroits
+4. Avant de rendre, tu vérifies que :
+   - Le programme est cohérent, synthétique et structuré
+   - Il contient les objectifs pédagogiques, les modalités d'évaluation, le public cible, les prérequis, la durée, la progression pédagogique, etc.
+   - Il respecte les critères de clarté, de lisibilité et de pertinence Qualiopi
+⚠️ En cas de doute ou d'information manquante dans le brief, indique-le dans le programme entre crochets [à compléter] sans inventer.
+À présent, génère le programme à partir des deux fichiers joints.</t>
+  </si>
+  <si>
+    <t>2.5_Le prompt permettant de générer le bon programme de formation au format Qualiopi</t>
+  </si>
+  <si>
+    <t>2.5_Le prompt créateur de programme</t>
+  </si>
+  <si>
+    <t>## Rôle
+Tu es un copywriter expert en marketing de la formation professionnelle. Tu maîtrises les structures persuasives orientées transformation (avant/après), la rédaction centrée bénéfices apprenants, et les codes visuels des plaquettes commerciales B2B.
+## Objectif
+Générer le contenu complet d'une plaquette de présentation commerciale pour le programme de formation fourni, afin de donner envie au lecteur de s'inscrire dès le premier jour, en utilisant le design système pour la mise en forme.
+## Contraintes
+- Longueur totale : entre 350 et 500 mots répartis sur les sections ci-dessous
+- Ton : [PROFESSIONNEL / DIRECT / INSPIRANT] — jamais condescendant, jamais vague
+- Langue : français, niveau C1, phrases actives et courtes
+- Interdire : jargon creux (« booster vos compétences »), promesses non vérifiables, adjectifs vides (« innovant », « révolutionnaire »)
+- Inclure : des formulations factuelles, des bénéfices concrets mesurables, des verbes d'action
+## Format de sortie
+Produis une plaquette avec ces éléments :
+1. Accroche (2 phrases max)
+   Une entrée en matière qui nomme le problème réel ou la tension que vit [PROFIL_CIBLE] avant la formation.
+2. Ce que vous allez apprendre — les éléments clés du programme
+   Tableau ou liste structurée des modules/compétences clés. Format : Module → Ce que vous maîtrisez à la sortie.
+3. Vos gains concrets
+   3 à 5 bénéfices formulés en "Vous serez capable de..." ou "À l'issue de cette formation, vous..." — orientés résultats mesurables, pas sur les contenus.
+4. La transformation apportée
+   Bloc "Avant / Après" en 2 colonnes : ce que vit l'apprenant avant la formation vs. ce qu'il vit après. 3 lignes minimum.
+5. Pour qui ce programme est-il fait ?
+   Critères d'adéquation positifs (profils qui bénéficient pleinement) et 1 critère d'exclusion (pour qui ce n'est PAS fait — renforce la crédibilité).
+6. Appel à l'action
+   1 phrase de clôture forte + 3 micro-CTA au choix : télécharger le programme, contacter un conseiller, s'inscrire directement. Format web-ready (texte de bouton + URL placeholder).</t>
   </si>
 </sst>
 </file>
@@ -2141,7 +2210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2163,9 +2232,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2405,6 +2471,9 @@
   <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </wetp:taskpane>
 </wetp:taskpanes>
 </file>
 
@@ -2422,13 +2491,28 @@
 </we:webextension>
 </file>
 
+<file path=xl/webextensions/webextension2.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{503296D5-C983-43BB-865D-CB288D8A389B}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="fr-FR" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;c4d73f7a-0a20-4ea8-b5d1-cc9b342408fe&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P46"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="40.46484375" customWidth="1"/>
-    <col min="2" max="2" width="255" customWidth="1"/>
+    <col min="2" max="2" width="120.73046875" customWidth="1"/>
+    <col min="7" max="7" width="38" customWidth="1"/>
     <col min="14" max="16" width="16" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2476,10 +2560,10 @@
         <v>13</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
@@ -2523,10 +2607,10 @@
         <v>26</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>27</v>
@@ -2573,10 +2657,10 @@
         <v>39</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P3" s="3" t="s">
         <v>27</v>
@@ -2623,16 +2707,16 @@
         <v>50</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P4" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:16" ht="384.75" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -2673,16 +2757,16 @@
         <v>58</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P5" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="171" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:16" ht="242.25" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>59</v>
       </c>
@@ -2723,10 +2807,10 @@
         <v>69</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P6" s="3" t="s">
         <v>27</v>
@@ -2734,66 +2818,66 @@
     </row>
     <row r="7" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
+        <v>375</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="C7" t="s">
         <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E7" t="s">
         <v>32</v>
       </c>
       <c r="F7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" t="s">
         <v>73</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>74</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>75</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>76</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>77</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>78</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>79</v>
       </c>
-      <c r="M7" t="s">
-        <v>80</v>
-      </c>
       <c r="N7" s="3" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P7" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="327.75" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E8" t="s">
         <v>63</v>
@@ -2802,31 +2886,31 @@
         <v>19</v>
       </c>
       <c r="G8" t="s">
+        <v>82</v>
+      </c>
+      <c r="H8" t="s">
         <v>83</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>84</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>85</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>86</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>87</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>88</v>
       </c>
-      <c r="M8" t="s">
-        <v>89</v>
-      </c>
       <c r="N8" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P8" s="3" t="s">
         <v>27</v>
@@ -2834,10 +2918,10 @@
     </row>
     <row r="9" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="C9" t="s">
         <v>16</v>
@@ -2852,48 +2936,48 @@
         <v>19</v>
       </c>
       <c r="G9" t="s">
+        <v>91</v>
+      </c>
+      <c r="H9" t="s">
         <v>92</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>93</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>94</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>95</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>96</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>97</v>
       </c>
-      <c r="M9" t="s">
-        <v>98</v>
-      </c>
       <c r="N9" s="3" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="P9" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="171" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
+        <v>98</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="C10" t="s">
         <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E10" t="s">
         <v>32</v>
@@ -2905,45 +2989,45 @@
         <v>33</v>
       </c>
       <c r="H10" t="s">
+        <v>101</v>
+      </c>
+      <c r="I10" t="s">
         <v>102</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>103</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>104</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>105</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>106</v>
       </c>
-      <c r="M10" t="s">
-        <v>107</v>
-      </c>
       <c r="N10" s="3" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P10" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="114" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:16" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="C11" t="s">
         <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E11" t="s">
         <v>63</v>
@@ -2952,42 +3036,42 @@
         <v>19</v>
       </c>
       <c r="G11" t="s">
+        <v>109</v>
+      </c>
+      <c r="H11" t="s">
         <v>110</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>111</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>112</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>113</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>114</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>115</v>
       </c>
-      <c r="M11" t="s">
-        <v>116</v>
-      </c>
       <c r="N11" s="3" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="P11" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="114" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>118</v>
       </c>
       <c r="C12" t="s">
         <v>61</v>
@@ -3005,28 +3089,28 @@
         <v>20</v>
       </c>
       <c r="H12" t="s">
+        <v>118</v>
+      </c>
+      <c r="I12" t="s">
         <v>119</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>120</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>121</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>122</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>123</v>
       </c>
-      <c r="M12" t="s">
-        <v>124</v>
-      </c>
       <c r="N12" s="3" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P12" s="3" t="s">
         <v>27</v>
@@ -3034,49 +3118,49 @@
     </row>
     <row r="13" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>126</v>
       </c>
       <c r="C13" t="s">
         <v>30</v>
       </c>
       <c r="D13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E13" t="s">
         <v>32</v>
       </c>
       <c r="F13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G13" t="s">
         <v>33</v>
       </c>
       <c r="H13" t="s">
+        <v>128</v>
+      </c>
+      <c r="I13" t="s">
         <v>129</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>130</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>131</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>132</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>133</v>
       </c>
-      <c r="M13" t="s">
-        <v>134</v>
-      </c>
       <c r="N13" s="3" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P13" s="3" t="s">
         <v>27</v>
@@ -3084,107 +3168,107 @@
     </row>
     <row r="14" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>135</v>
+        <v>376</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C14" t="s">
         <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E14" t="s">
         <v>18</v>
       </c>
       <c r="F14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" t="s">
         <v>73</v>
       </c>
-      <c r="G14" t="s">
-        <v>74</v>
-      </c>
       <c r="H14" t="s">
+        <v>135</v>
+      </c>
+      <c r="I14" t="s">
+        <v>136</v>
+      </c>
+      <c r="J14" t="s">
         <v>137</v>
       </c>
-      <c r="I14" t="s">
+      <c r="K14" t="s">
         <v>138</v>
       </c>
-      <c r="J14" t="s">
+      <c r="L14" t="s">
         <v>139</v>
       </c>
-      <c r="K14" t="s">
-        <v>140</v>
-      </c>
-      <c r="L14" t="s">
-        <v>141</v>
-      </c>
       <c r="N14" s="3" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P14" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="313.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:16" ht="342" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>142</v>
+        <v>377</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C15" t="s">
         <v>42</v>
       </c>
       <c r="D15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E15" t="s">
         <v>32</v>
       </c>
       <c r="F15" t="s">
+        <v>72</v>
+      </c>
+      <c r="G15" t="s">
         <v>73</v>
       </c>
-      <c r="G15" t="s">
-        <v>74</v>
-      </c>
       <c r="H15" t="s">
+        <v>141</v>
+      </c>
+      <c r="I15" t="s">
+        <v>142</v>
+      </c>
+      <c r="J15" t="s">
+        <v>143</v>
+      </c>
+      <c r="K15" t="s">
         <v>144</v>
       </c>
-      <c r="I15" t="s">
+      <c r="L15" t="s">
         <v>145</v>
       </c>
-      <c r="J15" t="s">
+      <c r="M15" t="s">
         <v>146</v>
       </c>
-      <c r="K15" t="s">
-        <v>147</v>
-      </c>
-      <c r="L15" t="s">
-        <v>148</v>
-      </c>
-      <c r="M15" t="s">
-        <v>149</v>
-      </c>
       <c r="N15" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P15" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:16" ht="228" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C16" t="s">
         <v>30</v>
@@ -3196,34 +3280,34 @@
         <v>32</v>
       </c>
       <c r="F16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G16" t="s">
+        <v>149</v>
+      </c>
+      <c r="H16" t="s">
+        <v>150</v>
+      </c>
+      <c r="I16" t="s">
+        <v>151</v>
+      </c>
+      <c r="J16" t="s">
         <v>152</v>
       </c>
-      <c r="H16" t="s">
+      <c r="K16" t="s">
         <v>153</v>
       </c>
-      <c r="I16" t="s">
+      <c r="L16" t="s">
         <v>154</v>
       </c>
-      <c r="J16" t="s">
+      <c r="M16" t="s">
         <v>155</v>
       </c>
-      <c r="K16" t="s">
-        <v>156</v>
-      </c>
-      <c r="L16" t="s">
-        <v>157</v>
-      </c>
-      <c r="M16" t="s">
-        <v>158</v>
-      </c>
       <c r="N16" s="3" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P16" s="3" t="s">
         <v>27</v>
@@ -3231,49 +3315,49 @@
     </row>
     <row r="17" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>159</v>
+        <v>380</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C17" t="s">
         <v>16</v>
       </c>
       <c r="D17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E17" t="s">
         <v>32</v>
       </c>
       <c r="F17" t="s">
+        <v>72</v>
+      </c>
+      <c r="G17" t="s">
         <v>73</v>
       </c>
-      <c r="G17" t="s">
-        <v>74</v>
-      </c>
       <c r="H17" t="s">
+        <v>157</v>
+      </c>
+      <c r="I17" t="s">
+        <v>158</v>
+      </c>
+      <c r="J17" t="s">
+        <v>159</v>
+      </c>
+      <c r="K17" t="s">
+        <v>160</v>
+      </c>
+      <c r="L17" t="s">
         <v>161</v>
       </c>
-      <c r="I17" t="s">
+      <c r="M17" t="s">
         <v>162</v>
       </c>
-      <c r="J17" t="s">
-        <v>163</v>
-      </c>
-      <c r="K17" t="s">
-        <v>164</v>
-      </c>
-      <c r="L17" t="s">
-        <v>165</v>
-      </c>
-      <c r="M17" t="s">
-        <v>166</v>
-      </c>
       <c r="N17" s="3" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>27</v>
@@ -3281,49 +3365,49 @@
     </row>
     <row r="18" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C18" t="s">
         <v>16</v>
       </c>
       <c r="D18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E18" t="s">
         <v>32</v>
       </c>
       <c r="F18" t="s">
+        <v>72</v>
+      </c>
+      <c r="G18" t="s">
         <v>73</v>
       </c>
-      <c r="G18" t="s">
-        <v>74</v>
-      </c>
       <c r="H18" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="I18" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="J18" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="K18" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L18" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M18" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P18" s="3" t="s">
         <v>27</v>
@@ -3331,10 +3415,10 @@
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B19" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C19" t="s">
         <v>42</v>
@@ -3349,31 +3433,31 @@
         <v>43</v>
       </c>
       <c r="G19" t="s">
+        <v>171</v>
+      </c>
+      <c r="H19" t="s">
+        <v>172</v>
+      </c>
+      <c r="I19" t="s">
+        <v>173</v>
+      </c>
+      <c r="J19" t="s">
+        <v>174</v>
+      </c>
+      <c r="K19" t="s">
+        <v>86</v>
+      </c>
+      <c r="L19" t="s">
         <v>175</v>
       </c>
-      <c r="H19" t="s">
+      <c r="M19" t="s">
         <v>176</v>
       </c>
-      <c r="I19" t="s">
-        <v>177</v>
-      </c>
-      <c r="J19" t="s">
-        <v>178</v>
-      </c>
-      <c r="K19" t="s">
-        <v>87</v>
-      </c>
-      <c r="L19" t="s">
-        <v>179</v>
-      </c>
-      <c r="M19" t="s">
-        <v>180</v>
-      </c>
       <c r="N19" s="3" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="P19" s="3" t="s">
         <v>27</v>
@@ -3381,10 +3465,10 @@
     </row>
     <row r="20" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C20" t="s">
         <v>42</v>
@@ -3399,48 +3483,48 @@
         <v>19</v>
       </c>
       <c r="G20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H20" t="s">
+        <v>179</v>
+      </c>
+      <c r="I20" t="s">
+        <v>180</v>
+      </c>
+      <c r="J20" t="s">
+        <v>181</v>
+      </c>
+      <c r="K20" t="s">
+        <v>86</v>
+      </c>
+      <c r="L20" t="s">
+        <v>182</v>
+      </c>
+      <c r="M20" t="s">
         <v>183</v>
       </c>
-      <c r="I20" t="s">
-        <v>184</v>
-      </c>
-      <c r="J20" t="s">
-        <v>185</v>
-      </c>
-      <c r="K20" t="s">
-        <v>87</v>
-      </c>
-      <c r="L20" t="s">
-        <v>186</v>
-      </c>
-      <c r="M20" t="s">
-        <v>187</v>
-      </c>
       <c r="N20" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P20" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="228" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:16" ht="270.75" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C21" t="s">
         <v>30</v>
       </c>
       <c r="D21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E21" t="s">
         <v>32</v>
@@ -3452,28 +3536,28 @@
         <v>33</v>
       </c>
       <c r="H21" t="s">
+        <v>186</v>
+      </c>
+      <c r="I21" t="s">
+        <v>187</v>
+      </c>
+      <c r="J21" t="s">
+        <v>188</v>
+      </c>
+      <c r="K21" t="s">
+        <v>189</v>
+      </c>
+      <c r="L21" t="s">
         <v>190</v>
       </c>
-      <c r="I21" t="s">
+      <c r="M21" t="s">
         <v>191</v>
       </c>
-      <c r="J21" t="s">
-        <v>192</v>
-      </c>
-      <c r="K21" t="s">
-        <v>193</v>
-      </c>
-      <c r="L21" t="s">
-        <v>194</v>
-      </c>
-      <c r="M21" t="s">
-        <v>195</v>
-      </c>
       <c r="N21" s="3" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P21" s="3" t="s">
         <v>27</v>
@@ -3481,110 +3565,110 @@
     </row>
     <row r="22" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C22" t="s">
         <v>30</v>
       </c>
       <c r="D22" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E22" t="s">
         <v>32</v>
       </c>
       <c r="F22" t="s">
+        <v>72</v>
+      </c>
+      <c r="G22" t="s">
         <v>73</v>
       </c>
-      <c r="G22" t="s">
-        <v>74</v>
-      </c>
       <c r="H22" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="I22" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="J22" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="K22" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="L22" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M22" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P22" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C23" t="s">
         <v>30</v>
       </c>
       <c r="D23" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E23" t="s">
         <v>32</v>
       </c>
       <c r="F23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G23" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="H23" t="s">
+        <v>200</v>
+      </c>
+      <c r="I23" t="s">
+        <v>201</v>
+      </c>
+      <c r="J23" t="s">
+        <v>202</v>
+      </c>
+      <c r="K23" t="s">
+        <v>77</v>
+      </c>
+      <c r="L23" t="s">
+        <v>203</v>
+      </c>
+      <c r="M23" t="s">
         <v>204</v>
       </c>
-      <c r="I23" t="s">
-        <v>205</v>
-      </c>
-      <c r="J23" t="s">
-        <v>206</v>
-      </c>
-      <c r="K23" t="s">
-        <v>78</v>
-      </c>
-      <c r="L23" t="s">
-        <v>207</v>
-      </c>
-      <c r="M23" t="s">
-        <v>208</v>
-      </c>
       <c r="N23" s="3" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P23" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:16" ht="57" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="C24" t="s">
         <v>30</v>
@@ -3602,39 +3686,39 @@
         <v>20</v>
       </c>
       <c r="H24" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="I24" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="J24" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="K24" t="s">
         <v>24</v>
       </c>
       <c r="L24" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="M24" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P24" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="384.75" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:16" ht="399" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>216</v>
+        <v>381</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C25" t="s">
         <v>42</v>
@@ -3646,84 +3730,84 @@
         <v>63</v>
       </c>
       <c r="F25" t="s">
+        <v>72</v>
+      </c>
+      <c r="G25" t="s">
         <v>73</v>
       </c>
-      <c r="G25" t="s">
-        <v>74</v>
-      </c>
       <c r="H25" t="s">
+        <v>213</v>
+      </c>
+      <c r="I25" t="s">
+        <v>214</v>
+      </c>
+      <c r="J25" t="s">
+        <v>215</v>
+      </c>
+      <c r="K25" t="s">
+        <v>216</v>
+      </c>
+      <c r="L25" t="s">
+        <v>217</v>
+      </c>
+      <c r="M25" t="s">
         <v>218</v>
       </c>
-      <c r="I25" t="s">
-        <v>219</v>
-      </c>
-      <c r="J25" t="s">
-        <v>220</v>
-      </c>
-      <c r="K25" t="s">
-        <v>221</v>
-      </c>
-      <c r="L25" t="s">
-        <v>222</v>
-      </c>
-      <c r="M25" t="s">
-        <v>223</v>
-      </c>
       <c r="N25" s="3" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P25" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="342" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="C26" t="s">
         <v>61</v>
       </c>
       <c r="D26" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="E26" t="s">
         <v>32</v>
       </c>
       <c r="F26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G26" t="s">
+        <v>222</v>
+      </c>
+      <c r="H26" t="s">
+        <v>223</v>
+      </c>
+      <c r="I26" t="s">
+        <v>224</v>
+      </c>
+      <c r="J26" t="s">
+        <v>225</v>
+      </c>
+      <c r="K26" t="s">
+        <v>121</v>
+      </c>
+      <c r="L26" t="s">
+        <v>226</v>
+      </c>
+      <c r="M26" t="s">
         <v>227</v>
       </c>
-      <c r="H26" t="s">
-        <v>228</v>
-      </c>
-      <c r="I26" t="s">
-        <v>229</v>
-      </c>
-      <c r="J26" t="s">
-        <v>230</v>
-      </c>
-      <c r="K26" t="s">
-        <v>122</v>
-      </c>
-      <c r="L26" t="s">
-        <v>231</v>
-      </c>
-      <c r="M26" t="s">
-        <v>232</v>
-      </c>
       <c r="N26" s="3" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="P26" s="3" t="s">
         <v>27</v>
@@ -3731,10 +3815,10 @@
     </row>
     <row r="27" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C27" t="s">
         <v>30</v>
@@ -3746,34 +3830,34 @@
         <v>63</v>
       </c>
       <c r="F27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G27" t="s">
+        <v>230</v>
+      </c>
+      <c r="H27" t="s">
+        <v>231</v>
+      </c>
+      <c r="I27" t="s">
+        <v>232</v>
+      </c>
+      <c r="J27" t="s">
+        <v>233</v>
+      </c>
+      <c r="K27" t="s">
+        <v>86</v>
+      </c>
+      <c r="L27" t="s">
+        <v>234</v>
+      </c>
+      <c r="M27" t="s">
         <v>235</v>
       </c>
-      <c r="H27" t="s">
-        <v>236</v>
-      </c>
-      <c r="I27" t="s">
-        <v>237</v>
-      </c>
-      <c r="J27" t="s">
-        <v>238</v>
-      </c>
-      <c r="K27" t="s">
-        <v>87</v>
-      </c>
-      <c r="L27" t="s">
-        <v>239</v>
-      </c>
-      <c r="M27" t="s">
-        <v>240</v>
-      </c>
       <c r="N27" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O27" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P27" s="3" t="s">
         <v>27</v>
@@ -3781,10 +3865,10 @@
     </row>
     <row r="28" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C28" t="s">
         <v>30</v>
@@ -3796,34 +3880,34 @@
         <v>63</v>
       </c>
       <c r="F28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G28" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="H28" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="I28" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="J28" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="K28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L28" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="M28" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P28" s="3" t="s">
         <v>27</v>
@@ -3831,10 +3915,10 @@
     </row>
     <row r="29" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="C29" t="s">
         <v>30</v>
@@ -3846,45 +3930,45 @@
         <v>32</v>
       </c>
       <c r="F29" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G29" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="H29" t="s">
+        <v>246</v>
+      </c>
+      <c r="I29" t="s">
+        <v>247</v>
+      </c>
+      <c r="J29" t="s">
+        <v>248</v>
+      </c>
+      <c r="K29" t="s">
+        <v>249</v>
+      </c>
+      <c r="L29" t="s">
         <v>250</v>
       </c>
-      <c r="H29" t="s">
+      <c r="M29" t="s">
         <v>251</v>
       </c>
-      <c r="I29" t="s">
-        <v>252</v>
-      </c>
-      <c r="J29" t="s">
-        <v>253</v>
-      </c>
-      <c r="K29" t="s">
-        <v>254</v>
-      </c>
-      <c r="L29" t="s">
-        <v>255</v>
-      </c>
-      <c r="M29" t="s">
-        <v>256</v>
-      </c>
       <c r="N29" s="3" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="P29" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:16" ht="66" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>42</v>
@@ -3896,45 +3980,45 @@
         <v>63</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P30" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>283</v>
+        <v>371</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>42</v>
@@ -3946,45 +4030,45 @@
         <v>32</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
       <c r="M31" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="N31" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="N31" s="3" t="s">
-        <v>286</v>
-      </c>
       <c r="O31" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="P31" s="3" t="s">
         <v>277</v>
-      </c>
-      <c r="P31" s="3" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="32" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>42</v>
@@ -3996,45 +4080,45 @@
         <v>32</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="M32" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="N32" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="N32" s="3" t="s">
-        <v>286</v>
-      </c>
       <c r="O32" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="P32" s="3" t="s">
         <v>277</v>
-      </c>
-      <c r="P32" s="3" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="33" spans="1:16" ht="120" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>16</v>
@@ -4046,45 +4130,45 @@
         <v>32</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="H33" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I33" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="I33" s="2" t="s">
-        <v>94</v>
-      </c>
       <c r="J33" s="2" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="K33" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="L33" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="L33" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="M33" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="P33" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="34" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>291</v>
+        <v>372</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>30</v>
@@ -4096,93 +4180,93 @@
         <v>32</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G34" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N34" s="3" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="35" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="36" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>42</v>
@@ -4194,42 +4278,42 @@
         <v>18</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="37" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>296</v>
+        <v>373</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>60</v>
@@ -4244,10 +4328,10 @@
         <v>63</v>
       </c>
       <c r="F37" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G37" s="6" t="s">
         <v>73</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>20</v>
       </c>
       <c r="H37" s="2" t="s">
         <v>64</v>
@@ -4265,24 +4349,24 @@
         <v>68</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N37" s="3" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="O37" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P37" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>297</v>
+        <v>374</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>30</v>
@@ -4294,145 +4378,145 @@
         <v>32</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N38" s="3" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="O38" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P38" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="39" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="40" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F40" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G40" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="H40" s="2" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="P40" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="41" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>302</v>
+        <v>383</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>322</v>
+        <v>382</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>42</v>
@@ -4444,95 +4528,95 @@
         <v>32</v>
       </c>
       <c r="F41" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G41" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G41" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="H41" s="2" t="s">
-        <v>359</v>
+        <v>347</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>361</v>
+        <v>349</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="42" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>362</v>
+        <v>350</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>363</v>
+        <v>351</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="43" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
-        <v>305</v>
+        <v>384</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>42</v>
@@ -4544,166 +4628,241 @@
         <v>18</v>
       </c>
       <c r="F43" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G43" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="G43" s="6" t="s">
-        <v>74</v>
-      </c>
       <c r="H43" s="2" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>368</v>
+        <v>356</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="O43" s="3" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="P43" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="44" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="6" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M44" s="2"/>
-      <c r="N44" s="3"/>
-      <c r="O44" s="3"/>
+      <c r="N44" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="O44" s="3" t="s">
+        <v>257</v>
+      </c>
       <c r="P44" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="45" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>42</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F45" s="9" t="s">
+      <c r="F45" s="2" t="s">
         <v>43</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>374</v>
+        <v>362</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>376</v>
+        <v>364</v>
+      </c>
+      <c r="N45" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="O45" s="3" t="s">
+        <v>257</v>
       </c>
       <c r="P45" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="46" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A46" s="9" t="s">
-        <v>309</v>
-      </c>
-      <c r="B46" s="10" t="s">
-        <v>327</v>
+      <c r="A46" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>315</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>42</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F46" s="9" t="s">
+      <c r="F46" s="2" t="s">
         <v>43</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H46" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="N46" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="O46" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="P46" s="3" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A47" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A48" t="s">
         <v>378</v>
       </c>
-      <c r="I46" s="2" t="s">
+      <c r="B48" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="J46" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="L46" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="P46" s="3" t="s">
-        <v>282</v>
+      <c r="C48" t="s">
+        <v>42</v>
+      </c>
+      <c r="D48" t="s">
+        <v>126</v>
+      </c>
+      <c r="E48" t="s">
+        <v>32</v>
+      </c>
+      <c r="F48" t="s">
+        <v>72</v>
+      </c>
+      <c r="G48" t="s">
+        <v>73</v>
+      </c>
+      <c r="H48" t="s">
+        <v>141</v>
+      </c>
+      <c r="I48" t="s">
+        <v>142</v>
+      </c>
+      <c r="J48" t="s">
+        <v>143</v>
+      </c>
+      <c r="K48" t="s">
+        <v>144</v>
+      </c>
+      <c r="L48" t="s">
+        <v>145</v>
+      </c>
+      <c r="M48" t="s">
+        <v>146</v>
+      </c>
+      <c r="N48" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="O48" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="P48" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:P48" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Mettre à jour la bibliothèque de prompts au 1er septembre 2026
Publie le nouveau classeur à 47 prompts et déclenche la régénération du site.
</commit_message>
<xml_diff>
--- a/data/BibliothèquePrompt.xlsx
+++ b/data/BibliothèquePrompt.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00_Nexellia\04_PRESTATIONS\Valeurs &amp; Talents\Session-2\20260826-27\Prompt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00_Nexellia\04_PRESTATIONS\Valeurs &amp; Talents\BibliothèquePrompt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{716DE54F-3FBB-4338-84E8-00E3E68720EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87B3E938-733D-44EE-9FC9-F1994C6C5E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22740" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="_Data" sheetId="2" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">_Data!$A$1:$P$48</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="386">
   <si>
     <t>Nom</t>
   </si>
@@ -330,9 +333,6 @@
   </si>
   <si>
     <t>Avoir un contenu à faire évaluer.</t>
-  </si>
-  <si>
-    <t>Choix du Dispositif Pédagogique</t>
   </si>
   <si>
     <t>## Rôle
@@ -684,9 +684,6 @@
     <t>Aucun.</t>
   </si>
   <si>
-    <t xml:space="preserve">Création de chaque séquence de formation </t>
-  </si>
-  <si>
     <t>## Rôle
 Tu es un assistant pédagogique intelligent, expert en ingénierie de formation professionnelle, parfaitement à jour sur les exigences du référentiel Qualiopi, la pédagogie des adultes (andragogie), l'inclusion, la ludopédagogie, et l'usage de l'IA en formation. Tu maîtrises les principes du format 3A (Appel – Apport – Ancrage) et tu es capable de proposer des solutions pédagogiques créatives et pertinentes tout en tenant compte des contraintes spécifiques (présentiel/distanciel, inclusion, durée, etc.).
 ## Compétences
@@ -738,9 +735,6 @@
     <t>{programme_formation}</t>
   </si>
   <si>
-    <t>Création Livret Stagiaire</t>
-  </si>
-  <si>
     <t>## Rôle
 Tu es un expert en pédagogie de la formation professionnelle, certifié Qualiopi, spécialiste de l'andragogie, de la ludopédagogie, de l'inclusion (handicap, troubles DYS, PMR, daltonisme) et de l'IA en formation.
 ## Objectif
@@ -813,9 +807,6 @@
   </si>
   <si>
     <t>Avoir une idée vague du public cible.</t>
-  </si>
-  <si>
-    <t>Déroulé Pédagogique &amp; Objectifs SMART</t>
   </si>
   <si>
     <t>## Rôle
@@ -1176,9 +1167,6 @@
     <t>Avoir eu une conversation avec l'IA aboutissant à un bon résultat.</t>
   </si>
   <si>
-    <t>Programme Qualiopi (Digiforma)</t>
-  </si>
-  <si>
     <t>## Rôle
 Tu es un expert en ingénierie pédagogique, maîtrisant parfaitement les exigences du référentiel Qualiopi (notamment les indicateurs 1 et 2) et les formats attendus dans l'outil Digiforma. Tu es aussi expert graphiste, designer et tu sais respecter au mieux les chartes graphiques des templates qu'on te met en pièce jointe.
 ## Objectif
@@ -1494,9 +1482,6 @@
     <t>V1 - S2 2026</t>
   </si>
   <si>
-    <t>Prompt créateur d’une commande Memory</t>
-  </si>
-  <si>
     <t>Toutes</t>
   </si>
   <si>
@@ -1518,9 +1503,6 @@
     <t>C2; C8</t>
   </si>
   <si>
-    <t>Prompt 1_ Les trucs et astuces pour avoir des réponses de qualité_la fonction memory</t>
-  </si>
-  <si>
     <t>ChatGPT, Gemini</t>
   </si>
   <si>
@@ -1533,12 +1515,6 @@
     <t>Le prompt créateur d’assistant</t>
   </si>
   <si>
-    <t>Prompt 1: Focus sur les prompts permettant de continuer à améliorer ses supports de formation</t>
-  </si>
-  <si>
-    <t>Prompt 2_ Les trucs et astuces pour avoir des réponses de qualité_la fonction memory</t>
-  </si>
-  <si>
     <t>Le prompt Scamper</t>
   </si>
   <si>
@@ -1551,16 +1527,10 @@
     <t>C3; C8</t>
   </si>
   <si>
-    <t>Le prompt permettant de générer le bon programme de formation au format Qualiopi – version Genspark</t>
-  </si>
-  <si>
     <t>Genspark</t>
   </si>
   <si>
     <t>Prompt pour la recherche approfondie</t>
-  </si>
-  <si>
-    <t>Le prompt créateur de programme</t>
   </si>
   <si>
     <t>Jour3_Sequence2</t>
@@ -1773,28 +1743,6 @@
   </si>
   <si>
     <t>## Rôle
-Tu es un expert en ingénierie pédagogique, maîtrisant parfaitement les exigences du référentiel Qualiopi (notamment les indicateurs 1 et 2) et les formats attendus dans l'outil Digiforma. Tu es aussi expert graphiste, designer, et tu sais respecter au mieux les chartes graphiques des templates qu'on te met en pièce jointe.
-## Objectif
-Construire un programme de formation au bon format.
-## Contraintes
-1. Tu reçois en entrée :
-   - Un brief de formation (en fichier joint)
-   - Un template de programme (modèle de l'entreprise, conforme Digiforma/Qualiopi) au format .pptx, format A4 portrait, police Calibri, corps de texte noir, titres en vert #94c11f
-2. À partir de ces deux documents :
-   - Tu complètes intégralement le programme de formation dans le respect strict du modèle fourni
-   - Tu respectes les titres, l'ordre, le vocabulaire et la mise en forme du template
-   - Tu n'inventes rien : tu t'appuies uniquement sur le brief client, sauf mention explicite t'autorisant à compléter certains points
-3. Tu produis un livrable :
-   - Une diapositive reprenant fidèlement la mise en page du modèle initial, avec les contenus insérés aux bons endroits
-4. Avant de rendre, tu vérifies que :
-   - Le programme est cohérent, synthétique et structuré
-   - Il contient les objectifs pédagogiques, les modalités d'évaluation, le public cible, les prérequis, la durée, la progression pédagogique, etc.
-   - Il respecte les critères de clarté, de lisibilité et de pertinence Qualiopi
-⚠️ En cas de doute ou d'information manquante dans le brief, indique-le dans le programme entre crochets [à compléter] sans inventer.
-À présent, génère le programme à partir des deux fichiers joints.</t>
-  </si>
-  <si>
-    <t>## Rôle
 Agis en tant que formateur expérimenté en entreprise et spécialiste du management.
 ## Objectif
 Je cherche à construire une offre et une formation sur le thème du management à distance et la gestion des équipes hybrides (mix présentiel et distanciel).
@@ -2096,6 +2044,127 @@
   </si>
   <si>
     <t>Micro-learning, Audio, Consolidation mémorielle</t>
+  </si>
+  <si>
+    <t>Création plaquette de présentation</t>
+  </si>
+  <si>
+    <t>Créateur d’une commande Memory</t>
+  </si>
+  <si>
+    <t>Memory - Générer un prompt pour une image</t>
+  </si>
+  <si>
+    <t>Améliorer ses supports de formation</t>
+  </si>
+  <si>
+    <t>Memory - Création veille</t>
+  </si>
+  <si>
+    <t>3_Choix du Dispositif Pédagogique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5_Création de chaque séquence de formation </t>
+  </si>
+  <si>
+    <t>7_Création Livret Stagiaire</t>
+  </si>
+  <si>
+    <t>7.1_Création Livret Stagiaire_HTML</t>
+  </si>
+  <si>
+    <t># Prompt — Transformation de support de formation en livret HTML interactif
+## Rôle
+Tu es un expert en développement front-end et en design pédagogique.
+Tu maîtrises la création d'interfaces HTML/CSS/JS élégantes, accessibles
+et fonctionnelles, pensées pour un usage autonome en formation.
+## Objectif
+Transformer le document Word "Support" (support participant de formation)
+en un **livret numérique dynamique au format HTML**, utilisable directement
+par chaque stagiaire depuis son navigateur.
+Le livret doit permettre au stagiaire de :
+- **Naviguer** rapidement vers la section qui l'intéresse via un menu latéral fixe
+- **Copier en un clic** les instructions/prompts présents dans le livret
+  pour les coller dans son outil IA
+- **Saisir ses réponses et commentaires** dans des zones d'écriture dédiées
+- **Joindre des fichiers** (captures, PDF, images) illustrant ses résultats
+- **Exporter son travail** au format PDF via un bouton "Enregistrer sous"
+## Contraintes
+### Contenu éditables
+- Les zones de saisie stagiaire ("espace stagiaire") sont **strictement limitées**
+  aux sections intitulées **"À vous de jouer"** dans le livret source
+- Le reste du contenu est en lecture seule, non modifiable
+### Design
+- Respecter la charte graphique (couleurs, typographie, style)
+- Interface **aérée, graphique et professionnelle**
+- Lisibilité optimale : hiérarchie visuelle claire, espaces généreux
+### Technique
+- Format : **fichier HTML unique autonome** (tout embarqué : CSS + JS)
+- Menu de navigation : **sidebar fixe à gauche**, avec ancres vers chaque section
+- Bouton "copier" : présent sous chaque bloc instruction/prompt
+- Zones d'upload : accepter images, PDF, DOCX
+- Export PDF : déclenché par un bouton dédié, via `window.print()` ou librairie JS
+- Compatibilité : navigateurs modernes (Chrome, Edge, Firefox), sans installation</t>
+  </si>
+  <si>
+    <t>4_Déroulé Pédagogique &amp; Objectifs SMART</t>
+  </si>
+  <si>
+    <t>6_Programme Qualiopi (Digiforma)</t>
+  </si>
+  <si>
+    <t>## Rôle
+Tu es un expert en ingénierie pédagogique, maîtrisant parfaitement les exigences du référentiel Qualiopi (notamment les indicateurs 1 et 2) et les formats attendus dans l'outil Digiforma. Tu es aussi expert graphiste, designer, et tu sais respecter au mieux les chartes graphiques des templates qu'on te met en pièce jointe.
+## Objectif
+Construire un programme de formation au bon format.
+## Contraintes
+1. Tu reçois en entrée :
+   - Un brief de formation (en fichier joint)
+   - Un template de programme (modèle de l'entreprise, conforme Digiforma/Qualiopi) au format .pptx, format A4 portrait, police Calibri, corps de texte noir
+2. À partir de ces deux documents :
+   - Tu complètes intégralement le programme de formation dans le respect strict du modèle fourni
+   - Tu respectes les titres, l'ordre, le vocabulaire et la mise en forme du template
+   - Tu n'inventes rien : tu t'appuies uniquement sur le brief client, sauf mention explicite t'autorisant à compléter certains points
+3. Tu produis un livrable :
+   - Une diapositive reprenant fidèlement la mise en page du modèle initial, avec les contenus insérés aux bons endroits
+4. Avant de rendre, tu vérifies que :
+   - Le programme est cohérent, synthétique et structuré
+   - Il contient les objectifs pédagogiques, les modalités d'évaluation, le public cible, les prérequis, la durée, la progression pédagogique, etc.
+   - Il respecte les critères de clarté, de lisibilité et de pertinence Qualiopi
+⚠️ En cas de doute ou d'information manquante dans le brief, indique-le dans le programme entre crochets [à compléter] sans inventer.
+À présent, génère le programme à partir des deux fichiers joints.</t>
+  </si>
+  <si>
+    <t>2.5_Le prompt permettant de générer le bon programme de formation au format Qualiopi</t>
+  </si>
+  <si>
+    <t>2.5_Le prompt créateur de programme</t>
+  </si>
+  <si>
+    <t>## Rôle
+Tu es un copywriter expert en marketing de la formation professionnelle. Tu maîtrises les structures persuasives orientées transformation (avant/après), la rédaction centrée bénéfices apprenants, et les codes visuels des plaquettes commerciales B2B.
+## Objectif
+Générer le contenu complet d'une plaquette de présentation commerciale pour le programme de formation fourni, afin de donner envie au lecteur de s'inscrire dès le premier jour, en utilisant le design système pour la mise en forme.
+## Contraintes
+- Longueur totale : entre 350 et 500 mots répartis sur les sections ci-dessous
+- Ton : [PROFESSIONNEL / DIRECT / INSPIRANT] — jamais condescendant, jamais vague
+- Langue : français, niveau C1, phrases actives et courtes
+- Interdire : jargon creux (« booster vos compétences »), promesses non vérifiables, adjectifs vides (« innovant », « révolutionnaire »)
+- Inclure : des formulations factuelles, des bénéfices concrets mesurables, des verbes d'action
+## Format de sortie
+Produis une plaquette avec ces éléments :
+1. Accroche (2 phrases max)
+   Une entrée en matière qui nomme le problème réel ou la tension que vit [PROFIL_CIBLE] avant la formation.
+2. Ce que vous allez apprendre — les éléments clés du programme
+   Tableau ou liste structurée des modules/compétences clés. Format : Module → Ce que vous maîtrisez à la sortie.
+3. Vos gains concrets
+   3 à 5 bénéfices formulés en "Vous serez capable de..." ou "À l'issue de cette formation, vous..." — orientés résultats mesurables, pas sur les contenus.
+4. La transformation apportée
+   Bloc "Avant / Après" en 2 colonnes : ce que vit l'apprenant avant la formation vs. ce qu'il vit après. 3 lignes minimum.
+5. Pour qui ce programme est-il fait ?
+   Critères d'adéquation positifs (profils qui bénéficient pleinement) et 1 critère d'exclusion (pour qui ce n'est PAS fait — renforce la crédibilité).
+6. Appel à l'action
+   1 phrase de clôture forte + 3 micro-CTA au choix : télécharger le programme, contacter un conseiller, s'inscrire directement. Format web-ready (texte de bouton + URL placeholder).</t>
   </si>
 </sst>
 </file>
@@ -2141,7 +2210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2163,9 +2232,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2405,6 +2471,9 @@
   <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </wetp:taskpane>
 </wetp:taskpanes>
 </file>
 
@@ -2422,13 +2491,28 @@
 </we:webextension>
 </file>
 
+<file path=xl/webextensions/webextension2.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{503296D5-C983-43BB-865D-CB288D8A389B}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="fr-FR" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;c4d73f7a-0a20-4ea8-b5d1-cc9b342408fe&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P46"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="40.46484375" customWidth="1"/>
-    <col min="2" max="2" width="255" customWidth="1"/>
+    <col min="2" max="2" width="120.73046875" customWidth="1"/>
+    <col min="7" max="7" width="38" customWidth="1"/>
     <col min="14" max="16" width="16" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2476,10 +2560,10 @@
         <v>13</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
@@ -2523,10 +2607,10 @@
         <v>26</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>27</v>
@@ -2573,10 +2657,10 @@
         <v>39</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P3" s="3" t="s">
         <v>27</v>
@@ -2623,16 +2707,16 @@
         <v>50</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P4" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:16" ht="384.75" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -2673,16 +2757,16 @@
         <v>58</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P5" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="171" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:16" ht="242.25" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>59</v>
       </c>
@@ -2723,10 +2807,10 @@
         <v>69</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P6" s="3" t="s">
         <v>27</v>
@@ -2734,66 +2818,66 @@
     </row>
     <row r="7" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
+        <v>375</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="C7" t="s">
         <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E7" t="s">
         <v>32</v>
       </c>
       <c r="F7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" t="s">
         <v>73</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>74</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>75</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>76</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>77</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>78</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>79</v>
       </c>
-      <c r="M7" t="s">
-        <v>80</v>
-      </c>
       <c r="N7" s="3" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P7" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="327.75" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E8" t="s">
         <v>63</v>
@@ -2802,31 +2886,31 @@
         <v>19</v>
       </c>
       <c r="G8" t="s">
+        <v>82</v>
+      </c>
+      <c r="H8" t="s">
         <v>83</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>84</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>85</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>86</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>87</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>88</v>
       </c>
-      <c r="M8" t="s">
-        <v>89</v>
-      </c>
       <c r="N8" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P8" s="3" t="s">
         <v>27</v>
@@ -2834,10 +2918,10 @@
     </row>
     <row r="9" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="C9" t="s">
         <v>16</v>
@@ -2852,48 +2936,48 @@
         <v>19</v>
       </c>
       <c r="G9" t="s">
+        <v>91</v>
+      </c>
+      <c r="H9" t="s">
         <v>92</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>93</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>94</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>95</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>96</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>97</v>
       </c>
-      <c r="M9" t="s">
-        <v>98</v>
-      </c>
       <c r="N9" s="3" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="P9" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="171" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
+        <v>98</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="C10" t="s">
         <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E10" t="s">
         <v>32</v>
@@ -2905,45 +2989,45 @@
         <v>33</v>
       </c>
       <c r="H10" t="s">
+        <v>101</v>
+      </c>
+      <c r="I10" t="s">
         <v>102</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>103</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>104</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>105</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>106</v>
       </c>
-      <c r="M10" t="s">
-        <v>107</v>
-      </c>
       <c r="N10" s="3" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P10" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="114" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:16" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="C11" t="s">
         <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E11" t="s">
         <v>63</v>
@@ -2952,42 +3036,42 @@
         <v>19</v>
       </c>
       <c r="G11" t="s">
+        <v>109</v>
+      </c>
+      <c r="H11" t="s">
         <v>110</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>111</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>112</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>113</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>114</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>115</v>
       </c>
-      <c r="M11" t="s">
-        <v>116</v>
-      </c>
       <c r="N11" s="3" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="P11" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="114" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>118</v>
       </c>
       <c r="C12" t="s">
         <v>61</v>
@@ -3005,28 +3089,28 @@
         <v>20</v>
       </c>
       <c r="H12" t="s">
+        <v>118</v>
+      </c>
+      <c r="I12" t="s">
         <v>119</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>120</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>121</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>122</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>123</v>
       </c>
-      <c r="M12" t="s">
-        <v>124</v>
-      </c>
       <c r="N12" s="3" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P12" s="3" t="s">
         <v>27</v>
@@ -3034,49 +3118,49 @@
     </row>
     <row r="13" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>126</v>
       </c>
       <c r="C13" t="s">
         <v>30</v>
       </c>
       <c r="D13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E13" t="s">
         <v>32</v>
       </c>
       <c r="F13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G13" t="s">
         <v>33</v>
       </c>
       <c r="H13" t="s">
+        <v>128</v>
+      </c>
+      <c r="I13" t="s">
         <v>129</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>130</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>131</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>132</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>133</v>
       </c>
-      <c r="M13" t="s">
-        <v>134</v>
-      </c>
       <c r="N13" s="3" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P13" s="3" t="s">
         <v>27</v>
@@ -3084,107 +3168,107 @@
     </row>
     <row r="14" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>135</v>
+        <v>376</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C14" t="s">
         <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E14" t="s">
         <v>18</v>
       </c>
       <c r="F14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" t="s">
         <v>73</v>
       </c>
-      <c r="G14" t="s">
-        <v>74</v>
-      </c>
       <c r="H14" t="s">
+        <v>135</v>
+      </c>
+      <c r="I14" t="s">
+        <v>136</v>
+      </c>
+      <c r="J14" t="s">
         <v>137</v>
       </c>
-      <c r="I14" t="s">
+      <c r="K14" t="s">
         <v>138</v>
       </c>
-      <c r="J14" t="s">
+      <c r="L14" t="s">
         <v>139</v>
       </c>
-      <c r="K14" t="s">
-        <v>140</v>
-      </c>
-      <c r="L14" t="s">
-        <v>141</v>
-      </c>
       <c r="N14" s="3" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P14" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="313.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:16" ht="342" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>142</v>
+        <v>377</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C15" t="s">
         <v>42</v>
       </c>
       <c r="D15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E15" t="s">
         <v>32</v>
       </c>
       <c r="F15" t="s">
+        <v>72</v>
+      </c>
+      <c r="G15" t="s">
         <v>73</v>
       </c>
-      <c r="G15" t="s">
-        <v>74</v>
-      </c>
       <c r="H15" t="s">
+        <v>141</v>
+      </c>
+      <c r="I15" t="s">
+        <v>142</v>
+      </c>
+      <c r="J15" t="s">
+        <v>143</v>
+      </c>
+      <c r="K15" t="s">
         <v>144</v>
       </c>
-      <c r="I15" t="s">
+      <c r="L15" t="s">
         <v>145</v>
       </c>
-      <c r="J15" t="s">
+      <c r="M15" t="s">
         <v>146</v>
       </c>
-      <c r="K15" t="s">
-        <v>147</v>
-      </c>
-      <c r="L15" t="s">
-        <v>148</v>
-      </c>
-      <c r="M15" t="s">
-        <v>149</v>
-      </c>
       <c r="N15" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P15" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="185.25" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:16" ht="228" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C16" t="s">
         <v>30</v>
@@ -3196,34 +3280,34 @@
         <v>32</v>
       </c>
       <c r="F16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G16" t="s">
+        <v>149</v>
+      </c>
+      <c r="H16" t="s">
+        <v>150</v>
+      </c>
+      <c r="I16" t="s">
+        <v>151</v>
+      </c>
+      <c r="J16" t="s">
         <v>152</v>
       </c>
-      <c r="H16" t="s">
+      <c r="K16" t="s">
         <v>153</v>
       </c>
-      <c r="I16" t="s">
+      <c r="L16" t="s">
         <v>154</v>
       </c>
-      <c r="J16" t="s">
+      <c r="M16" t="s">
         <v>155</v>
       </c>
-      <c r="K16" t="s">
-        <v>156</v>
-      </c>
-      <c r="L16" t="s">
-        <v>157</v>
-      </c>
-      <c r="M16" t="s">
-        <v>158</v>
-      </c>
       <c r="N16" s="3" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P16" s="3" t="s">
         <v>27</v>
@@ -3231,49 +3315,49 @@
     </row>
     <row r="17" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>159</v>
+        <v>380</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C17" t="s">
         <v>16</v>
       </c>
       <c r="D17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E17" t="s">
         <v>32</v>
       </c>
       <c r="F17" t="s">
+        <v>72</v>
+      </c>
+      <c r="G17" t="s">
         <v>73</v>
       </c>
-      <c r="G17" t="s">
-        <v>74</v>
-      </c>
       <c r="H17" t="s">
+        <v>157</v>
+      </c>
+      <c r="I17" t="s">
+        <v>158</v>
+      </c>
+      <c r="J17" t="s">
+        <v>159</v>
+      </c>
+      <c r="K17" t="s">
+        <v>160</v>
+      </c>
+      <c r="L17" t="s">
         <v>161</v>
       </c>
-      <c r="I17" t="s">
+      <c r="M17" t="s">
         <v>162</v>
       </c>
-      <c r="J17" t="s">
-        <v>163</v>
-      </c>
-      <c r="K17" t="s">
-        <v>164</v>
-      </c>
-      <c r="L17" t="s">
-        <v>165</v>
-      </c>
-      <c r="M17" t="s">
-        <v>166</v>
-      </c>
       <c r="N17" s="3" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>27</v>
@@ -3281,49 +3365,49 @@
     </row>
     <row r="18" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C18" t="s">
         <v>16</v>
       </c>
       <c r="D18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E18" t="s">
         <v>32</v>
       </c>
       <c r="F18" t="s">
+        <v>72</v>
+      </c>
+      <c r="G18" t="s">
         <v>73</v>
       </c>
-      <c r="G18" t="s">
-        <v>74</v>
-      </c>
       <c r="H18" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="I18" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="J18" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="K18" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L18" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M18" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P18" s="3" t="s">
         <v>27</v>
@@ -3331,10 +3415,10 @@
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B19" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C19" t="s">
         <v>42</v>
@@ -3349,31 +3433,31 @@
         <v>43</v>
       </c>
       <c r="G19" t="s">
+        <v>171</v>
+      </c>
+      <c r="H19" t="s">
+        <v>172</v>
+      </c>
+      <c r="I19" t="s">
+        <v>173</v>
+      </c>
+      <c r="J19" t="s">
+        <v>174</v>
+      </c>
+      <c r="K19" t="s">
+        <v>86</v>
+      </c>
+      <c r="L19" t="s">
         <v>175</v>
       </c>
-      <c r="H19" t="s">
+      <c r="M19" t="s">
         <v>176</v>
       </c>
-      <c r="I19" t="s">
-        <v>177</v>
-      </c>
-      <c r="J19" t="s">
-        <v>178</v>
-      </c>
-      <c r="K19" t="s">
-        <v>87</v>
-      </c>
-      <c r="L19" t="s">
-        <v>179</v>
-      </c>
-      <c r="M19" t="s">
-        <v>180</v>
-      </c>
       <c r="N19" s="3" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="P19" s="3" t="s">
         <v>27</v>
@@ -3381,10 +3465,10 @@
     </row>
     <row r="20" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C20" t="s">
         <v>42</v>
@@ -3399,48 +3483,48 @@
         <v>19</v>
       </c>
       <c r="G20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H20" t="s">
+        <v>179</v>
+      </c>
+      <c r="I20" t="s">
+        <v>180</v>
+      </c>
+      <c r="J20" t="s">
+        <v>181</v>
+      </c>
+      <c r="K20" t="s">
+        <v>86</v>
+      </c>
+      <c r="L20" t="s">
+        <v>182</v>
+      </c>
+      <c r="M20" t="s">
         <v>183</v>
       </c>
-      <c r="I20" t="s">
-        <v>184</v>
-      </c>
-      <c r="J20" t="s">
-        <v>185</v>
-      </c>
-      <c r="K20" t="s">
-        <v>87</v>
-      </c>
-      <c r="L20" t="s">
-        <v>186</v>
-      </c>
-      <c r="M20" t="s">
-        <v>187</v>
-      </c>
       <c r="N20" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P20" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="228" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:16" ht="270.75" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C21" t="s">
         <v>30</v>
       </c>
       <c r="D21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E21" t="s">
         <v>32</v>
@@ -3452,28 +3536,28 @@
         <v>33</v>
       </c>
       <c r="H21" t="s">
+        <v>186</v>
+      </c>
+      <c r="I21" t="s">
+        <v>187</v>
+      </c>
+      <c r="J21" t="s">
+        <v>188</v>
+      </c>
+      <c r="K21" t="s">
+        <v>189</v>
+      </c>
+      <c r="L21" t="s">
         <v>190</v>
       </c>
-      <c r="I21" t="s">
+      <c r="M21" t="s">
         <v>191</v>
       </c>
-      <c r="J21" t="s">
-        <v>192</v>
-      </c>
-      <c r="K21" t="s">
-        <v>193</v>
-      </c>
-      <c r="L21" t="s">
-        <v>194</v>
-      </c>
-      <c r="M21" t="s">
-        <v>195</v>
-      </c>
       <c r="N21" s="3" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P21" s="3" t="s">
         <v>27</v>
@@ -3481,110 +3565,110 @@
     </row>
     <row r="22" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C22" t="s">
         <v>30</v>
       </c>
       <c r="D22" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E22" t="s">
         <v>32</v>
       </c>
       <c r="F22" t="s">
+        <v>72</v>
+      </c>
+      <c r="G22" t="s">
         <v>73</v>
       </c>
-      <c r="G22" t="s">
-        <v>74</v>
-      </c>
       <c r="H22" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="I22" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="J22" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="K22" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="L22" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M22" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P22" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C23" t="s">
         <v>30</v>
       </c>
       <c r="D23" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E23" t="s">
         <v>32</v>
       </c>
       <c r="F23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G23" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="H23" t="s">
+        <v>200</v>
+      </c>
+      <c r="I23" t="s">
+        <v>201</v>
+      </c>
+      <c r="J23" t="s">
+        <v>202</v>
+      </c>
+      <c r="K23" t="s">
+        <v>77</v>
+      </c>
+      <c r="L23" t="s">
+        <v>203</v>
+      </c>
+      <c r="M23" t="s">
         <v>204</v>
       </c>
-      <c r="I23" t="s">
-        <v>205</v>
-      </c>
-      <c r="J23" t="s">
-        <v>206</v>
-      </c>
-      <c r="K23" t="s">
-        <v>78</v>
-      </c>
-      <c r="L23" t="s">
-        <v>207</v>
-      </c>
-      <c r="M23" t="s">
-        <v>208</v>
-      </c>
       <c r="N23" s="3" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P23" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:16" ht="57" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="C24" t="s">
         <v>30</v>
@@ -3602,39 +3686,39 @@
         <v>20</v>
       </c>
       <c r="H24" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="I24" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="J24" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="K24" t="s">
         <v>24</v>
       </c>
       <c r="L24" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="M24" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P24" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="384.75" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:16" ht="399" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>216</v>
+        <v>381</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C25" t="s">
         <v>42</v>
@@ -3646,84 +3730,84 @@
         <v>63</v>
       </c>
       <c r="F25" t="s">
+        <v>72</v>
+      </c>
+      <c r="G25" t="s">
         <v>73</v>
       </c>
-      <c r="G25" t="s">
-        <v>74</v>
-      </c>
       <c r="H25" t="s">
+        <v>213</v>
+      </c>
+      <c r="I25" t="s">
+        <v>214</v>
+      </c>
+      <c r="J25" t="s">
+        <v>215</v>
+      </c>
+      <c r="K25" t="s">
+        <v>216</v>
+      </c>
+      <c r="L25" t="s">
+        <v>217</v>
+      </c>
+      <c r="M25" t="s">
         <v>218</v>
       </c>
-      <c r="I25" t="s">
-        <v>219</v>
-      </c>
-      <c r="J25" t="s">
-        <v>220</v>
-      </c>
-      <c r="K25" t="s">
-        <v>221</v>
-      </c>
-      <c r="L25" t="s">
-        <v>222</v>
-      </c>
-      <c r="M25" t="s">
-        <v>223</v>
-      </c>
       <c r="N25" s="3" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P25" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="342" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="C26" t="s">
         <v>61</v>
       </c>
       <c r="D26" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="E26" t="s">
         <v>32</v>
       </c>
       <c r="F26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G26" t="s">
+        <v>222</v>
+      </c>
+      <c r="H26" t="s">
+        <v>223</v>
+      </c>
+      <c r="I26" t="s">
+        <v>224</v>
+      </c>
+      <c r="J26" t="s">
+        <v>225</v>
+      </c>
+      <c r="K26" t="s">
+        <v>121</v>
+      </c>
+      <c r="L26" t="s">
+        <v>226</v>
+      </c>
+      <c r="M26" t="s">
         <v>227</v>
       </c>
-      <c r="H26" t="s">
-        <v>228</v>
-      </c>
-      <c r="I26" t="s">
-        <v>229</v>
-      </c>
-      <c r="J26" t="s">
-        <v>230</v>
-      </c>
-      <c r="K26" t="s">
-        <v>122</v>
-      </c>
-      <c r="L26" t="s">
-        <v>231</v>
-      </c>
-      <c r="M26" t="s">
-        <v>232</v>
-      </c>
       <c r="N26" s="3" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="P26" s="3" t="s">
         <v>27</v>
@@ -3731,10 +3815,10 @@
     </row>
     <row r="27" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C27" t="s">
         <v>30</v>
@@ -3746,34 +3830,34 @@
         <v>63</v>
       </c>
       <c r="F27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G27" t="s">
+        <v>230</v>
+      </c>
+      <c r="H27" t="s">
+        <v>231</v>
+      </c>
+      <c r="I27" t="s">
+        <v>232</v>
+      </c>
+      <c r="J27" t="s">
+        <v>233</v>
+      </c>
+      <c r="K27" t="s">
+        <v>86</v>
+      </c>
+      <c r="L27" t="s">
+        <v>234</v>
+      </c>
+      <c r="M27" t="s">
         <v>235</v>
       </c>
-      <c r="H27" t="s">
-        <v>236</v>
-      </c>
-      <c r="I27" t="s">
-        <v>237</v>
-      </c>
-      <c r="J27" t="s">
-        <v>238</v>
-      </c>
-      <c r="K27" t="s">
-        <v>87</v>
-      </c>
-      <c r="L27" t="s">
-        <v>239</v>
-      </c>
-      <c r="M27" t="s">
-        <v>240</v>
-      </c>
       <c r="N27" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O27" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P27" s="3" t="s">
         <v>27</v>
@@ -3781,10 +3865,10 @@
     </row>
     <row r="28" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C28" t="s">
         <v>30</v>
@@ -3796,34 +3880,34 @@
         <v>63</v>
       </c>
       <c r="F28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G28" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="H28" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="I28" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="J28" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="K28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L28" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="M28" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P28" s="3" t="s">
         <v>27</v>
@@ -3831,10 +3915,10 @@
     </row>
     <row r="29" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="C29" t="s">
         <v>30</v>
@@ -3846,45 +3930,45 @@
         <v>32</v>
       </c>
       <c r="F29" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G29" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="H29" t="s">
+        <v>246</v>
+      </c>
+      <c r="I29" t="s">
+        <v>247</v>
+      </c>
+      <c r="J29" t="s">
+        <v>248</v>
+      </c>
+      <c r="K29" t="s">
+        <v>249</v>
+      </c>
+      <c r="L29" t="s">
         <v>250</v>
       </c>
-      <c r="H29" t="s">
+      <c r="M29" t="s">
         <v>251</v>
       </c>
-      <c r="I29" t="s">
-        <v>252</v>
-      </c>
-      <c r="J29" t="s">
-        <v>253</v>
-      </c>
-      <c r="K29" t="s">
-        <v>254</v>
-      </c>
-      <c r="L29" t="s">
-        <v>255</v>
-      </c>
-      <c r="M29" t="s">
-        <v>256</v>
-      </c>
       <c r="N29" s="3" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="P29" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:16" ht="66" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>42</v>
@@ -3896,45 +3980,45 @@
         <v>63</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="P30" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>283</v>
+        <v>371</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>42</v>
@@ -3946,45 +4030,45 @@
         <v>32</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
       <c r="M31" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="N31" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="N31" s="3" t="s">
-        <v>286</v>
-      </c>
       <c r="O31" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="P31" s="3" t="s">
         <v>277</v>
-      </c>
-      <c r="P31" s="3" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="32" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>42</v>
@@ -3996,45 +4080,45 @@
         <v>32</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="M32" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="N32" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="N32" s="3" t="s">
-        <v>286</v>
-      </c>
       <c r="O32" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="P32" s="3" t="s">
         <v>277</v>
-      </c>
-      <c r="P32" s="3" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="33" spans="1:16" ht="120" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>16</v>
@@ -4046,45 +4130,45 @@
         <v>32</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="H33" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I33" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="I33" s="2" t="s">
-        <v>94</v>
-      </c>
       <c r="J33" s="2" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="K33" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="L33" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="L33" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="M33" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="P33" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="34" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>291</v>
+        <v>372</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>30</v>
@@ -4096,93 +4180,93 @@
         <v>32</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G34" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N34" s="3" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="35" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="36" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>42</v>
@@ -4194,42 +4278,42 @@
         <v>18</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="37" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>296</v>
+        <v>373</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>60</v>
@@ -4244,10 +4328,10 @@
         <v>63</v>
       </c>
       <c r="F37" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G37" s="6" t="s">
         <v>73</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>20</v>
       </c>
       <c r="H37" s="2" t="s">
         <v>64</v>
@@ -4265,24 +4349,24 @@
         <v>68</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N37" s="3" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="O37" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P37" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>297</v>
+        <v>374</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>30</v>
@@ -4294,145 +4378,145 @@
         <v>32</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N38" s="3" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="O38" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P38" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="39" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="40" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F40" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G40" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="H40" s="2" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="P40" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="41" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>302</v>
+        <v>383</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>322</v>
+        <v>382</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>42</v>
@@ -4444,95 +4528,95 @@
         <v>32</v>
       </c>
       <c r="F41" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G41" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G41" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="H41" s="2" t="s">
-        <v>359</v>
+        <v>347</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>361</v>
+        <v>349</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="42" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>362</v>
+        <v>350</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>363</v>
+        <v>351</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="43" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
-        <v>305</v>
+        <v>384</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>42</v>
@@ -4544,166 +4628,241 @@
         <v>18</v>
       </c>
       <c r="F43" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G43" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="G43" s="6" t="s">
-        <v>74</v>
-      </c>
       <c r="H43" s="2" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>368</v>
+        <v>356</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="O43" s="3" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="P43" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="44" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="6" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M44" s="2"/>
-      <c r="N44" s="3"/>
-      <c r="O44" s="3"/>
+      <c r="N44" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="O44" s="3" t="s">
+        <v>257</v>
+      </c>
       <c r="P44" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="45" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>42</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F45" s="9" t="s">
+      <c r="F45" s="2" t="s">
         <v>43</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>374</v>
+        <v>362</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>376</v>
+        <v>364</v>
+      </c>
+      <c r="N45" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="O45" s="3" t="s">
+        <v>257</v>
       </c>
       <c r="P45" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="46" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A46" s="9" t="s">
-        <v>309</v>
-      </c>
-      <c r="B46" s="10" t="s">
-        <v>327</v>
+      <c r="A46" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>315</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>42</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F46" s="9" t="s">
+      <c r="F46" s="2" t="s">
         <v>43</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H46" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="N46" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="O46" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="P46" s="3" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A47" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A48" t="s">
         <v>378</v>
       </c>
-      <c r="I46" s="2" t="s">
+      <c r="B48" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="J46" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="L46" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="P46" s="3" t="s">
-        <v>282</v>
+      <c r="C48" t="s">
+        <v>42</v>
+      </c>
+      <c r="D48" t="s">
+        <v>126</v>
+      </c>
+      <c r="E48" t="s">
+        <v>32</v>
+      </c>
+      <c r="F48" t="s">
+        <v>72</v>
+      </c>
+      <c r="G48" t="s">
+        <v>73</v>
+      </c>
+      <c r="H48" t="s">
+        <v>141</v>
+      </c>
+      <c r="I48" t="s">
+        <v>142</v>
+      </c>
+      <c r="J48" t="s">
+        <v>143</v>
+      </c>
+      <c r="K48" t="s">
+        <v>144</v>
+      </c>
+      <c r="L48" t="s">
+        <v>145</v>
+      </c>
+      <c r="M48" t="s">
+        <v>146</v>
+      </c>
+      <c r="N48" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="O48" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="P48" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:P48" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Mettre à jour la bibliothèque Excel au 2 septembre 2026
</commit_message>
<xml_diff>
--- a/data/BibliothèquePrompt.xlsx
+++ b/data/BibliothèquePrompt.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00_Nexellia\04_PRESTATIONS\Valeurs &amp; Talents\BibliothèquePrompt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87B3E938-733D-44EE-9FC9-F1994C6C5E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{375C7924-B2FA-4393-B6A3-71EA752EB589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22740" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-6060" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="_Data" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">_Data!$A$1:$P$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">_Data!$A$1:$P$47</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="372">
   <si>
     <t>Nom</t>
   </si>
@@ -773,9 +773,6 @@
     <t>Avoir défini la séquence 3A (Prompt P008).</t>
   </si>
   <si>
-    <t>Définition Persona et Enjeux</t>
-  </si>
-  <si>
     <t>## Rôle
 Agis en tant que formateur expérimenté en entreprise et spécialiste de la thématique &lt;A compléter en fonction de votre contexte&gt;. Tu es expert Qualiopi et tu connais toutes les exigences réglementaires du référentiel. Tu es en particulier au fait de toutes les pédagogies favorisant l'inclusion et limitant les risques de mises en situation de handicap (notamment au niveau des supports pédagogiques qui seront générés et notamment les maladies en dys, la malvoyance, le daltonisme… les jeux et mises en situation que tu proposeras pourront être réalisées par des personnes en PMR).
 ## Objectif
@@ -1119,9 +1116,6 @@
     <t>Développer des contenus de formation • Concevoir des supports multimédias • Stimuler l'engagement d'apprenants</t>
   </si>
   <si>
-    <t>Liste Compétences à travailler (Taxonomie Bloom)</t>
-  </si>
-  <si>
     <t>## Rôle
 Agis en tant qu'expert en ingénierie pédagogique. Tu maîtrises toutes les techniques pédagogiques modernes, participatives. Tu maîtrises la ludopédagogie et la taxonomie de Bloom. Tu es expert Qualiopi et tu connais toutes les exigences réglementaires du référentiel. Tu es en particulier au fait de toutes les pédagogies favorisant l'inclusion et limitant les risques de mises en situation de handicap (notamment au niveau des supports pédagogiques qui seront générés et notamment les maladies en dys, la malvoyance, le daltonisme… les jeux et mises en situation que tu proposeras pourront être réalisées par des personnes en PMR).
 ## Objectif
@@ -1254,36 +1248,6 @@
     <t>Avoir un PDF de newsletter.</t>
   </si>
   <si>
-    <t>Script Slides Gamma</t>
-  </si>
-  <si>
-    <t>## Rôle
-Tu es un expert en pédagogie inclusive et en conception de supports de formation professionnelle. Tu maîtrises parfaitement l'outil Gamma.app, les contraintes d'accessibilité (troubles DYS, daltonisme), et les bonnes pratiques de conception graphique pour des contenus impactants et inclusifs.
-## Compétences mobilisées
-- Structuration pédagogique claire et accessible
-- Synthèse et vulgarisation de contenus de formation
-- Design de présentation optimisé pour Gamma (visibilité, rythme, hiérarchie)
-- Conception graphique inclusive (polices, contrastes, couleurs compatibles DYS et daltonisme)
-## Contexte
-Tu dois créer un script de slideshow (8 diapos) à partir d'une séquence de formation professionnelle fournie par l'utilisateur, afin de servir de support d'animation pour un formateur. Ce slideshow sera intégré à Gamma.
-## Objectif
-Transformer une séquence pédagogique brute en 8 slides claires, sans titre visible, pensées pour animer la formation à l'oral (pas pour être lues seules). Elles doivent permettre au formateur de suivre le fil pédagogique, tout en respectant les principes d'accessibilité visuelle.
-## Tâches à réaliser
-1. Demander à l'utilisateur d'uploader la séquence de formation ou le livret stagiaire détaillant la séquence de formation.
-2. Une fois le contenu reçu, proposer un découpage en 8 slides structurées, visuellement attractives, sans surcharge, avec :
-   - Mots-clés ou schémas simples
-   - Éléments visuels sobres mais évocateurs
-   - Contraste fort et police sans serif (OpenDyslexic, Arial, Verdana...)
-   - Aucun rouge/vert direct (éviter le piège daltonien)
-   - Ton professionnel et dynamique
-   - Pas de texte narratif complet : uniquement points clés et visuels supports
-## Contraintes
-- Langue : Français
-- Format : Slides pour Gamma.app (1 idée = 1 slide, design clair, responsive)
-- Accessibilité : Compatible DYS, daltonisme, lecture orale facile
-- Utilisation : Support oral d'animation, non autoportant</t>
-  </si>
-  <si>
     <t>Jour1_Sequence4</t>
   </si>
   <si>
@@ -1293,67 +1257,10 @@
     <t>Création rapide de supports visuels de formation.</t>
   </si>
   <si>
-    <t>Gamma, Support formation, Support stagiaire</t>
-  </si>
-  <si>
     <t>{séquence_formation}</t>
   </si>
   <si>
     <t>Utiliser l'outil Gamma.app par la suite.</t>
-  </si>
-  <si>
-    <t>Script Slides Genspark</t>
-  </si>
-  <si>
-    <t>## Rôle
-Tu es un expert de la plateforme Genspark, graphiste spécialisé en formation professionnelle. Tu maîtrises parfaitement les principes de pédagogie inclusive (troubles DYS, daltonisme, accessibilité cognitive), la conception de slides engageants pour les formateurs, et l'intégration fluide de chartes graphiques.
-## Objectif
-Créer un prompt optimisé à insérer dans Genspark, qui générera un slideshow structuré, impactant et accessible, servant de support d'animation pour une séquence de formation professionnelle.
-## Compétences mobilisées
-- Design pédagogique (clarté, rythme, cohérence)
-- Accessibilité et inclusion (polices sans empattement, contrastes adaptés, pictos clairs)
-- Graphisme orienté formation
-- Connaissance des troubles DYS et exigences RGPD
-- Sens du storytelling et de la hiérarchisation visuelle
-## Tâche
-1. **Demander au formateur** :
-   - Le descriptif précis de la séquence de formation (thème, objectifs, durée, public visé)
-   - Les éléments visuels de la charte graphique à intégrer (couleurs, polices, icônes, logos)
-2. **Générer un prompt à insérer dans Genspark** qui permet :
-   - La création de slides structurées autour des 3A (Appel – Apport – Ancrage)
-   - L'invitation à uploader un **logo** du client
-   - L'utilisation d'un **exemple de présentation réussie** comme source d'inspiration visuelle
-## Processus
-- Analyser le contenu fourni par le formateur
-- Extraire les messages clés à placer dans le slideshow (en évitant le texte "lourd")
-- Générer un enchaînement logique et dynamique des diapos (max 8)
-- Rédiger les indications à intégrer dans Genspark pour que l'outil produise une présentation attractive et inclusive
-## Caractéristiques du prompt final
-- Langage inclusif et clair
-- Consignes précises pour le design : contraste élevé, structure par blocs, icônes explicites
-- Éviter toute donnée nominative ou sensible (RGPD)
-- Support animé oralement : ne pas tout écrire sur les slides, prévoir un usage en support d'animation
----
-Souhaites-tu que je passe à la **rédaction du prompt à coller dans Genspark** maintenant ? Si oui, il me faudrait :
-1. Le descriptif de la **séquence pédagogique concernée**
-2. Les **éléments de charte graphique** (codes couleurs, typo, logo si possible)
-3. Un lien ou une description d'un **exemple de présentation réussie** que tu veux prendre comme modèle
-Une fois ces 3 éléments fournis, je te fournis le prompt Genspark finalisé. On y va ?</t>
-  </si>
-  <si>
-    <t>Générer un prompt spécifique à coller dans Genspark pour créer une présentation pédagogique inclusive.</t>
-  </si>
-  <si>
-    <t>Création de slides via Genspark.</t>
-  </si>
-  <si>
-    <t>Genspark, Support formation, Support stagiaire</t>
-  </si>
-  <si>
-    <t>{charte_graphique}, {descriptif_séquence}, {exemple_modèle}</t>
-  </si>
-  <si>
-    <t>Utiliser l'outil Genspark.</t>
   </si>
   <si>
     <t>Veille IA Formation</t>
@@ -1500,9 +1407,6 @@
     <t>Automatisation_ Création des assistants IA</t>
   </si>
   <si>
-    <t>C2; C8</t>
-  </si>
-  <si>
     <t>ChatGPT, Gemini</t>
   </si>
   <si>
@@ -1525,9 +1429,6 @@
   </si>
   <si>
     <t>C3; C8</t>
-  </si>
-  <si>
-    <t>Genspark</t>
   </si>
   <si>
     <t>Prompt pour la recherche approfondie</t>
@@ -1763,35 +1664,6 @@
   </si>
   <si>
     <t>## Rôle
-Tu es un expert pédagogique, spécialiste de la formation.
-## Objectif
-À partir du brief fourni par l'utilisateur, générer un programme de formation complet au format texte respectant le schéma défini.
-## Règles de génération du contenu
-Le programme doit contenir les éléments principaux suivants :
-1. **Titre de la formation** : proposer un titre basé sur le brief ; si explicitement donné, le reprendre, sinon proposer un titre approprié.
-2. **Description en quelques lignes** : description attractive basée sur le brief, donnant envie d'assister à la formation (5 phrases maximum).
-3. **Durée** : durée si précisée dans le brief, sinon mettre « À remplir ».
-4. **Profil stagiaire** : profil basé sur le brief ; si explicitement donné, le reprendre, sinon proposer un profil approprié (10 mots maximum).
-5. **Délai d'accès** : « 2 semaines » par défaut, sauf mention contraire du brief.
-6. **Objectif général** : objectif général basé sur le brief ; si explicitement donné, le reprendre, sinon proposer un objectif approprié.
-7. **Prérequis** : « Aucun » par défaut, sauf mention contraire du brief.
-8. **Modalités pédagogiques** : indiquer présentielle, distancielle ou mixte, basé sur le brief ; si non précisé, « À remplir ».
-9. **Prix** : « Selon devis ».
-10. **En savoir plus** : « +33 6 81 25 53 88 (entre 8h30 et 19h en semaine) ou mickael.loeuille@valeurs-et-talents.fr ».
-11. **Lieu de formation** : lieu si précisé dans le brief, sinon « À remplir ».
-12. **Objectifs** : 5 objectifs maximum, rédigés selon la taxonomie de Bloom, basés sur le brief client.
-13. **Déroulé détaillé de la formation** : déroulé pédagogique détaillé et timé, basé sur la durée du brief (ou, si non précisée, un déroulé séquencé répondant aux objectifs). Chaque séquence est rédigée comme suit :
-   - Séquence n° [numéro]
-   - [Titre de la séquence]
-   - Durée : [durée]
-   - Objectif : [objectif visé pour cette séquence]
-   - [Description détaillée de la séquence]
-14. **Organisation de la formation** : « Équipe pédagogique : un formateur expert de la formation professionnelle, et dans la thématique de formation. Moyens pédagogiques et techniques : support de formation, dispositif de suivi de l'exécution et de l'évaluation des résultats de la formation, ateliers de mise en pratique tout au long de la formation, QCM ».
-15. **Modalités et délais d'accès** : « Accessibilité / Handicap : nos formations sont ouvertes à tous. En cas de doute, nous invitons à prendre contact directement avec notre référent handicap, en amont de la formation, pour discuter et, au besoin, adapter notre pédagogie et nos activités en fonction des situations de handicap qui pourraient se présenter. Le cas échéant, si nous ne sommes pas en mesure de vous accueillir, nous saurons vous orienter vers notre partenaire l'Agefiph. Contact : mickael.loeuille@valeurs-et-talents.fr / 06 81 25 53 88. Modalité et délai d'accès : notre organisme de formation s'engage à répondre en 48h à toute demande d'information. Une fois le contact établi, nous envisagerons conjointement la date la plus appropriée en fonction de vos besoins et de vos enjeux. Sauf cas particulier, la mise en place de la formation pourra se faire dans les 15 jours suivant votre demande. Pour toute information, nous contacter par mail ou téléphone : mickael.loeuille@valeurs-et-talents.fr — 06 81 25 53 88 (8h30-19h30 tous les jours de la semaine) ».
-16. **Nos indicateurs de performance et de qualité** : « Net Promoter Score : ».</t>
-  </si>
-  <si>
-    <t>## Rôle
 Tu es un producteur audio spécialisé dans la création de présentations de formations engageantes et persuasives.
 ## Objectif
 Générer un script audio, puis le transformer en narration fluide, professionnelle et dynamique.
@@ -1977,15 +1849,6 @@
     <t>Développer des contenus de formation • Stimuler l'engagement d'apprenants</t>
   </si>
   <si>
-    <t>Générer un programme de formation au format Qualiopi/Digiforma à partir d'un brief et d'un template, via Genspark.</t>
-  </si>
-  <si>
-    <t>Création du document programme de formation conforme au référentiel Qualiopi.</t>
-  </si>
-  <si>
-    <t>{brief_formation}, {template_programme}</t>
-  </si>
-  <si>
     <t>Concevoir une offre et une formation complète sur le management à distance et les équipes hybrides, avec étude de marché, supports et podcast promotionnel.</t>
   </si>
   <si>
@@ -1998,18 +1861,6 @@
     <t>{formation_standard_manager}, {programme_vierge}, {exemple_déroulé_pédagogique}, {exemple_livret_stagiaire}</t>
   </si>
   <si>
-    <t>Générer un programme de formation complet et structuré à partir d'un brief, selon un schéma texte prédéfini.</t>
-  </si>
-  <si>
-    <t>Création rapide d'un programme de formation standardisé.</t>
-  </si>
-  <si>
-    <t>Automatiser la gestion administrative • Développer des contenus de formation</t>
-  </si>
-  <si>
-    <t>{brief_formation}</t>
-  </si>
-  <si>
     <t>Générer le script d'une présentation audio persuasive pour promouvoir une formation.</t>
   </si>
   <si>
@@ -2065,12 +1916,6 @@
   </si>
   <si>
     <t xml:space="preserve">5_Création de chaque séquence de formation </t>
-  </si>
-  <si>
-    <t>7_Création Livret Stagiaire</t>
-  </si>
-  <si>
-    <t>7.1_Création Livret Stagiaire_HTML</t>
   </si>
   <si>
     <t># Prompt — Transformation de support de formation en livret HTML interactif
@@ -2114,34 +1959,6 @@
   </si>
   <si>
     <t>## Rôle
-Tu es un expert en ingénierie pédagogique, maîtrisant parfaitement les exigences du référentiel Qualiopi (notamment les indicateurs 1 et 2) et les formats attendus dans l'outil Digiforma. Tu es aussi expert graphiste, designer, et tu sais respecter au mieux les chartes graphiques des templates qu'on te met en pièce jointe.
-## Objectif
-Construire un programme de formation au bon format.
-## Contraintes
-1. Tu reçois en entrée :
-   - Un brief de formation (en fichier joint)
-   - Un template de programme (modèle de l'entreprise, conforme Digiforma/Qualiopi) au format .pptx, format A4 portrait, police Calibri, corps de texte noir
-2. À partir de ces deux documents :
-   - Tu complètes intégralement le programme de formation dans le respect strict du modèle fourni
-   - Tu respectes les titres, l'ordre, le vocabulaire et la mise en forme du template
-   - Tu n'inventes rien : tu t'appuies uniquement sur le brief client, sauf mention explicite t'autorisant à compléter certains points
-3. Tu produis un livrable :
-   - Une diapositive reprenant fidèlement la mise en page du modèle initial, avec les contenus insérés aux bons endroits
-4. Avant de rendre, tu vérifies que :
-   - Le programme est cohérent, synthétique et structuré
-   - Il contient les objectifs pédagogiques, les modalités d'évaluation, le public cible, les prérequis, la durée, la progression pédagogique, etc.
-   - Il respecte les critères de clarté, de lisibilité et de pertinence Qualiopi
-⚠️ En cas de doute ou d'information manquante dans le brief, indique-le dans le programme entre crochets [à compléter] sans inventer.
-À présent, génère le programme à partir des deux fichiers joints.</t>
-  </si>
-  <si>
-    <t>2.5_Le prompt permettant de générer le bon programme de formation au format Qualiopi</t>
-  </si>
-  <si>
-    <t>2.5_Le prompt créateur de programme</t>
-  </si>
-  <si>
-    <t>## Rôle
 Tu es un copywriter expert en marketing de la formation professionnelle. Tu maîtrises les structures persuasives orientées transformation (avant/après), la rédaction centrée bénéfices apprenants, et les codes visuels des plaquettes commerciales B2B.
 ## Objectif
 Générer le contenu complet d'une plaquette de présentation commerciale pour le programme de formation fourni, afin de donner envie au lecteur de s'inscrire dès le premier jour, en utilisant le design système pour la mise en forme.
@@ -2165,6 +1982,189 @@
    Critères d'adéquation positifs (profils qui bénéficient pleinement) et 1 critère d'exclusion (pour qui ce n'est PAS fait — renforce la crédibilité).
 6. Appel à l'action
    1 phrase de clôture forte + 3 micro-CTA au choix : télécharger le programme, contacter un conseiller, s'inscrire directement. Format web-ready (texte de bouton + URL placeholder).</t>
+  </si>
+  <si>
+    <t>1_Définition Persona et Enjeux</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autocritque </t>
+  </si>
+  <si>
+    <t>## Rôle
+Agis en tant que relecteur critique expert en ingénierie de prompts. Passe en revue les réponses proposées par d'autres IA ou par l'utilisateur.
+## Objectif
+Identifie les forces et faiblesses de la réponse analyse et donne une note de 0 à 5. Justifie ta réponse et propose au moins 3 améliorations concrètes. 
+## Contraintes
+Sois factuel et rigoureux, sans complésance. Structure : « Analyse critique », « Suggestions d'amélioration », « Conclusion sur la qualité de la réponse ». Si la réponse est incomplete, formule une version optimisée.</t>
+  </si>
+  <si>
+    <t>Evaluation d'une réponse.</t>
+  </si>
+  <si>
+    <t>7_Script contenu de Slides</t>
+  </si>
+  <si>
+    <t>## Rôle
+Tu es un expert en pédagogie inclusive et en conception de supports de formation professionnelle. Tu maîtrises parfaitement  les contraintes d'accessibilité (troubles DYS, daltonisme), et les bonnes pratiques de conception graphique pour des contenus impactants et inclusifs.
+## Compétences mobilisées
+- Structuration pédagogique claire et accessible
+- Synthèse et vulgarisation de contenus de formation
+- Design de présentation optimisé (visibilité, rythme, hiérarchie)
+- Conception graphique inclusive (polices, contrastes, couleurs compatibles DYS et daltonisme)
+## Contexte
+Tu dois créer un script de slideshow  à partir d'une séquence de formation professionnelle fournie par l'utilisateur, afin de servir de support d'animation pour un formateur. 
+## Objectif
+Transformer une séquence pédagogique brute en  slides claires, sans titre visible, pensées pour animer la formation à l'oral (pas pour être lues seules). Elles doivent permettre au formateur de suivre le fil pédagogique, tout en respectant les principes d'accessibilité visuelle.
+## Tâches à réaliser
+1. Demander à l'utilisateur d'uploader la séquence de formation ou le livret stagiaire détaillant la séquence de formation.
+2. Une fois le contenu reçu, proposer un découpage en slides structurées, visuellement attractives, sans surcharge, avec :
+   - Mots-clés ou schémas simples
+   - Éléments visuels sobres mais évocateurs
+   - Contraste fort et police sans serif (OpenDyslexic, Arial, Verdana...)
+   - Aucun rouge/vert direct (éviter le piège daltonien)
+   - Ton professionnel et dynamique
+   - Pas de texte narratif complet : uniquement points clés et visuels supports
+## Contraintes
+- Langue : Français
+- Format : Textes  et consignes claires pour la création de slides (1 idée = 1 slide, design clair, responsive)
+- Accessibilité : Compatible DYS, daltonisme, lecture orale facile
+- Utilisation : Support oral d'animation, non autoportant</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Support formation, Support stagiaire</t>
+  </si>
+  <si>
+    <t>Création rapide du slideshow de formation.</t>
+  </si>
+  <si>
+    <t>## Rôle
+Tu es un expert en pédagogie inclusive et en conception de supports de formation professionnelle. Tu maîtrises parfaitement  les contraintes d'accessibilité (troubles DYS, daltonisme), et les bonnes pratiques de conception graphique pour des contenus impactants et inclusifs.
+## Compétences mobilisées
+- Structuration pédagogique claire et accessible
+- Synthèse et vulgarisation de contenus de formation
+- Design de présentation optimisé (visibilité, rythme, hiérarchie)
+- Conception graphique inclusive (polices, contrastes, couleurs compatibles DYS et daltonisme)
+## Contexte
+Tu dois créer un script de slideshow  à partir d'une séquence de formation professionnelle fournie par l'utilisateur, afin de servir de support d'animation pour un formateur. 
+# RÔLE
+Tu es un expert en conception de supports de formation professionnelle pour adultes,
+spécialisé en pédagogie inclusive et en design graphique accessible. Tu maîtrises :
+- les contraintes liées aux troubles DYS (dyslexie, dyspraxie, dyscalculie)
+- le daltonisme (deutéranopie, protanopie, tritanopie)
+- les normes WCAG 2.1 (niveau AA minimum, AAA pour les éléments critiques)
+- la théorie de la charge cognitive (Sweller) et les principes andragogiques
+---
+# MISSION
+Transforme le script fourni en spécifications de diapositives structurées, 
+pédagogiquement efficaces et entièrement accessibles, en respectant strictement 
+la charte graphique fournie.
+Pour chaque diapositive identifiée dans le script, produis une fiche de 
+spécification complète selon le format défini en section FORMAT DE SORTIE.
+---
+# INPUTS
+## Script complet
+[COLLER LE SCRIPT ICI — inclure pour chaque diapo : numéro, titre,
+contenu brut, intention pédagogique ou notes formateur si disponibles]
+## Charte graphique
+[COLLER LA CHARTE ICI — inclure : palette HEX, typographies (noms + 
+tailles de base), logo, gabarits disponibles, ton éditorial]
+---
+# RÈGLES DE CONCEPTION GRAPHIQUE
+## Principe cardinal
+Une idée = une diapositive. JAMAIS de surcharge. Si le script dépasse ce seuil
+pour une diapo, découpe en plusieurs et signale-le explicitement.
+## Hiérarchie visuelle
+- Titre : accroche ou question, pas un résumé — maximum 8 mots
+- Corps : 3 éléments maximum par diapo (texte + visuel + donnée)
+- Ordre de lecture naturel (haut-gauche → droite → bas) guide le placement
+## Densité et espace
+- Règle du respir : 40 % minimum de la diapositive reste neutre/blanc
+- Marges de sécurité : 8 % minimum sur chaque bord
+- Espacement inter-blocs : ≥ 16 pt
+## Typographie
+- Corps de texte : taille minimale 24 pt (projection) / 18 pt (PDF/lecture)
+- Interlignage : ≥ 1,5x — critique pour les profils DYS
+- JAMAIS de police serif pour les corps de texte : utiliser sans-serif
+  (Arial, Open Sans, Atkinson Hyperlegible en priorité si hors charte)
+- JAMAIS d'italique pur sur les contenus essentiels
+- Gras réservé à 1 seul mot-clé par phrase maximum
+---
+# RÈGLES D'ACCESSIBILITÉ
+## Daltonisme (OBLIGATOIRE)
+- La couleur ne DOIT JAMAIS être le seul vecteur d'information :
+  toujours doubler d'une icône, d'un motif ou d'un libellé
+- Contraste texte/fond : minimum 4,5:1 (WCAG AA), viser 7:1 (AAA)
+  pour les informations critiques
+- Palettes sûres : bleu/orange, bleu/jaune — ÉVITER rouge/vert seuls
+- Signaler tout conflit avec la charte et proposer une alternative conforme
+## Troubles DYS (OBLIGATOIRE)
+- Phrases ≤ 15 mots — une idée par phrase
+- Alignement gauche UNIQUEMENT — jamais de justification
+- Mots-clés : encadrer ou surligner, jamais en italique
+- Puces simples (•) pour les listes non ordonnées
+- Schéma + légende courte &gt; pavé de texte
+- Texte sur image : TOUJOURS avec fond de contraste ou bandeau opaque
+## Structure et navigation
+- Numérotation visible sur chaque diapo : format "X / N_total"
+- Titre visible sur toutes les diapositives, même les visuelles
+- Récapitulatif en fin de séquence thématique (≤ 3 points clés)
+---
+# RÈGLES PÉDAGOGIQUES
+## Ancrage et mémorisation
+- Ouvrir chaque bloc thématique par une question ou une situation-problème
+- Clore chaque bloc par un "retenez que…" ou une synthèse visuelle
+- Intercaler une pause active toutes les 7 à 10 diapositives
+  (question ouverte, réflexion individuelle, ou mini-sondage)
+## Cohérence cognitive
+- Progresser selon la taxonomie de Bloom : chaque diapo sert un objectif
+  opérationnel identifiable (savoir / comprendre / appliquer / analyser)
+- L'exemple concret PRÉCÈDE ou illustre IMMÉDIATEMENT le concept abstrait
+- Charge cognitive : fractionner en séquences de 3 éléments max (Sweller)
+- Animations (si disponibles) : révèlent une information à la fois — jamais décoratives
+---
+# FORMAT DE SORTIE
+Pour chaque diapositive, produis exactement :
+---
+### Diapo [N] — [TITRE AFFICHÉ]
+**Gabarit** : [titre seul / titre + texte / titre + visuel / 2 colonnes /
+              citation / tableau / schéma / pause active / récapitulatif]
+**Texte affiché** :
+[Texte exact à afficher sur la diapositive — respecter les contraintes DYS]
+**Éléments visuels** :
+[Description précise : type (photo / icône / schéma / graphique / pictogramme),
+sujet, style, placement sur la diapo]
+**Palette utilisée** :
+[Références HEX issues de la charte — fond, texte principal, accent, secondaire]
+**Note accessibilité** :
+[Vérification contraste, alternative non-couleur, point DYS spécifique à cette diapo]
+**Note pédagogique** :
+[Objectif Bloom visé, lien avec la séquence, consigne formateur si nécessaire]
+**Alerte** (si applicable) :
+[Diapo découpée depuis le script / Conflit charte-accessibilité / Densité excessive détectée]
+---
+---
+# CONTRAINTES FINALES
+1. RESPECTER la charte : aucune couleur, police ou gabarit hors charte sans
+   justification explicite dans la note accessibilité
+2. Si une contrainte d'accessibilité entre en CONFLIT avec la charte :
+   signaler le conflit, proposer une alternative conforme, ne pas ignorer
+3. Si une diapo du script est TROP DENSE : la découper, numéroter les
+   sous-diapositives (ex. : 4a, 4b), signaler dans le champ Alerte
+4. Numérotation CONTINUE et cohérente sur l'ensemble du jeu final
+5. Si une intention pédagogique est ABSENTE du script pour une diapo,
+   en déduire une à partir du contexte et la signaler comme [déduit]</t>
+  </si>
+  <si>
+    <t>8_Création de Slides</t>
+  </si>
+  <si>
+    <t>9_Création Livret Stagiaire</t>
+  </si>
+  <si>
+    <t>9_Création Livret Stagiaire_HTML</t>
+  </si>
+  <si>
+    <t>2_Liste Compétences à travailler (Taxonomie Bloom)</t>
   </si>
 </sst>
 </file>
@@ -2507,17 +2507,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="40.46484375" customWidth="1"/>
+    <col min="1" max="1" width="40.46484375" style="8" customWidth="1"/>
     <col min="2" max="2" width="120.73046875" customWidth="1"/>
     <col min="7" max="7" width="38" customWidth="1"/>
     <col min="14" max="16" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
@@ -2560,14 +2560,14 @@
         <v>13</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+      <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -2607,17 +2607,17 @@
         <v>26</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="171" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+      <c r="A3" s="8" t="s">
         <v>28</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -2657,17 +2657,17 @@
         <v>39</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="P3" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+      <c r="A4" s="8" t="s">
         <v>40</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -2707,17 +2707,17 @@
         <v>50</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="P4" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="384.75" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+      <c r="A5" s="8" t="s">
         <v>51</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -2757,17 +2757,17 @@
         <v>58</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P5" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="242.25" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+      <c r="A6" s="8" t="s">
         <v>59</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -2807,18 +2807,18 @@
         <v>69</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P6" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>375</v>
+      <c r="A7" s="8" t="s">
+        <v>353</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>70</v>
@@ -2857,17 +2857,17 @@
         <v>79</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P7" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
+      <c r="A8" s="8" t="s">
         <v>80</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -2907,17 +2907,17 @@
         <v>88</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P8" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
+      <c r="A9" s="8" t="s">
         <v>89</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -2957,17 +2957,17 @@
         <v>97</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
       <c r="P9" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
+      <c r="A10" s="8" t="s">
         <v>98</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -3007,17 +3007,17 @@
         <v>106</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="P10" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="128.25" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
+      <c r="A11" s="8" t="s">
         <v>107</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -3057,21 +3057,21 @@
         <v>115</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
       <c r="P11" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>116</v>
+    <row r="12" spans="1:16" ht="128.25" x14ac:dyDescent="0.45">
+      <c r="A12" s="8" t="s">
+        <v>360</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>117</v>
+        <v>361</v>
       </c>
       <c r="C12" t="s">
         <v>61</v>
@@ -3092,7 +3092,7 @@
         <v>118</v>
       </c>
       <c r="I12" t="s">
-        <v>119</v>
+        <v>362</v>
       </c>
       <c r="J12" t="s">
         <v>120</v>
@@ -3107,118 +3107,121 @@
         <v>123</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="P12" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>124</v>
+    <row r="13" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
+      <c r="A13" s="8" t="s">
+        <v>116</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C13" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>126</v>
+        <v>17</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="F13" t="s">
-        <v>127</v>
+        <v>19</v>
       </c>
       <c r="G13" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="H13" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="I13" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="J13" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K13" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="L13" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="M13" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>268</v>
+        <v>242</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
       <c r="P13" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>376</v>
+      <c r="A14" s="8" t="s">
+        <v>124</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="C14" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
         <v>126</v>
       </c>
       <c r="E14" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="F14" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
       <c r="G14" t="s">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="H14" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="I14" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="J14" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="K14" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="L14" t="s">
-        <v>139</v>
+        <v>132</v>
+      </c>
+      <c r="M14" t="s">
+        <v>133</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="P14" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="342" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
-        <v>377</v>
+    <row r="15" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A15" s="8" t="s">
+        <v>354</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C15" t="s">
         <v>42</v>
@@ -3227,7 +3230,7 @@
         <v>126</v>
       </c>
       <c r="E15" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F15" t="s">
         <v>72</v>
@@ -3236,45 +3239,42 @@
         <v>73</v>
       </c>
       <c r="H15" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="I15" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="J15" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="K15" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="L15" t="s">
-        <v>145</v>
-      </c>
-      <c r="M15" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>263</v>
+        <v>250</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P15" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="228" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>147</v>
+    <row r="16" spans="1:16" ht="342" x14ac:dyDescent="0.45">
+      <c r="A16" s="8" t="s">
+        <v>369</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D16" t="s">
-        <v>31</v>
+        <v>126</v>
       </c>
       <c r="E16" t="s">
         <v>32</v>
@@ -3283,48 +3283,48 @@
         <v>72</v>
       </c>
       <c r="G16" t="s">
-        <v>149</v>
+        <v>73</v>
       </c>
       <c r="H16" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="I16" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="J16" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="K16" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="L16" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="M16" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>269</v>
+        <v>251</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P16" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
-        <v>380</v>
+    <row r="17" spans="1:16" ht="228" x14ac:dyDescent="0.45">
+      <c r="A17" s="8" t="s">
+        <v>359</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="C17" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D17" t="s">
-        <v>126</v>
+        <v>31</v>
       </c>
       <c r="E17" t="s">
         <v>32</v>
@@ -3333,48 +3333,48 @@
         <v>72</v>
       </c>
       <c r="G17" t="s">
-        <v>73</v>
+        <v>148</v>
       </c>
       <c r="H17" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="I17" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="J17" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="K17" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="L17" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="M17" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
-        <v>163</v>
+      <c r="A18" s="8" t="s">
+        <v>356</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="C18" t="s">
         <v>16</v>
       </c>
       <c r="D18" t="s">
-        <v>100</v>
+        <v>126</v>
       </c>
       <c r="E18" t="s">
         <v>32</v>
@@ -3386,89 +3386,89 @@
         <v>73</v>
       </c>
       <c r="H18" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="I18" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="J18" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="K18" t="s">
-        <v>113</v>
+        <v>159</v>
       </c>
       <c r="L18" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="M18" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>263</v>
+        <v>250</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P18" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
-        <v>169</v>
-      </c>
-      <c r="B19" t="s">
-        <v>170</v>
+    <row r="19" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A19" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>163</v>
       </c>
       <c r="C19" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="D19" t="s">
-        <v>17</v>
+        <v>100</v>
       </c>
       <c r="E19" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="F19" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="G19" t="s">
-        <v>171</v>
+        <v>73</v>
       </c>
       <c r="H19" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="I19" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="J19" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="K19" t="s">
-        <v>86</v>
+        <v>113</v>
       </c>
       <c r="L19" t="s">
-        <v>175</v>
+        <v>139</v>
       </c>
       <c r="M19" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>270</v>
+        <v>251</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>267</v>
+        <v>248</v>
       </c>
       <c r="P19" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
-        <v>177</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>178</v>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A20" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B20" t="s">
+        <v>169</v>
       </c>
       <c r="C20" t="s">
         <v>42</v>
@@ -3477,154 +3477,154 @@
         <v>17</v>
       </c>
       <c r="E20" t="s">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="F20" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="G20" t="s">
-        <v>82</v>
+        <v>170</v>
       </c>
       <c r="H20" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="I20" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="J20" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="K20" t="s">
         <v>86</v>
       </c>
       <c r="L20" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="M20" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P20" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="270.75" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
-        <v>184</v>
+    <row r="21" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A21" s="8" t="s">
+        <v>176</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="C21" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>126</v>
+        <v>17</v>
       </c>
       <c r="E21" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F21" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="G21" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="H21" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="I21" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="J21" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="K21" t="s">
-        <v>189</v>
+        <v>86</v>
       </c>
       <c r="L21" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="M21" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>268</v>
+        <v>251</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="P21" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
-        <v>192</v>
+    <row r="22" spans="1:16" ht="270.75" x14ac:dyDescent="0.45">
+      <c r="A22" s="8" t="s">
+        <v>183</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="C22" t="s">
         <v>30</v>
       </c>
       <c r="D22" t="s">
-        <v>100</v>
+        <v>126</v>
       </c>
       <c r="E22" t="s">
         <v>32</v>
       </c>
       <c r="F22" t="s">
-        <v>72</v>
+        <v>43</v>
       </c>
       <c r="G22" t="s">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="H22" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="I22" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="J22" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="K22" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="L22" t="s">
-        <v>139</v>
+        <v>189</v>
       </c>
       <c r="M22" t="s">
-        <v>168</v>
+        <v>190</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="P22" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
-        <v>198</v>
+    <row r="23" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A23" s="8" t="s">
+        <v>191</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="C23" t="s">
         <v>30</v>
       </c>
       <c r="D23" t="s">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="E23" t="s">
         <v>32</v>
@@ -3633,228 +3633,228 @@
         <v>72</v>
       </c>
       <c r="G23" t="s">
-        <v>149</v>
+        <v>73</v>
       </c>
       <c r="H23" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="I23" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="J23" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="K23" t="s">
-        <v>77</v>
+        <v>196</v>
       </c>
       <c r="L23" t="s">
-        <v>203</v>
+        <v>139</v>
       </c>
       <c r="M23" t="s">
-        <v>204</v>
+        <v>167</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>269</v>
+        <v>251</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P23" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="57" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
-        <v>205</v>
+    <row r="24" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
+      <c r="A24" s="8" t="s">
+        <v>371</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C24" t="s">
         <v>30</v>
       </c>
       <c r="D24" t="s">
-        <v>17</v>
+        <v>126</v>
       </c>
       <c r="E24" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="F24" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="G24" t="s">
-        <v>20</v>
+        <v>148</v>
       </c>
       <c r="H24" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="I24" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="J24" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="K24" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="L24" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="M24" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="P24" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="399" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
-        <v>381</v>
+    <row r="25" spans="1:16" ht="57" x14ac:dyDescent="0.45">
+      <c r="A25" s="8" t="s">
+        <v>203</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="C25" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D25" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="E25" t="s">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="F25" t="s">
-        <v>72</v>
+        <v>19</v>
       </c>
       <c r="G25" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="H25" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="I25" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="J25" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="K25" t="s">
-        <v>216</v>
+        <v>24</v>
       </c>
       <c r="L25" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="M25" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>262</v>
+        <v>242</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="P25" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
-        <v>219</v>
+    <row r="26" spans="1:16" ht="399" x14ac:dyDescent="0.45">
+      <c r="A26" s="8" t="s">
+        <v>357</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="C26" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D26" t="s">
-        <v>221</v>
+        <v>31</v>
       </c>
       <c r="E26" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="F26" t="s">
         <v>72</v>
       </c>
       <c r="G26" t="s">
-        <v>222</v>
+        <v>73</v>
       </c>
       <c r="H26" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="I26" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="J26" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="K26" t="s">
-        <v>121</v>
+        <v>214</v>
       </c>
       <c r="L26" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="M26" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>272</v>
+        <v>248</v>
       </c>
       <c r="P26" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A27" t="s">
-        <v>228</v>
+    <row r="27" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
+      <c r="A27" s="8" t="s">
+        <v>217</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="C27" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="D27" t="s">
-        <v>31</v>
+        <v>219</v>
       </c>
       <c r="E27" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="F27" t="s">
         <v>72</v>
       </c>
       <c r="G27" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="H27" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="I27" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="J27" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="K27" t="s">
-        <v>86</v>
+        <v>121</v>
       </c>
       <c r="L27" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="M27" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="O27" s="3" t="s">
         <v>260</v>
@@ -3864,17 +3864,17 @@
       </c>
     </row>
     <row r="28" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A28" t="s">
-        <v>236</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>237</v>
+      <c r="A28" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>364</v>
       </c>
       <c r="C28" t="s">
         <v>30</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E28" t="s">
         <v>63</v>
@@ -3883,42 +3883,42 @@
         <v>72</v>
       </c>
       <c r="G28" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="H28" t="s">
-        <v>238</v>
-      </c>
-      <c r="I28" t="s">
-        <v>239</v>
-      </c>
-      <c r="J28" t="s">
-        <v>240</v>
+        <v>227</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>365</v>
       </c>
       <c r="K28" t="s">
         <v>86</v>
       </c>
       <c r="L28" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="M28" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P28" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A29" t="s">
-        <v>243</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>244</v>
+      <c r="A29" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>367</v>
       </c>
       <c r="C29" t="s">
         <v>30</v>
@@ -3927,98 +3927,98 @@
         <v>31</v>
       </c>
       <c r="E29" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="F29" t="s">
         <v>72</v>
       </c>
-      <c r="G29" s="8" t="s">
-        <v>245</v>
+      <c r="G29" t="s">
+        <v>226</v>
       </c>
       <c r="H29" t="s">
-        <v>246</v>
+        <v>227</v>
       </c>
       <c r="I29" t="s">
-        <v>247</v>
-      </c>
-      <c r="J29" t="s">
+        <v>228</v>
+      </c>
+      <c r="J29" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="K29" t="s">
+        <v>86</v>
+      </c>
+      <c r="L29" t="s">
+        <v>229</v>
+      </c>
+      <c r="M29" t="s">
+        <v>230</v>
+      </c>
+      <c r="N29" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="O29" s="3" t="s">
         <v>248</v>
-      </c>
-      <c r="K29" t="s">
-        <v>249</v>
-      </c>
-      <c r="L29" t="s">
-        <v>250</v>
-      </c>
-      <c r="M29" t="s">
-        <v>251</v>
-      </c>
-      <c r="N29" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="O29" s="3" t="s">
-        <v>272</v>
       </c>
       <c r="P29" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="66" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="M30" s="2" t="s">
-        <v>275</v>
+    <row r="30" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A30" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C30" t="s">
+        <v>30</v>
+      </c>
+      <c r="D30" t="s">
+        <v>31</v>
+      </c>
+      <c r="E30" t="s">
+        <v>32</v>
+      </c>
+      <c r="F30" t="s">
+        <v>72</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="H30" t="s">
+        <v>234</v>
+      </c>
+      <c r="I30" t="s">
+        <v>235</v>
+      </c>
+      <c r="J30" t="s">
+        <v>236</v>
+      </c>
+      <c r="K30" t="s">
+        <v>237</v>
+      </c>
+      <c r="L30" t="s">
+        <v>238</v>
+      </c>
+      <c r="M30" t="s">
+        <v>239</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>276</v>
+        <v>259</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="P30" s="3" t="s">
-        <v>277</v>
+        <v>27</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="2" t="s">
-        <v>371</v>
+    <row r="31" spans="1:16" ht="66" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A31" s="6" t="s">
+        <v>261</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>302</v>
+        <v>287</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>42</v>
@@ -4027,48 +4027,48 @@
         <v>17</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>20</v>
+        <v>127</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>281</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>320</v>
+        <v>301</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>321</v>
+        <v>302</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>279</v>
+        <v>262</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>322</v>
+        <v>303</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>323</v>
+        <v>304</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N31" s="3" t="s">
-        <v>280</v>
+        <v>264</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>272</v>
+        <v>245</v>
       </c>
       <c r="P31" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="2" t="s">
-        <v>281</v>
+    <row r="32" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A32" s="6" t="s">
+        <v>349</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>303</v>
+        <v>288</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>42</v>
@@ -4080,48 +4080,48 @@
         <v>32</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>300</v>
+        <v>20</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>324</v>
+        <v>305</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>325</v>
+        <v>306</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>282</v>
+        <v>267</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>95</v>
+        <v>307</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>326</v>
+        <v>308</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N32" s="3" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="O32" s="3" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="P32" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="120" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="2" t="s">
-        <v>283</v>
+    <row r="33" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="6" t="s">
+        <v>269</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>304</v>
+        <v>289</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>17</v>
@@ -4130,48 +4130,48 @@
         <v>32</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>245</v>
+        <v>286</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>92</v>
+        <v>309</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>93</v>
+        <v>310</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>327</v>
+        <v>270</v>
       </c>
       <c r="K33" s="2" t="s">
         <v>95</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>96</v>
+        <v>311</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="O33" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="P33" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="P33" s="3" t="s">
-        <v>277</v>
-      </c>
     </row>
-    <row r="34" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="2" t="s">
-        <v>372</v>
+    <row r="34" spans="1:16" ht="120" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="6" t="s">
+        <v>271</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>305</v>
+        <v>290</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>17</v>
@@ -4180,349 +4180,349 @@
         <v>32</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>20</v>
+        <v>233</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>328</v>
+        <v>92</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>329</v>
+        <v>93</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>285</v>
+        <v>312</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>330</v>
+        <v>96</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N34" s="3" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A35" s="2" t="s">
-        <v>286</v>
+    <row r="35" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A35" s="6" t="s">
+        <v>350</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>306</v>
+        <v>291</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="G35" s="2"/>
+        <v>266</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>20</v>
+      </c>
       <c r="H35" s="2" t="s">
-        <v>331</v>
+        <v>313</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>332</v>
+        <v>314</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>287</v>
+        <v>272</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>86</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>333</v>
+        <v>315</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N35" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="O35" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="P35" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A36" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="M36" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="O35" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="P35" s="3" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="G36" s="6" t="s">
-        <v>299</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>275</v>
-      </c>
       <c r="N36" s="3" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
       <c r="O36" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="P36" s="3" t="s">
         <v>265</v>
-      </c>
-      <c r="P36" s="3" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="37" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="2" t="s">
-        <v>373</v>
+      <c r="A37" s="6" t="s">
+        <v>275</v>
       </c>
       <c r="B37" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="N37" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="O37" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="P37" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A38" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="B38" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D38" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E38" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F37" s="2" t="s">
+      <c r="F38" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G37" s="6" t="s">
+      <c r="G38" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="H38" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="I37" s="2" t="s">
+      <c r="I38" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J37" s="2" t="s">
+      <c r="J38" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K37" s="2" t="s">
+      <c r="K38" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="L37" s="2" t="s">
+      <c r="L38" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="M37" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="N37" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="O37" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="P37" s="3" t="s">
-        <v>277</v>
+      <c r="M38" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="N38" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="O38" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="P38" s="3" t="s">
+        <v>265</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
-      <c r="A38" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>308</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="G38" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="J38" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="K38" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="L38" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="M38" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="N38" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="O38" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="P38" s="3" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A39" s="2" t="s">
-        <v>289</v>
+    <row r="39" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
+      <c r="A39" s="6" t="s">
+        <v>352</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>309</v>
+        <v>294</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>341</v>
+        <v>323</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>342</v>
+        <v>324</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>287</v>
+        <v>272</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>24</v>
+        <v>237</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>343</v>
+        <v>325</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
-    <row r="40" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="2" t="s">
-        <v>290</v>
+    <row r="40" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A40" s="6" t="s">
+        <v>276</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>310</v>
+        <v>295</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G40" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="G40" s="6" t="s">
         <v>73</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>344</v>
+        <v>326</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>345</v>
+        <v>327</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>291</v>
+        <v>274</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>346</v>
+        <v>24</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>139</v>
+        <v>328</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>292</v>
+        <v>249</v>
       </c>
       <c r="O40" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="P40" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="P40" s="3" t="s">
+    </row>
+    <row r="41" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A41" s="6" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="41" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="2" t="s">
-        <v>383</v>
-      </c>
       <c r="B41" s="3" t="s">
-        <v>382</v>
+        <v>296</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>31</v>
+        <v>126</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>32</v>
@@ -4534,39 +4534,39 @@
         <v>73</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>347</v>
+        <v>329</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>348</v>
+        <v>330</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>293</v>
+        <v>278</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>216</v>
+        <v>331</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>349</v>
+        <v>139</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>262</v>
+        <v>279</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
     <row r="42" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="2" t="s">
-        <v>294</v>
+      <c r="A42" s="6" t="s">
+        <v>280</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>311</v>
+        <v>297</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>16</v>
@@ -4578,98 +4578,96 @@
         <v>63</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>350</v>
+        <v>332</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>351</v>
+        <v>333</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>352</v>
+        <v>334</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>353</v>
+        <v>335</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
     <row r="43" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A43" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>312</v>
+      <c r="A43" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>298</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>31</v>
+        <v>100</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>72</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>73</v>
+        <v>109</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>354</v>
+        <v>336</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>355</v>
+        <v>337</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>291</v>
+        <v>339</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>356</v>
+        <v>338</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="M43" s="2" t="s">
-        <v>275</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="M43" s="2"/>
       <c r="N43" s="3" t="s">
-        <v>284</v>
+        <v>264</v>
       </c>
       <c r="O43" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="P43" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="P43" s="3" t="s">
-        <v>277</v>
-      </c>
     </row>
-    <row r="44" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A44" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="B44" s="7" t="s">
-        <v>313</v>
+        <v>282</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>299</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>100</v>
@@ -4678,49 +4676,48 @@
         <v>32</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G44" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G44" s="8" t="s">
         <v>109</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>358</v>
+        <v>340</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>361</v>
+        <v>343</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>360</v>
+        <v>113</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="M44" s="2"/>
+        <v>342</v>
+      </c>
       <c r="N44" s="3" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="P44" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
     <row r="45" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A45" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>314</v>
+      <c r="A45" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>300</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>42</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>100</v>
+        <v>126</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>32</v>
@@ -4732,137 +4729,90 @@
         <v>109</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>362</v>
+        <v>344</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>363</v>
+        <v>345</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>365</v>
+        <v>347</v>
       </c>
       <c r="K45" s="2" t="s">
         <v>113</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>364</v>
+        <v>346</v>
       </c>
       <c r="N45" s="3" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="O45" s="3" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="P45" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
     <row r="46" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A46" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="B46" s="9" t="s">
-        <v>315</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="G46" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="H46" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="I46" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="J46" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="L46" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="N46" s="3" t="s">
-        <v>276</v>
-      </c>
-      <c r="O46" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="P46" s="3" t="s">
-        <v>277</v>
+      <c r="A46" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="47" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A47" s="2" t="s">
+      <c r="A47" s="8" t="s">
         <v>370</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A48" t="s">
-        <v>378</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>379</v>
-      </c>
-      <c r="C48" t="s">
+        <v>355</v>
+      </c>
+      <c r="C47" t="s">
         <v>42</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D47" t="s">
         <v>126</v>
       </c>
-      <c r="E48" t="s">
+      <c r="E47" t="s">
         <v>32</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F47" t="s">
         <v>72</v>
       </c>
-      <c r="G48" t="s">
+      <c r="G47" t="s">
         <v>73</v>
       </c>
-      <c r="H48" t="s">
+      <c r="H47" t="s">
         <v>141</v>
       </c>
-      <c r="I48" t="s">
+      <c r="I47" t="s">
         <v>142</v>
       </c>
-      <c r="J48" t="s">
+      <c r="J47" t="s">
         <v>143</v>
       </c>
-      <c r="K48" t="s">
+      <c r="K47" t="s">
         <v>144</v>
       </c>
-      <c r="L48" t="s">
+      <c r="L47" t="s">
         <v>145</v>
       </c>
-      <c r="M48" t="s">
+      <c r="M47" t="s">
         <v>146</v>
       </c>
-      <c r="N48" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="O48" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="P48" s="3" t="s">
+      <c r="N47" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="O47" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="P47" s="3" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P48" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:P47" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Mettre à jour la bibliothèque de prompts au 2 septembre 2026
Publie le classeur à 46 prompts et déclenche la régénération du site.
</commit_message>
<xml_diff>
--- a/data/BibliothèquePrompt.xlsx
+++ b/data/BibliothèquePrompt.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00_Nexellia\04_PRESTATIONS\Valeurs &amp; Talents\BibliothèquePrompt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87B3E938-733D-44EE-9FC9-F1994C6C5E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{375C7924-B2FA-4393-B6A3-71EA752EB589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22740" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-6060" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="_Data" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">_Data!$A$1:$P$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">_Data!$A$1:$P$47</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="372">
   <si>
     <t>Nom</t>
   </si>
@@ -773,9 +773,6 @@
     <t>Avoir défini la séquence 3A (Prompt P008).</t>
   </si>
   <si>
-    <t>Définition Persona et Enjeux</t>
-  </si>
-  <si>
     <t>## Rôle
 Agis en tant que formateur expérimenté en entreprise et spécialiste de la thématique &lt;A compléter en fonction de votre contexte&gt;. Tu es expert Qualiopi et tu connais toutes les exigences réglementaires du référentiel. Tu es en particulier au fait de toutes les pédagogies favorisant l'inclusion et limitant les risques de mises en situation de handicap (notamment au niveau des supports pédagogiques qui seront générés et notamment les maladies en dys, la malvoyance, le daltonisme… les jeux et mises en situation que tu proposeras pourront être réalisées par des personnes en PMR).
 ## Objectif
@@ -1119,9 +1116,6 @@
     <t>Développer des contenus de formation • Concevoir des supports multimédias • Stimuler l'engagement d'apprenants</t>
   </si>
   <si>
-    <t>Liste Compétences à travailler (Taxonomie Bloom)</t>
-  </si>
-  <si>
     <t>## Rôle
 Agis en tant qu'expert en ingénierie pédagogique. Tu maîtrises toutes les techniques pédagogiques modernes, participatives. Tu maîtrises la ludopédagogie et la taxonomie de Bloom. Tu es expert Qualiopi et tu connais toutes les exigences réglementaires du référentiel. Tu es en particulier au fait de toutes les pédagogies favorisant l'inclusion et limitant les risques de mises en situation de handicap (notamment au niveau des supports pédagogiques qui seront générés et notamment les maladies en dys, la malvoyance, le daltonisme… les jeux et mises en situation que tu proposeras pourront être réalisées par des personnes en PMR).
 ## Objectif
@@ -1254,36 +1248,6 @@
     <t>Avoir un PDF de newsletter.</t>
   </si>
   <si>
-    <t>Script Slides Gamma</t>
-  </si>
-  <si>
-    <t>## Rôle
-Tu es un expert en pédagogie inclusive et en conception de supports de formation professionnelle. Tu maîtrises parfaitement l'outil Gamma.app, les contraintes d'accessibilité (troubles DYS, daltonisme), et les bonnes pratiques de conception graphique pour des contenus impactants et inclusifs.
-## Compétences mobilisées
-- Structuration pédagogique claire et accessible
-- Synthèse et vulgarisation de contenus de formation
-- Design de présentation optimisé pour Gamma (visibilité, rythme, hiérarchie)
-- Conception graphique inclusive (polices, contrastes, couleurs compatibles DYS et daltonisme)
-## Contexte
-Tu dois créer un script de slideshow (8 diapos) à partir d'une séquence de formation professionnelle fournie par l'utilisateur, afin de servir de support d'animation pour un formateur. Ce slideshow sera intégré à Gamma.
-## Objectif
-Transformer une séquence pédagogique brute en 8 slides claires, sans titre visible, pensées pour animer la formation à l'oral (pas pour être lues seules). Elles doivent permettre au formateur de suivre le fil pédagogique, tout en respectant les principes d'accessibilité visuelle.
-## Tâches à réaliser
-1. Demander à l'utilisateur d'uploader la séquence de formation ou le livret stagiaire détaillant la séquence de formation.
-2. Une fois le contenu reçu, proposer un découpage en 8 slides structurées, visuellement attractives, sans surcharge, avec :
-   - Mots-clés ou schémas simples
-   - Éléments visuels sobres mais évocateurs
-   - Contraste fort et police sans serif (OpenDyslexic, Arial, Verdana...)
-   - Aucun rouge/vert direct (éviter le piège daltonien)
-   - Ton professionnel et dynamique
-   - Pas de texte narratif complet : uniquement points clés et visuels supports
-## Contraintes
-- Langue : Français
-- Format : Slides pour Gamma.app (1 idée = 1 slide, design clair, responsive)
-- Accessibilité : Compatible DYS, daltonisme, lecture orale facile
-- Utilisation : Support oral d'animation, non autoportant</t>
-  </si>
-  <si>
     <t>Jour1_Sequence4</t>
   </si>
   <si>
@@ -1293,67 +1257,10 @@
     <t>Création rapide de supports visuels de formation.</t>
   </si>
   <si>
-    <t>Gamma, Support formation, Support stagiaire</t>
-  </si>
-  <si>
     <t>{séquence_formation}</t>
   </si>
   <si>
     <t>Utiliser l'outil Gamma.app par la suite.</t>
-  </si>
-  <si>
-    <t>Script Slides Genspark</t>
-  </si>
-  <si>
-    <t>## Rôle
-Tu es un expert de la plateforme Genspark, graphiste spécialisé en formation professionnelle. Tu maîtrises parfaitement les principes de pédagogie inclusive (troubles DYS, daltonisme, accessibilité cognitive), la conception de slides engageants pour les formateurs, et l'intégration fluide de chartes graphiques.
-## Objectif
-Créer un prompt optimisé à insérer dans Genspark, qui générera un slideshow structuré, impactant et accessible, servant de support d'animation pour une séquence de formation professionnelle.
-## Compétences mobilisées
-- Design pédagogique (clarté, rythme, cohérence)
-- Accessibilité et inclusion (polices sans empattement, contrastes adaptés, pictos clairs)
-- Graphisme orienté formation
-- Connaissance des troubles DYS et exigences RGPD
-- Sens du storytelling et de la hiérarchisation visuelle
-## Tâche
-1. **Demander au formateur** :
-   - Le descriptif précis de la séquence de formation (thème, objectifs, durée, public visé)
-   - Les éléments visuels de la charte graphique à intégrer (couleurs, polices, icônes, logos)
-2. **Générer un prompt à insérer dans Genspark** qui permet :
-   - La création de slides structurées autour des 3A (Appel – Apport – Ancrage)
-   - L'invitation à uploader un **logo** du client
-   - L'utilisation d'un **exemple de présentation réussie** comme source d'inspiration visuelle
-## Processus
-- Analyser le contenu fourni par le formateur
-- Extraire les messages clés à placer dans le slideshow (en évitant le texte "lourd")
-- Générer un enchaînement logique et dynamique des diapos (max 8)
-- Rédiger les indications à intégrer dans Genspark pour que l'outil produise une présentation attractive et inclusive
-## Caractéristiques du prompt final
-- Langage inclusif et clair
-- Consignes précises pour le design : contraste élevé, structure par blocs, icônes explicites
-- Éviter toute donnée nominative ou sensible (RGPD)
-- Support animé oralement : ne pas tout écrire sur les slides, prévoir un usage en support d'animation
----
-Souhaites-tu que je passe à la **rédaction du prompt à coller dans Genspark** maintenant ? Si oui, il me faudrait :
-1. Le descriptif de la **séquence pédagogique concernée**
-2. Les **éléments de charte graphique** (codes couleurs, typo, logo si possible)
-3. Un lien ou une description d'un **exemple de présentation réussie** que tu veux prendre comme modèle
-Une fois ces 3 éléments fournis, je te fournis le prompt Genspark finalisé. On y va ?</t>
-  </si>
-  <si>
-    <t>Générer un prompt spécifique à coller dans Genspark pour créer une présentation pédagogique inclusive.</t>
-  </si>
-  <si>
-    <t>Création de slides via Genspark.</t>
-  </si>
-  <si>
-    <t>Genspark, Support formation, Support stagiaire</t>
-  </si>
-  <si>
-    <t>{charte_graphique}, {descriptif_séquence}, {exemple_modèle}</t>
-  </si>
-  <si>
-    <t>Utiliser l'outil Genspark.</t>
   </si>
   <si>
     <t>Veille IA Formation</t>
@@ -1500,9 +1407,6 @@
     <t>Automatisation_ Création des assistants IA</t>
   </si>
   <si>
-    <t>C2; C8</t>
-  </si>
-  <si>
     <t>ChatGPT, Gemini</t>
   </si>
   <si>
@@ -1525,9 +1429,6 @@
   </si>
   <si>
     <t>C3; C8</t>
-  </si>
-  <si>
-    <t>Genspark</t>
   </si>
   <si>
     <t>Prompt pour la recherche approfondie</t>
@@ -1763,35 +1664,6 @@
   </si>
   <si>
     <t>## Rôle
-Tu es un expert pédagogique, spécialiste de la formation.
-## Objectif
-À partir du brief fourni par l'utilisateur, générer un programme de formation complet au format texte respectant le schéma défini.
-## Règles de génération du contenu
-Le programme doit contenir les éléments principaux suivants :
-1. **Titre de la formation** : proposer un titre basé sur le brief ; si explicitement donné, le reprendre, sinon proposer un titre approprié.
-2. **Description en quelques lignes** : description attractive basée sur le brief, donnant envie d'assister à la formation (5 phrases maximum).
-3. **Durée** : durée si précisée dans le brief, sinon mettre « À remplir ».
-4. **Profil stagiaire** : profil basé sur le brief ; si explicitement donné, le reprendre, sinon proposer un profil approprié (10 mots maximum).
-5. **Délai d'accès** : « 2 semaines » par défaut, sauf mention contraire du brief.
-6. **Objectif général** : objectif général basé sur le brief ; si explicitement donné, le reprendre, sinon proposer un objectif approprié.
-7. **Prérequis** : « Aucun » par défaut, sauf mention contraire du brief.
-8. **Modalités pédagogiques** : indiquer présentielle, distancielle ou mixte, basé sur le brief ; si non précisé, « À remplir ».
-9. **Prix** : « Selon devis ».
-10. **En savoir plus** : « +33 6 81 25 53 88 (entre 8h30 et 19h en semaine) ou mickael.loeuille@valeurs-et-talents.fr ».
-11. **Lieu de formation** : lieu si précisé dans le brief, sinon « À remplir ».
-12. **Objectifs** : 5 objectifs maximum, rédigés selon la taxonomie de Bloom, basés sur le brief client.
-13. **Déroulé détaillé de la formation** : déroulé pédagogique détaillé et timé, basé sur la durée du brief (ou, si non précisée, un déroulé séquencé répondant aux objectifs). Chaque séquence est rédigée comme suit :
-   - Séquence n° [numéro]
-   - [Titre de la séquence]
-   - Durée : [durée]
-   - Objectif : [objectif visé pour cette séquence]
-   - [Description détaillée de la séquence]
-14. **Organisation de la formation** : « Équipe pédagogique : un formateur expert de la formation professionnelle, et dans la thématique de formation. Moyens pédagogiques et techniques : support de formation, dispositif de suivi de l'exécution et de l'évaluation des résultats de la formation, ateliers de mise en pratique tout au long de la formation, QCM ».
-15. **Modalités et délais d'accès** : « Accessibilité / Handicap : nos formations sont ouvertes à tous. En cas de doute, nous invitons à prendre contact directement avec notre référent handicap, en amont de la formation, pour discuter et, au besoin, adapter notre pédagogie et nos activités en fonction des situations de handicap qui pourraient se présenter. Le cas échéant, si nous ne sommes pas en mesure de vous accueillir, nous saurons vous orienter vers notre partenaire l'Agefiph. Contact : mickael.loeuille@valeurs-et-talents.fr / 06 81 25 53 88. Modalité et délai d'accès : notre organisme de formation s'engage à répondre en 48h à toute demande d'information. Une fois le contact établi, nous envisagerons conjointement la date la plus appropriée en fonction de vos besoins et de vos enjeux. Sauf cas particulier, la mise en place de la formation pourra se faire dans les 15 jours suivant votre demande. Pour toute information, nous contacter par mail ou téléphone : mickael.loeuille@valeurs-et-talents.fr — 06 81 25 53 88 (8h30-19h30 tous les jours de la semaine) ».
-16. **Nos indicateurs de performance et de qualité** : « Net Promoter Score : ».</t>
-  </si>
-  <si>
-    <t>## Rôle
 Tu es un producteur audio spécialisé dans la création de présentations de formations engageantes et persuasives.
 ## Objectif
 Générer un script audio, puis le transformer en narration fluide, professionnelle et dynamique.
@@ -1977,15 +1849,6 @@
     <t>Développer des contenus de formation • Stimuler l'engagement d'apprenants</t>
   </si>
   <si>
-    <t>Générer un programme de formation au format Qualiopi/Digiforma à partir d'un brief et d'un template, via Genspark.</t>
-  </si>
-  <si>
-    <t>Création du document programme de formation conforme au référentiel Qualiopi.</t>
-  </si>
-  <si>
-    <t>{brief_formation}, {template_programme}</t>
-  </si>
-  <si>
     <t>Concevoir une offre et une formation complète sur le management à distance et les équipes hybrides, avec étude de marché, supports et podcast promotionnel.</t>
   </si>
   <si>
@@ -1998,18 +1861,6 @@
     <t>{formation_standard_manager}, {programme_vierge}, {exemple_déroulé_pédagogique}, {exemple_livret_stagiaire}</t>
   </si>
   <si>
-    <t>Générer un programme de formation complet et structuré à partir d'un brief, selon un schéma texte prédéfini.</t>
-  </si>
-  <si>
-    <t>Création rapide d'un programme de formation standardisé.</t>
-  </si>
-  <si>
-    <t>Automatiser la gestion administrative • Développer des contenus de formation</t>
-  </si>
-  <si>
-    <t>{brief_formation}</t>
-  </si>
-  <si>
     <t>Générer le script d'une présentation audio persuasive pour promouvoir une formation.</t>
   </si>
   <si>
@@ -2065,12 +1916,6 @@
   </si>
   <si>
     <t xml:space="preserve">5_Création de chaque séquence de formation </t>
-  </si>
-  <si>
-    <t>7_Création Livret Stagiaire</t>
-  </si>
-  <si>
-    <t>7.1_Création Livret Stagiaire_HTML</t>
   </si>
   <si>
     <t># Prompt — Transformation de support de formation en livret HTML interactif
@@ -2114,34 +1959,6 @@
   </si>
   <si>
     <t>## Rôle
-Tu es un expert en ingénierie pédagogique, maîtrisant parfaitement les exigences du référentiel Qualiopi (notamment les indicateurs 1 et 2) et les formats attendus dans l'outil Digiforma. Tu es aussi expert graphiste, designer, et tu sais respecter au mieux les chartes graphiques des templates qu'on te met en pièce jointe.
-## Objectif
-Construire un programme de formation au bon format.
-## Contraintes
-1. Tu reçois en entrée :
-   - Un brief de formation (en fichier joint)
-   - Un template de programme (modèle de l'entreprise, conforme Digiforma/Qualiopi) au format .pptx, format A4 portrait, police Calibri, corps de texte noir
-2. À partir de ces deux documents :
-   - Tu complètes intégralement le programme de formation dans le respect strict du modèle fourni
-   - Tu respectes les titres, l'ordre, le vocabulaire et la mise en forme du template
-   - Tu n'inventes rien : tu t'appuies uniquement sur le brief client, sauf mention explicite t'autorisant à compléter certains points
-3. Tu produis un livrable :
-   - Une diapositive reprenant fidèlement la mise en page du modèle initial, avec les contenus insérés aux bons endroits
-4. Avant de rendre, tu vérifies que :
-   - Le programme est cohérent, synthétique et structuré
-   - Il contient les objectifs pédagogiques, les modalités d'évaluation, le public cible, les prérequis, la durée, la progression pédagogique, etc.
-   - Il respecte les critères de clarté, de lisibilité et de pertinence Qualiopi
-⚠️ En cas de doute ou d'information manquante dans le brief, indique-le dans le programme entre crochets [à compléter] sans inventer.
-À présent, génère le programme à partir des deux fichiers joints.</t>
-  </si>
-  <si>
-    <t>2.5_Le prompt permettant de générer le bon programme de formation au format Qualiopi</t>
-  </si>
-  <si>
-    <t>2.5_Le prompt créateur de programme</t>
-  </si>
-  <si>
-    <t>## Rôle
 Tu es un copywriter expert en marketing de la formation professionnelle. Tu maîtrises les structures persuasives orientées transformation (avant/après), la rédaction centrée bénéfices apprenants, et les codes visuels des plaquettes commerciales B2B.
 ## Objectif
 Générer le contenu complet d'une plaquette de présentation commerciale pour le programme de formation fourni, afin de donner envie au lecteur de s'inscrire dès le premier jour, en utilisant le design système pour la mise en forme.
@@ -2165,6 +1982,189 @@
    Critères d'adéquation positifs (profils qui bénéficient pleinement) et 1 critère d'exclusion (pour qui ce n'est PAS fait — renforce la crédibilité).
 6. Appel à l'action
    1 phrase de clôture forte + 3 micro-CTA au choix : télécharger le programme, contacter un conseiller, s'inscrire directement. Format web-ready (texte de bouton + URL placeholder).</t>
+  </si>
+  <si>
+    <t>1_Définition Persona et Enjeux</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autocritque </t>
+  </si>
+  <si>
+    <t>## Rôle
+Agis en tant que relecteur critique expert en ingénierie de prompts. Passe en revue les réponses proposées par d'autres IA ou par l'utilisateur.
+## Objectif
+Identifie les forces et faiblesses de la réponse analyse et donne une note de 0 à 5. Justifie ta réponse et propose au moins 3 améliorations concrètes. 
+## Contraintes
+Sois factuel et rigoureux, sans complésance. Structure : « Analyse critique », « Suggestions d'amélioration », « Conclusion sur la qualité de la réponse ». Si la réponse est incomplete, formule une version optimisée.</t>
+  </si>
+  <si>
+    <t>Evaluation d'une réponse.</t>
+  </si>
+  <si>
+    <t>7_Script contenu de Slides</t>
+  </si>
+  <si>
+    <t>## Rôle
+Tu es un expert en pédagogie inclusive et en conception de supports de formation professionnelle. Tu maîtrises parfaitement  les contraintes d'accessibilité (troubles DYS, daltonisme), et les bonnes pratiques de conception graphique pour des contenus impactants et inclusifs.
+## Compétences mobilisées
+- Structuration pédagogique claire et accessible
+- Synthèse et vulgarisation de contenus de formation
+- Design de présentation optimisé (visibilité, rythme, hiérarchie)
+- Conception graphique inclusive (polices, contrastes, couleurs compatibles DYS et daltonisme)
+## Contexte
+Tu dois créer un script de slideshow  à partir d'une séquence de formation professionnelle fournie par l'utilisateur, afin de servir de support d'animation pour un formateur. 
+## Objectif
+Transformer une séquence pédagogique brute en  slides claires, sans titre visible, pensées pour animer la formation à l'oral (pas pour être lues seules). Elles doivent permettre au formateur de suivre le fil pédagogique, tout en respectant les principes d'accessibilité visuelle.
+## Tâches à réaliser
+1. Demander à l'utilisateur d'uploader la séquence de formation ou le livret stagiaire détaillant la séquence de formation.
+2. Une fois le contenu reçu, proposer un découpage en slides structurées, visuellement attractives, sans surcharge, avec :
+   - Mots-clés ou schémas simples
+   - Éléments visuels sobres mais évocateurs
+   - Contraste fort et police sans serif (OpenDyslexic, Arial, Verdana...)
+   - Aucun rouge/vert direct (éviter le piège daltonien)
+   - Ton professionnel et dynamique
+   - Pas de texte narratif complet : uniquement points clés et visuels supports
+## Contraintes
+- Langue : Français
+- Format : Textes  et consignes claires pour la création de slides (1 idée = 1 slide, design clair, responsive)
+- Accessibilité : Compatible DYS, daltonisme, lecture orale facile
+- Utilisation : Support oral d'animation, non autoportant</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Support formation, Support stagiaire</t>
+  </si>
+  <si>
+    <t>Création rapide du slideshow de formation.</t>
+  </si>
+  <si>
+    <t>## Rôle
+Tu es un expert en pédagogie inclusive et en conception de supports de formation professionnelle. Tu maîtrises parfaitement  les contraintes d'accessibilité (troubles DYS, daltonisme), et les bonnes pratiques de conception graphique pour des contenus impactants et inclusifs.
+## Compétences mobilisées
+- Structuration pédagogique claire et accessible
+- Synthèse et vulgarisation de contenus de formation
+- Design de présentation optimisé (visibilité, rythme, hiérarchie)
+- Conception graphique inclusive (polices, contrastes, couleurs compatibles DYS et daltonisme)
+## Contexte
+Tu dois créer un script de slideshow  à partir d'une séquence de formation professionnelle fournie par l'utilisateur, afin de servir de support d'animation pour un formateur. 
+# RÔLE
+Tu es un expert en conception de supports de formation professionnelle pour adultes,
+spécialisé en pédagogie inclusive et en design graphique accessible. Tu maîtrises :
+- les contraintes liées aux troubles DYS (dyslexie, dyspraxie, dyscalculie)
+- le daltonisme (deutéranopie, protanopie, tritanopie)
+- les normes WCAG 2.1 (niveau AA minimum, AAA pour les éléments critiques)
+- la théorie de la charge cognitive (Sweller) et les principes andragogiques
+---
+# MISSION
+Transforme le script fourni en spécifications de diapositives structurées, 
+pédagogiquement efficaces et entièrement accessibles, en respectant strictement 
+la charte graphique fournie.
+Pour chaque diapositive identifiée dans le script, produis une fiche de 
+spécification complète selon le format défini en section FORMAT DE SORTIE.
+---
+# INPUTS
+## Script complet
+[COLLER LE SCRIPT ICI — inclure pour chaque diapo : numéro, titre,
+contenu brut, intention pédagogique ou notes formateur si disponibles]
+## Charte graphique
+[COLLER LA CHARTE ICI — inclure : palette HEX, typographies (noms + 
+tailles de base), logo, gabarits disponibles, ton éditorial]
+---
+# RÈGLES DE CONCEPTION GRAPHIQUE
+## Principe cardinal
+Une idée = une diapositive. JAMAIS de surcharge. Si le script dépasse ce seuil
+pour une diapo, découpe en plusieurs et signale-le explicitement.
+## Hiérarchie visuelle
+- Titre : accroche ou question, pas un résumé — maximum 8 mots
+- Corps : 3 éléments maximum par diapo (texte + visuel + donnée)
+- Ordre de lecture naturel (haut-gauche → droite → bas) guide le placement
+## Densité et espace
+- Règle du respir : 40 % minimum de la diapositive reste neutre/blanc
+- Marges de sécurité : 8 % minimum sur chaque bord
+- Espacement inter-blocs : ≥ 16 pt
+## Typographie
+- Corps de texte : taille minimale 24 pt (projection) / 18 pt (PDF/lecture)
+- Interlignage : ≥ 1,5x — critique pour les profils DYS
+- JAMAIS de police serif pour les corps de texte : utiliser sans-serif
+  (Arial, Open Sans, Atkinson Hyperlegible en priorité si hors charte)
+- JAMAIS d'italique pur sur les contenus essentiels
+- Gras réservé à 1 seul mot-clé par phrase maximum
+---
+# RÈGLES D'ACCESSIBILITÉ
+## Daltonisme (OBLIGATOIRE)
+- La couleur ne DOIT JAMAIS être le seul vecteur d'information :
+  toujours doubler d'une icône, d'un motif ou d'un libellé
+- Contraste texte/fond : minimum 4,5:1 (WCAG AA), viser 7:1 (AAA)
+  pour les informations critiques
+- Palettes sûres : bleu/orange, bleu/jaune — ÉVITER rouge/vert seuls
+- Signaler tout conflit avec la charte et proposer une alternative conforme
+## Troubles DYS (OBLIGATOIRE)
+- Phrases ≤ 15 mots — une idée par phrase
+- Alignement gauche UNIQUEMENT — jamais de justification
+- Mots-clés : encadrer ou surligner, jamais en italique
+- Puces simples (•) pour les listes non ordonnées
+- Schéma + légende courte &gt; pavé de texte
+- Texte sur image : TOUJOURS avec fond de contraste ou bandeau opaque
+## Structure et navigation
+- Numérotation visible sur chaque diapo : format "X / N_total"
+- Titre visible sur toutes les diapositives, même les visuelles
+- Récapitulatif en fin de séquence thématique (≤ 3 points clés)
+---
+# RÈGLES PÉDAGOGIQUES
+## Ancrage et mémorisation
+- Ouvrir chaque bloc thématique par une question ou une situation-problème
+- Clore chaque bloc par un "retenez que…" ou une synthèse visuelle
+- Intercaler une pause active toutes les 7 à 10 diapositives
+  (question ouverte, réflexion individuelle, ou mini-sondage)
+## Cohérence cognitive
+- Progresser selon la taxonomie de Bloom : chaque diapo sert un objectif
+  opérationnel identifiable (savoir / comprendre / appliquer / analyser)
+- L'exemple concret PRÉCÈDE ou illustre IMMÉDIATEMENT le concept abstrait
+- Charge cognitive : fractionner en séquences de 3 éléments max (Sweller)
+- Animations (si disponibles) : révèlent une information à la fois — jamais décoratives
+---
+# FORMAT DE SORTIE
+Pour chaque diapositive, produis exactement :
+---
+### Diapo [N] — [TITRE AFFICHÉ]
+**Gabarit** : [titre seul / titre + texte / titre + visuel / 2 colonnes /
+              citation / tableau / schéma / pause active / récapitulatif]
+**Texte affiché** :
+[Texte exact à afficher sur la diapositive — respecter les contraintes DYS]
+**Éléments visuels** :
+[Description précise : type (photo / icône / schéma / graphique / pictogramme),
+sujet, style, placement sur la diapo]
+**Palette utilisée** :
+[Références HEX issues de la charte — fond, texte principal, accent, secondaire]
+**Note accessibilité** :
+[Vérification contraste, alternative non-couleur, point DYS spécifique à cette diapo]
+**Note pédagogique** :
+[Objectif Bloom visé, lien avec la séquence, consigne formateur si nécessaire]
+**Alerte** (si applicable) :
+[Diapo découpée depuis le script / Conflit charte-accessibilité / Densité excessive détectée]
+---
+---
+# CONTRAINTES FINALES
+1. RESPECTER la charte : aucune couleur, police ou gabarit hors charte sans
+   justification explicite dans la note accessibilité
+2. Si une contrainte d'accessibilité entre en CONFLIT avec la charte :
+   signaler le conflit, proposer une alternative conforme, ne pas ignorer
+3. Si une diapo du script est TROP DENSE : la découper, numéroter les
+   sous-diapositives (ex. : 4a, 4b), signaler dans le champ Alerte
+4. Numérotation CONTINUE et cohérente sur l'ensemble du jeu final
+5. Si une intention pédagogique est ABSENTE du script pour une diapo,
+   en déduire une à partir du contexte et la signaler comme [déduit]</t>
+  </si>
+  <si>
+    <t>8_Création de Slides</t>
+  </si>
+  <si>
+    <t>9_Création Livret Stagiaire</t>
+  </si>
+  <si>
+    <t>9_Création Livret Stagiaire_HTML</t>
+  </si>
+  <si>
+    <t>2_Liste Compétences à travailler (Taxonomie Bloom)</t>
   </si>
 </sst>
 </file>
@@ -2507,17 +2507,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="40.46484375" customWidth="1"/>
+    <col min="1" max="1" width="40.46484375" style="8" customWidth="1"/>
     <col min="2" max="2" width="120.73046875" customWidth="1"/>
     <col min="7" max="7" width="38" customWidth="1"/>
     <col min="14" max="16" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
@@ -2560,14 +2560,14 @@
         <v>13</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+      <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -2607,17 +2607,17 @@
         <v>26</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="171" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+      <c r="A3" s="8" t="s">
         <v>28</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -2657,17 +2657,17 @@
         <v>39</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="P3" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+      <c r="A4" s="8" t="s">
         <v>40</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -2707,17 +2707,17 @@
         <v>50</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="P4" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="384.75" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+      <c r="A5" s="8" t="s">
         <v>51</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -2757,17 +2757,17 @@
         <v>58</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P5" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="242.25" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+      <c r="A6" s="8" t="s">
         <v>59</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -2807,18 +2807,18 @@
         <v>69</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P6" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>375</v>
+      <c r="A7" s="8" t="s">
+        <v>353</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>70</v>
@@ -2857,17 +2857,17 @@
         <v>79</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P7" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
+      <c r="A8" s="8" t="s">
         <v>80</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -2907,17 +2907,17 @@
         <v>88</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P8" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
+      <c r="A9" s="8" t="s">
         <v>89</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -2957,17 +2957,17 @@
         <v>97</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
       <c r="P9" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
+      <c r="A10" s="8" t="s">
         <v>98</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -3007,17 +3007,17 @@
         <v>106</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="P10" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="128.25" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
+      <c r="A11" s="8" t="s">
         <v>107</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -3057,21 +3057,21 @@
         <v>115</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
       <c r="P11" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>116</v>
+    <row r="12" spans="1:16" ht="128.25" x14ac:dyDescent="0.45">
+      <c r="A12" s="8" t="s">
+        <v>360</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>117</v>
+        <v>361</v>
       </c>
       <c r="C12" t="s">
         <v>61</v>
@@ -3092,7 +3092,7 @@
         <v>118</v>
       </c>
       <c r="I12" t="s">
-        <v>119</v>
+        <v>362</v>
       </c>
       <c r="J12" t="s">
         <v>120</v>
@@ -3107,118 +3107,121 @@
         <v>123</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="P12" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>124</v>
+    <row r="13" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
+      <c r="A13" s="8" t="s">
+        <v>116</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C13" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>126</v>
+        <v>17</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="F13" t="s">
-        <v>127</v>
+        <v>19</v>
       </c>
       <c r="G13" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="H13" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="I13" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="J13" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K13" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="L13" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="M13" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>268</v>
+        <v>242</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
       <c r="P13" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>376</v>
+      <c r="A14" s="8" t="s">
+        <v>124</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="C14" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
         <v>126</v>
       </c>
       <c r="E14" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="F14" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
       <c r="G14" t="s">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="H14" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="I14" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="J14" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="K14" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="L14" t="s">
-        <v>139</v>
+        <v>132</v>
+      </c>
+      <c r="M14" t="s">
+        <v>133</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="P14" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="342" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
-        <v>377</v>
+    <row r="15" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A15" s="8" t="s">
+        <v>354</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C15" t="s">
         <v>42</v>
@@ -3227,7 +3230,7 @@
         <v>126</v>
       </c>
       <c r="E15" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F15" t="s">
         <v>72</v>
@@ -3236,45 +3239,42 @@
         <v>73</v>
       </c>
       <c r="H15" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="I15" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="J15" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="K15" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="L15" t="s">
-        <v>145</v>
-      </c>
-      <c r="M15" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>263</v>
+        <v>250</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P15" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="228" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>147</v>
+    <row r="16" spans="1:16" ht="342" x14ac:dyDescent="0.45">
+      <c r="A16" s="8" t="s">
+        <v>369</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D16" t="s">
-        <v>31</v>
+        <v>126</v>
       </c>
       <c r="E16" t="s">
         <v>32</v>
@@ -3283,48 +3283,48 @@
         <v>72</v>
       </c>
       <c r="G16" t="s">
-        <v>149</v>
+        <v>73</v>
       </c>
       <c r="H16" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="I16" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="J16" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="K16" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="L16" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="M16" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>269</v>
+        <v>251</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P16" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
-        <v>380</v>
+    <row r="17" spans="1:16" ht="228" x14ac:dyDescent="0.45">
+      <c r="A17" s="8" t="s">
+        <v>359</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="C17" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D17" t="s">
-        <v>126</v>
+        <v>31</v>
       </c>
       <c r="E17" t="s">
         <v>32</v>
@@ -3333,48 +3333,48 @@
         <v>72</v>
       </c>
       <c r="G17" t="s">
-        <v>73</v>
+        <v>148</v>
       </c>
       <c r="H17" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="I17" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="J17" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="K17" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="L17" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="M17" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
-        <v>163</v>
+      <c r="A18" s="8" t="s">
+        <v>356</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="C18" t="s">
         <v>16</v>
       </c>
       <c r="D18" t="s">
-        <v>100</v>
+        <v>126</v>
       </c>
       <c r="E18" t="s">
         <v>32</v>
@@ -3386,89 +3386,89 @@
         <v>73</v>
       </c>
       <c r="H18" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="I18" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="J18" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="K18" t="s">
-        <v>113</v>
+        <v>159</v>
       </c>
       <c r="L18" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="M18" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>263</v>
+        <v>250</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P18" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
-        <v>169</v>
-      </c>
-      <c r="B19" t="s">
-        <v>170</v>
+    <row r="19" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A19" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>163</v>
       </c>
       <c r="C19" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="D19" t="s">
-        <v>17</v>
+        <v>100</v>
       </c>
       <c r="E19" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="F19" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="G19" t="s">
-        <v>171</v>
+        <v>73</v>
       </c>
       <c r="H19" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="I19" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="J19" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="K19" t="s">
-        <v>86</v>
+        <v>113</v>
       </c>
       <c r="L19" t="s">
-        <v>175</v>
+        <v>139</v>
       </c>
       <c r="M19" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>270</v>
+        <v>251</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>267</v>
+        <v>248</v>
       </c>
       <c r="P19" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
-        <v>177</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>178</v>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A20" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B20" t="s">
+        <v>169</v>
       </c>
       <c r="C20" t="s">
         <v>42</v>
@@ -3477,154 +3477,154 @@
         <v>17</v>
       </c>
       <c r="E20" t="s">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="F20" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="G20" t="s">
-        <v>82</v>
+        <v>170</v>
       </c>
       <c r="H20" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="I20" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="J20" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="K20" t="s">
         <v>86</v>
       </c>
       <c r="L20" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="M20" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="P20" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="270.75" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
-        <v>184</v>
+    <row r="21" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A21" s="8" t="s">
+        <v>176</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="C21" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>126</v>
+        <v>17</v>
       </c>
       <c r="E21" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F21" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="G21" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="H21" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="I21" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="J21" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="K21" t="s">
-        <v>189</v>
+        <v>86</v>
       </c>
       <c r="L21" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="M21" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>268</v>
+        <v>251</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="P21" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
-        <v>192</v>
+    <row r="22" spans="1:16" ht="270.75" x14ac:dyDescent="0.45">
+      <c r="A22" s="8" t="s">
+        <v>183</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="C22" t="s">
         <v>30</v>
       </c>
       <c r="D22" t="s">
-        <v>100</v>
+        <v>126</v>
       </c>
       <c r="E22" t="s">
         <v>32</v>
       </c>
       <c r="F22" t="s">
-        <v>72</v>
+        <v>43</v>
       </c>
       <c r="G22" t="s">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="H22" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="I22" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="J22" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="K22" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="L22" t="s">
-        <v>139</v>
+        <v>189</v>
       </c>
       <c r="M22" t="s">
-        <v>168</v>
+        <v>190</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="P22" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
-        <v>198</v>
+    <row r="23" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A23" s="8" t="s">
+        <v>191</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="C23" t="s">
         <v>30</v>
       </c>
       <c r="D23" t="s">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="E23" t="s">
         <v>32</v>
@@ -3633,228 +3633,228 @@
         <v>72</v>
       </c>
       <c r="G23" t="s">
-        <v>149</v>
+        <v>73</v>
       </c>
       <c r="H23" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="I23" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="J23" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="K23" t="s">
-        <v>77</v>
+        <v>196</v>
       </c>
       <c r="L23" t="s">
-        <v>203</v>
+        <v>139</v>
       </c>
       <c r="M23" t="s">
-        <v>204</v>
+        <v>167</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>269</v>
+        <v>251</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P23" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="57" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
-        <v>205</v>
+    <row r="24" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
+      <c r="A24" s="8" t="s">
+        <v>371</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C24" t="s">
         <v>30</v>
       </c>
       <c r="D24" t="s">
-        <v>17</v>
+        <v>126</v>
       </c>
       <c r="E24" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="F24" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="G24" t="s">
-        <v>20</v>
+        <v>148</v>
       </c>
       <c r="H24" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="I24" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="J24" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="K24" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="L24" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="M24" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="P24" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="399" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
-        <v>381</v>
+    <row r="25" spans="1:16" ht="57" x14ac:dyDescent="0.45">
+      <c r="A25" s="8" t="s">
+        <v>203</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="C25" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D25" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="E25" t="s">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="F25" t="s">
-        <v>72</v>
+        <v>19</v>
       </c>
       <c r="G25" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="H25" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="I25" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="J25" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="K25" t="s">
-        <v>216</v>
+        <v>24</v>
       </c>
       <c r="L25" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="M25" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>262</v>
+        <v>242</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="P25" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
-        <v>219</v>
+    <row r="26" spans="1:16" ht="399" x14ac:dyDescent="0.45">
+      <c r="A26" s="8" t="s">
+        <v>357</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="C26" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D26" t="s">
-        <v>221</v>
+        <v>31</v>
       </c>
       <c r="E26" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="F26" t="s">
         <v>72</v>
       </c>
       <c r="G26" t="s">
-        <v>222</v>
+        <v>73</v>
       </c>
       <c r="H26" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="I26" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="J26" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="K26" t="s">
-        <v>121</v>
+        <v>214</v>
       </c>
       <c r="L26" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="M26" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>272</v>
+        <v>248</v>
       </c>
       <c r="P26" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A27" t="s">
-        <v>228</v>
+    <row r="27" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
+      <c r="A27" s="8" t="s">
+        <v>217</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="C27" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="D27" t="s">
-        <v>31</v>
+        <v>219</v>
       </c>
       <c r="E27" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="F27" t="s">
         <v>72</v>
       </c>
       <c r="G27" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="H27" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="I27" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="J27" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="K27" t="s">
-        <v>86</v>
+        <v>121</v>
       </c>
       <c r="L27" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="M27" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="O27" s="3" t="s">
         <v>260</v>
@@ -3864,17 +3864,17 @@
       </c>
     </row>
     <row r="28" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A28" t="s">
-        <v>236</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>237</v>
+      <c r="A28" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>364</v>
       </c>
       <c r="C28" t="s">
         <v>30</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E28" t="s">
         <v>63</v>
@@ -3883,42 +3883,42 @@
         <v>72</v>
       </c>
       <c r="G28" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="H28" t="s">
-        <v>238</v>
-      </c>
-      <c r="I28" t="s">
-        <v>239</v>
-      </c>
-      <c r="J28" t="s">
-        <v>240</v>
+        <v>227</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>365</v>
       </c>
       <c r="K28" t="s">
         <v>86</v>
       </c>
       <c r="L28" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="M28" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="P28" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A29" t="s">
-        <v>243</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>244</v>
+      <c r="A29" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>367</v>
       </c>
       <c r="C29" t="s">
         <v>30</v>
@@ -3927,98 +3927,98 @@
         <v>31</v>
       </c>
       <c r="E29" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="F29" t="s">
         <v>72</v>
       </c>
-      <c r="G29" s="8" t="s">
-        <v>245</v>
+      <c r="G29" t="s">
+        <v>226</v>
       </c>
       <c r="H29" t="s">
-        <v>246</v>
+        <v>227</v>
       </c>
       <c r="I29" t="s">
-        <v>247</v>
-      </c>
-      <c r="J29" t="s">
+        <v>228</v>
+      </c>
+      <c r="J29" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="K29" t="s">
+        <v>86</v>
+      </c>
+      <c r="L29" t="s">
+        <v>229</v>
+      </c>
+      <c r="M29" t="s">
+        <v>230</v>
+      </c>
+      <c r="N29" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="O29" s="3" t="s">
         <v>248</v>
-      </c>
-      <c r="K29" t="s">
-        <v>249</v>
-      </c>
-      <c r="L29" t="s">
-        <v>250</v>
-      </c>
-      <c r="M29" t="s">
-        <v>251</v>
-      </c>
-      <c r="N29" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="O29" s="3" t="s">
-        <v>272</v>
       </c>
       <c r="P29" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="66" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="M30" s="2" t="s">
-        <v>275</v>
+    <row r="30" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A30" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C30" t="s">
+        <v>30</v>
+      </c>
+      <c r="D30" t="s">
+        <v>31</v>
+      </c>
+      <c r="E30" t="s">
+        <v>32</v>
+      </c>
+      <c r="F30" t="s">
+        <v>72</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="H30" t="s">
+        <v>234</v>
+      </c>
+      <c r="I30" t="s">
+        <v>235</v>
+      </c>
+      <c r="J30" t="s">
+        <v>236</v>
+      </c>
+      <c r="K30" t="s">
+        <v>237</v>
+      </c>
+      <c r="L30" t="s">
+        <v>238</v>
+      </c>
+      <c r="M30" t="s">
+        <v>239</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>276</v>
+        <v>259</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="P30" s="3" t="s">
-        <v>277</v>
+        <v>27</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="2" t="s">
-        <v>371</v>
+    <row r="31" spans="1:16" ht="66" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A31" s="6" t="s">
+        <v>261</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>302</v>
+        <v>287</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>42</v>
@@ -4027,48 +4027,48 @@
         <v>17</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>20</v>
+        <v>127</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>281</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>320</v>
+        <v>301</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>321</v>
+        <v>302</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>279</v>
+        <v>262</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>322</v>
+        <v>303</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>323</v>
+        <v>304</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N31" s="3" t="s">
-        <v>280</v>
+        <v>264</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>272</v>
+        <v>245</v>
       </c>
       <c r="P31" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="2" t="s">
-        <v>281</v>
+    <row r="32" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A32" s="6" t="s">
+        <v>349</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>303</v>
+        <v>288</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>42</v>
@@ -4080,48 +4080,48 @@
         <v>32</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>300</v>
+        <v>20</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>324</v>
+        <v>305</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>325</v>
+        <v>306</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>282</v>
+        <v>267</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>95</v>
+        <v>307</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>326</v>
+        <v>308</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N32" s="3" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="O32" s="3" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="P32" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="120" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="2" t="s">
-        <v>283</v>
+    <row r="33" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="6" t="s">
+        <v>269</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>304</v>
+        <v>289</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>17</v>
@@ -4130,48 +4130,48 @@
         <v>32</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>245</v>
+        <v>286</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>92</v>
+        <v>309</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>93</v>
+        <v>310</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>327</v>
+        <v>270</v>
       </c>
       <c r="K33" s="2" t="s">
         <v>95</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>96</v>
+        <v>311</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="O33" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="P33" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="P33" s="3" t="s">
-        <v>277</v>
-      </c>
     </row>
-    <row r="34" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="2" t="s">
-        <v>372</v>
+    <row r="34" spans="1:16" ht="120" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="6" t="s">
+        <v>271</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>305</v>
+        <v>290</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>17</v>
@@ -4180,349 +4180,349 @@
         <v>32</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>20</v>
+        <v>233</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>328</v>
+        <v>92</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>329</v>
+        <v>93</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>285</v>
+        <v>312</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>330</v>
+        <v>96</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N34" s="3" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A35" s="2" t="s">
-        <v>286</v>
+    <row r="35" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A35" s="6" t="s">
+        <v>350</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>306</v>
+        <v>291</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="G35" s="2"/>
+        <v>266</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>20</v>
+      </c>
       <c r="H35" s="2" t="s">
-        <v>331</v>
+        <v>313</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>332</v>
+        <v>314</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>287</v>
+        <v>272</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>86</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>333</v>
+        <v>315</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N35" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="O35" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="P35" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A36" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="M36" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="O35" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="P35" s="3" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="G36" s="6" t="s">
-        <v>299</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>275</v>
-      </c>
       <c r="N36" s="3" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
       <c r="O36" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="P36" s="3" t="s">
         <v>265</v>
-      </c>
-      <c r="P36" s="3" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="37" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="2" t="s">
-        <v>373</v>
+      <c r="A37" s="6" t="s">
+        <v>275</v>
       </c>
       <c r="B37" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="N37" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="O37" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="P37" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A38" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="B38" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D38" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E38" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F37" s="2" t="s">
+      <c r="F38" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G37" s="6" t="s">
+      <c r="G38" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="H38" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="I37" s="2" t="s">
+      <c r="I38" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J37" s="2" t="s">
+      <c r="J38" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K37" s="2" t="s">
+      <c r="K38" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="L37" s="2" t="s">
+      <c r="L38" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="M37" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="N37" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="O37" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="P37" s="3" t="s">
-        <v>277</v>
+      <c r="M38" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="N38" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="O38" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="P38" s="3" t="s">
+        <v>265</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
-      <c r="A38" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>308</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="G38" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="J38" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="K38" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="L38" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="M38" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="N38" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="O38" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="P38" s="3" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A39" s="2" t="s">
-        <v>289</v>
+    <row r="39" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
+      <c r="A39" s="6" t="s">
+        <v>352</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>309</v>
+        <v>294</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>341</v>
+        <v>323</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>342</v>
+        <v>324</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>287</v>
+        <v>272</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>24</v>
+        <v>237</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>343</v>
+        <v>325</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
-    <row r="40" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="2" t="s">
-        <v>290</v>
+    <row r="40" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A40" s="6" t="s">
+        <v>276</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>310</v>
+        <v>295</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G40" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="G40" s="6" t="s">
         <v>73</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>344</v>
+        <v>326</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>345</v>
+        <v>327</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>291</v>
+        <v>274</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>346</v>
+        <v>24</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>139</v>
+        <v>328</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>292</v>
+        <v>249</v>
       </c>
       <c r="O40" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="P40" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="P40" s="3" t="s">
+    </row>
+    <row r="41" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A41" s="6" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="41" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="2" t="s">
-        <v>383</v>
-      </c>
       <c r="B41" s="3" t="s">
-        <v>382</v>
+        <v>296</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>31</v>
+        <v>126</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>32</v>
@@ -4534,39 +4534,39 @@
         <v>73</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>347</v>
+        <v>329</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>348</v>
+        <v>330</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>293</v>
+        <v>278</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>216</v>
+        <v>331</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>349</v>
+        <v>139</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>262</v>
+        <v>279</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
     <row r="42" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="2" t="s">
-        <v>294</v>
+      <c r="A42" s="6" t="s">
+        <v>280</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>311</v>
+        <v>297</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>16</v>
@@ -4578,98 +4578,96 @@
         <v>63</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>350</v>
+        <v>332</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>351</v>
+        <v>333</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>352</v>
+        <v>334</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>353</v>
+        <v>335</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
     <row r="43" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A43" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>312</v>
+      <c r="A43" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>298</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>31</v>
+        <v>100</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>72</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>73</v>
+        <v>109</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>354</v>
+        <v>336</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>355</v>
+        <v>337</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>291</v>
+        <v>339</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>356</v>
+        <v>338</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="M43" s="2" t="s">
-        <v>275</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="M43" s="2"/>
       <c r="N43" s="3" t="s">
-        <v>284</v>
+        <v>264</v>
       </c>
       <c r="O43" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="P43" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="P43" s="3" t="s">
-        <v>277</v>
-      </c>
     </row>
-    <row r="44" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A44" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="B44" s="7" t="s">
-        <v>313</v>
+        <v>282</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>299</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>100</v>
@@ -4678,49 +4676,48 @@
         <v>32</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G44" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G44" s="8" t="s">
         <v>109</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>358</v>
+        <v>340</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>361</v>
+        <v>343</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>360</v>
+        <v>113</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="M44" s="2"/>
+        <v>342</v>
+      </c>
       <c r="N44" s="3" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="P44" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
     <row r="45" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A45" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>314</v>
+      <c r="A45" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>300</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>42</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>100</v>
+        <v>126</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>32</v>
@@ -4732,137 +4729,90 @@
         <v>109</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>362</v>
+        <v>344</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>363</v>
+        <v>345</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>365</v>
+        <v>347</v>
       </c>
       <c r="K45" s="2" t="s">
         <v>113</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>364</v>
+        <v>346</v>
       </c>
       <c r="N45" s="3" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="O45" s="3" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="P45" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
     <row r="46" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A46" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="B46" s="9" t="s">
-        <v>315</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="G46" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="H46" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="I46" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="J46" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="L46" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="N46" s="3" t="s">
-        <v>276</v>
-      </c>
-      <c r="O46" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="P46" s="3" t="s">
-        <v>277</v>
+      <c r="A46" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="47" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A47" s="2" t="s">
+      <c r="A47" s="8" t="s">
         <v>370</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
-      <c r="A48" t="s">
-        <v>378</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>379</v>
-      </c>
-      <c r="C48" t="s">
+        <v>355</v>
+      </c>
+      <c r="C47" t="s">
         <v>42</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D47" t="s">
         <v>126</v>
       </c>
-      <c r="E48" t="s">
+      <c r="E47" t="s">
         <v>32</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F47" t="s">
         <v>72</v>
       </c>
-      <c r="G48" t="s">
+      <c r="G47" t="s">
         <v>73</v>
       </c>
-      <c r="H48" t="s">
+      <c r="H47" t="s">
         <v>141</v>
       </c>
-      <c r="I48" t="s">
+      <c r="I47" t="s">
         <v>142</v>
       </c>
-      <c r="J48" t="s">
+      <c r="J47" t="s">
         <v>143</v>
       </c>
-      <c r="K48" t="s">
+      <c r="K47" t="s">
         <v>144</v>
       </c>
-      <c r="L48" t="s">
+      <c r="L47" t="s">
         <v>145</v>
       </c>
-      <c r="M48" t="s">
+      <c r="M47" t="s">
         <v>146</v>
       </c>
-      <c r="N48" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="O48" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="P48" s="3" t="s">
+      <c r="N47" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="O47" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="P47" s="3" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P48" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:P47" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualiser deux prompts de création de slides
</commit_message>
<xml_diff>
--- a/data/BibliothèquePrompt.xlsx
+++ b/data/BibliothèquePrompt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00_Nexellia\04_PRESTATIONS\Valeurs &amp; Talents\BibliothèquePrompt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{375C7924-B2FA-4393-B6A3-71EA752EB589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{396A56F5-BA2D-4C3D-8E78-1FBCE21BA2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-6060" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="371">
   <si>
     <t>Nom</t>
   </si>
@@ -1246,9 +1246,6 @@
   </si>
   <si>
     <t>Avoir un PDF de newsletter.</t>
-  </si>
-  <si>
-    <t>Jour1_Sequence4</t>
   </si>
   <si>
     <t>Préparer le script textuel optimisé pour générer automatiquement une présentation via l'outil Gamma.</t>
@@ -2507,6 +2504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:P47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -2560,13 +2558,13 @@
         <v>13</v>
       </c>
       <c r="O1" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="P1" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="P1" s="5" t="s">
-        <v>241</v>
-      </c>
     </row>
-    <row r="2" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
@@ -2607,16 +2605,16 @@
         <v>26</v>
       </c>
       <c r="N2" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="O2" s="3" t="s">
         <v>242</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>243</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="171" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:16" ht="171" hidden="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
         <v>28</v>
       </c>
@@ -2657,16 +2655,16 @@
         <v>39</v>
       </c>
       <c r="N3" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="O3" s="3" t="s">
         <v>244</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>245</v>
       </c>
       <c r="P3" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
         <v>40</v>
       </c>
@@ -2707,16 +2705,16 @@
         <v>50</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="P4" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="384.75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:16" ht="384.75" hidden="1" x14ac:dyDescent="0.45">
       <c r="A5" s="8" t="s">
         <v>51</v>
       </c>
@@ -2757,16 +2755,16 @@
         <v>58</v>
       </c>
       <c r="N5" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="O5" s="3" t="s">
         <v>247</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>248</v>
       </c>
       <c r="P5" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="242.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:16" ht="242.25" hidden="1" x14ac:dyDescent="0.45">
       <c r="A6" s="8" t="s">
         <v>59</v>
       </c>
@@ -2807,18 +2805,18 @@
         <v>69</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P6" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A7" s="8" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>70</v>
@@ -2857,16 +2855,16 @@
         <v>79</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P7" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:16" ht="370.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A8" s="8" t="s">
         <v>80</v>
       </c>
@@ -2907,16 +2905,16 @@
         <v>88</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P8" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A9" s="8" t="s">
         <v>89</v>
       </c>
@@ -2957,16 +2955,16 @@
         <v>97</v>
       </c>
       <c r="N9" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="O9" s="3" t="s">
         <v>252</v>
-      </c>
-      <c r="O9" s="3" t="s">
-        <v>253</v>
       </c>
       <c r="P9" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:16" ht="199.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A10" s="8" t="s">
         <v>98</v>
       </c>
@@ -3007,16 +3005,16 @@
         <v>106</v>
       </c>
       <c r="N10" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="O10" s="3" t="s">
         <v>244</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>245</v>
       </c>
       <c r="P10" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:16" ht="128.25" hidden="1" x14ac:dyDescent="0.45">
       <c r="A11" s="8" t="s">
         <v>107</v>
       </c>
@@ -3057,21 +3055,21 @@
         <v>115</v>
       </c>
       <c r="N11" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="O11" s="3" t="s">
         <v>254</v>
-      </c>
-      <c r="O11" s="3" t="s">
-        <v>255</v>
       </c>
       <c r="P11" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:16" ht="128.25" hidden="1" x14ac:dyDescent="0.45">
       <c r="A12" s="8" t="s">
+        <v>359</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>360</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>361</v>
       </c>
       <c r="C12" t="s">
         <v>61</v>
@@ -3092,7 +3090,7 @@
         <v>118</v>
       </c>
       <c r="I12" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="J12" t="s">
         <v>120</v>
@@ -3107,16 +3105,16 @@
         <v>123</v>
       </c>
       <c r="N12" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="O12" s="3" t="s">
         <v>242</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>243</v>
       </c>
       <c r="P12" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:16" ht="142.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A13" s="8" t="s">
         <v>116</v>
       </c>
@@ -3157,16 +3155,16 @@
         <v>123</v>
       </c>
       <c r="N13" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="O13" s="3" t="s">
         <v>242</v>
-      </c>
-      <c r="O13" s="3" t="s">
-        <v>243</v>
       </c>
       <c r="P13" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A14" s="8" t="s">
         <v>124</v>
       </c>
@@ -3207,18 +3205,18 @@
         <v>133</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="P14" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A15" s="8" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>134</v>
@@ -3254,18 +3252,18 @@
         <v>139</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P15" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="342" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:16" ht="342" hidden="1" x14ac:dyDescent="0.45">
       <c r="A16" s="8" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>140</v>
@@ -3304,18 +3302,18 @@
         <v>146</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P16" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="228" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:16" ht="228" hidden="1" x14ac:dyDescent="0.45">
       <c r="A17" s="8" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>147</v>
@@ -3354,18 +3352,18 @@
         <v>154</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A18" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>155</v>
@@ -3404,16 +3402,16 @@
         <v>161</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P18" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A19" s="8" t="s">
         <v>162</v>
       </c>
@@ -3454,16 +3452,16 @@
         <v>167</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P19" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.45">
       <c r="A20" s="8" t="s">
         <v>168</v>
       </c>
@@ -3504,16 +3502,16 @@
         <v>175</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="P20" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A21" s="8" t="s">
         <v>176</v>
       </c>
@@ -3554,16 +3552,16 @@
         <v>182</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P21" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="270.75" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:16" ht="270.75" hidden="1" x14ac:dyDescent="0.45">
       <c r="A22" s="8" t="s">
         <v>183</v>
       </c>
@@ -3604,16 +3602,16 @@
         <v>190</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="P22" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A23" s="8" t="s">
         <v>191</v>
       </c>
@@ -3654,18 +3652,18 @@
         <v>167</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P23" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:16" ht="199.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A24" s="8" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>197</v>
@@ -3704,16 +3702,16 @@
         <v>202</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P24" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="57" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:16" ht="57" hidden="1" x14ac:dyDescent="0.45">
       <c r="A25" s="8" t="s">
         <v>203</v>
       </c>
@@ -3754,18 +3752,18 @@
         <v>209</v>
       </c>
       <c r="N25" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="O25" s="3" t="s">
         <v>242</v>
-      </c>
-      <c r="O25" s="3" t="s">
-        <v>243</v>
       </c>
       <c r="P25" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="399" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:16" ht="399" hidden="1" x14ac:dyDescent="0.45">
       <c r="A26" s="8" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>210</v>
@@ -3804,16 +3802,16 @@
         <v>216</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P26" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:16" ht="370.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A27" s="8" t="s">
         <v>217</v>
       </c>
@@ -3854,10 +3852,10 @@
         <v>225</v>
       </c>
       <c r="N27" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="O27" s="3" t="s">
         <v>259</v>
-      </c>
-      <c r="O27" s="3" t="s">
-        <v>260</v>
       </c>
       <c r="P27" s="3" t="s">
         <v>27</v>
@@ -3865,10 +3863,10 @@
     </row>
     <row r="28" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A28" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="B28" s="9" t="s">
         <v>363</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>364</v>
       </c>
       <c r="C28" t="s">
         <v>30</v>
@@ -3883,31 +3881,31 @@
         <v>72</v>
       </c>
       <c r="G28" t="s">
+        <v>73</v>
+      </c>
+      <c r="H28" t="s">
         <v>226</v>
       </c>
-      <c r="H28" t="s">
-        <v>227</v>
-      </c>
       <c r="I28" s="8" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="K28" t="s">
         <v>86</v>
       </c>
       <c r="L28" t="s">
+        <v>228</v>
+      </c>
+      <c r="M28" t="s">
         <v>229</v>
       </c>
-      <c r="M28" t="s">
-        <v>230</v>
-      </c>
       <c r="N28" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P28" s="3" t="s">
         <v>27</v>
@@ -3915,10 +3913,10 @@
     </row>
     <row r="29" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A29" s="8" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C29" t="s">
         <v>30</v>
@@ -3933,42 +3931,42 @@
         <v>72</v>
       </c>
       <c r="G29" t="s">
+        <v>73</v>
+      </c>
+      <c r="H29" t="s">
         <v>226</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>227</v>
       </c>
-      <c r="I29" t="s">
-        <v>228</v>
-      </c>
       <c r="J29" s="8" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="K29" t="s">
         <v>86</v>
       </c>
       <c r="L29" t="s">
+        <v>228</v>
+      </c>
+      <c r="M29" t="s">
         <v>229</v>
       </c>
-      <c r="M29" t="s">
-        <v>230</v>
-      </c>
       <c r="N29" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P29" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A30" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>231</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>232</v>
       </c>
       <c r="C30" t="s">
         <v>30</v>
@@ -3983,42 +3981,42 @@
         <v>72</v>
       </c>
       <c r="G30" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="H30" t="s">
         <v>233</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>234</v>
       </c>
-      <c r="I30" t="s">
+      <c r="J30" t="s">
         <v>235</v>
       </c>
-      <c r="J30" t="s">
+      <c r="K30" t="s">
         <v>236</v>
       </c>
-      <c r="K30" t="s">
+      <c r="L30" t="s">
         <v>237</v>
       </c>
-      <c r="L30" t="s">
+      <c r="M30" t="s">
         <v>238</v>
       </c>
-      <c r="M30" t="s">
-        <v>239</v>
-      </c>
       <c r="N30" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="O30" s="3" t="s">
         <v>259</v>
-      </c>
-      <c r="O30" s="3" t="s">
-        <v>260</v>
       </c>
       <c r="P30" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="66" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:16" ht="66" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>42</v>
@@ -4033,42 +4031,42 @@
         <v>127</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H31" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="I31" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="J31" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="K31" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="J31" s="2" t="s">
+      <c r="L31" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="M31" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="K31" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="M31" s="2" t="s">
+      <c r="N31" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="N31" s="3" t="s">
+      <c r="O31" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="P31" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="O31" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="P31" s="3" t="s">
-        <v>265</v>
-      </c>
     </row>
-    <row r="32" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:16" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="6" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>42</v>
@@ -4080,45 +4078,45 @@
         <v>32</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H32" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="I32" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="J32" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="K32" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="J32" s="2" t="s">
+      <c r="L32" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="N32" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="K32" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="L32" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="N32" s="3" t="s">
+      <c r="O32" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="P32" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="O32" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="P32" s="3" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="6" t="s">
-        <v>269</v>
-      </c>
       <c r="B33" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>42</v>
@@ -4130,45 +4128,45 @@
         <v>32</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="H33" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="I33" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="I33" s="2" t="s">
-        <v>310</v>
-      </c>
       <c r="J33" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="K33" s="2" t="s">
         <v>95</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="P33" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="120" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:16" ht="120" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>16</v>
@@ -4180,10 +4178,10 @@
         <v>32</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>92</v>
@@ -4192,7 +4190,7 @@
         <v>93</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>95</v>
@@ -4201,24 +4199,24 @@
         <v>96</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N34" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="O34" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="O34" s="3" t="s">
-        <v>253</v>
-      </c>
       <c r="P34" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:16" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="6" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>30</v>
@@ -4230,45 +4228,45 @@
         <v>32</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G35" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H35" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="I35" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="I35" s="2" t="s">
-        <v>314</v>
-      </c>
       <c r="J35" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>86</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:16" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>30</v>
@@ -4280,43 +4278,43 @@
         <v>32</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="I36" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="I36" s="2" t="s">
-        <v>317</v>
-      </c>
       <c r="J36" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>86</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:16" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>42</v>
@@ -4328,42 +4326,42 @@
         <v>18</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H37" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="I37" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="I37" s="2" t="s">
+      <c r="J37" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="K37" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="J37" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="K37" s="2" t="s">
+      <c r="L37" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="L37" s="2" t="s">
-        <v>322</v>
-      </c>
       <c r="M37" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N37" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="O37" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="O37" s="3" t="s">
-        <v>253</v>
-      </c>
       <c r="P37" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:16" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="6" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>60</v>
@@ -4399,24 +4397,24 @@
         <v>68</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N38" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="O38" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P38" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="39" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:16" ht="142.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A39" s="6" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>30</v>
@@ -4428,45 +4426,45 @@
         <v>32</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H39" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="I39" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="I39" s="2" t="s">
+      <c r="J39" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="L39" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="J39" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="K39" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="L39" s="2" t="s">
-        <v>325</v>
-      </c>
       <c r="M39" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="40" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:16" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>30</v>
@@ -4478,45 +4476,45 @@
         <v>32</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G40" s="6" t="s">
         <v>73</v>
       </c>
       <c r="H40" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="I40" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="I40" s="2" t="s">
-        <v>327</v>
-      </c>
       <c r="J40" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="K40" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P40" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="41" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:16" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>30</v>
@@ -4534,39 +4532,39 @@
         <v>73</v>
       </c>
       <c r="H41" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="I41" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="J41" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="K41" s="2" t="s">
         <v>330</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>331</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>139</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N41" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="O41" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="P41" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A42" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="O41" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="P41" s="3" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="6" t="s">
-        <v>280</v>
-      </c>
       <c r="B42" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>16</v>
@@ -4578,45 +4576,45 @@
         <v>63</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H42" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="I42" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="I42" s="2" t="s">
+      <c r="J42" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="K42" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="J42" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="K42" s="2" t="s">
+      <c r="L42" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="L42" s="2" t="s">
-        <v>335</v>
-      </c>
       <c r="M42" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="43" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:16" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>30</v>
@@ -4634,37 +4632,37 @@
         <v>109</v>
       </c>
       <c r="H43" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="I43" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="I43" s="2" t="s">
+      <c r="J43" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="K43" s="2" t="s">
         <v>337</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>338</v>
       </c>
       <c r="L43" s="2" t="s">
         <v>139</v>
       </c>
       <c r="M43" s="2"/>
       <c r="N43" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="O43" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="P43" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="O43" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="P43" s="3" t="s">
-        <v>265</v>
-      </c>
     </row>
-    <row r="44" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A44" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>42</v>
@@ -4682,36 +4680,36 @@
         <v>109</v>
       </c>
       <c r="H44" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="I44" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="I44" s="2" t="s">
-        <v>341</v>
-      </c>
       <c r="J44" s="2" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="K44" s="2" t="s">
         <v>113</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="N44" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="O44" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="P44" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="O44" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="P44" s="3" t="s">
-        <v>265</v>
-      </c>
     </row>
-    <row r="45" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A45" s="6" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>42</v>
@@ -4729,44 +4727,44 @@
         <v>109</v>
       </c>
       <c r="H45" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="I45" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="I45" s="2" t="s">
-        <v>345</v>
-      </c>
       <c r="J45" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="K45" s="2" t="s">
         <v>113</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="N45" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="O45" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="P45" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="O45" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="P45" s="3" t="s">
-        <v>265</v>
-      </c>
     </row>
-    <row r="46" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A46" s="6" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
-    <row r="47" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A47" s="8" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C47" t="s">
         <v>42</v>
@@ -4802,17 +4800,23 @@
         <v>146</v>
       </c>
       <c r="N47" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O47" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P47" s="3" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P47" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:P47" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="Jour1_Sequence4"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualiser les prompts de création de slides
Publie les corrections des deux fiches et régénère le site.
</commit_message>
<xml_diff>
--- a/data/BibliothèquePrompt.xlsx
+++ b/data/BibliothèquePrompt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00_Nexellia\04_PRESTATIONS\Valeurs &amp; Talents\BibliothèquePrompt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{375C7924-B2FA-4393-B6A3-71EA752EB589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{396A56F5-BA2D-4C3D-8E78-1FBCE21BA2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-6060" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="371">
   <si>
     <t>Nom</t>
   </si>
@@ -1246,9 +1246,6 @@
   </si>
   <si>
     <t>Avoir un PDF de newsletter.</t>
-  </si>
-  <si>
-    <t>Jour1_Sequence4</t>
   </si>
   <si>
     <t>Préparer le script textuel optimisé pour générer automatiquement une présentation via l'outil Gamma.</t>
@@ -2507,6 +2504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:P47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -2560,13 +2558,13 @@
         <v>13</v>
       </c>
       <c r="O1" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="P1" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="P1" s="5" t="s">
-        <v>241</v>
-      </c>
     </row>
-    <row r="2" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
@@ -2607,16 +2605,16 @@
         <v>26</v>
       </c>
       <c r="N2" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="O2" s="3" t="s">
         <v>242</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>243</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="171" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:16" ht="171" hidden="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
         <v>28</v>
       </c>
@@ -2657,16 +2655,16 @@
         <v>39</v>
       </c>
       <c r="N3" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="O3" s="3" t="s">
         <v>244</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>245</v>
       </c>
       <c r="P3" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
         <v>40</v>
       </c>
@@ -2707,16 +2705,16 @@
         <v>50</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="P4" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="384.75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:16" ht="384.75" hidden="1" x14ac:dyDescent="0.45">
       <c r="A5" s="8" t="s">
         <v>51</v>
       </c>
@@ -2757,16 +2755,16 @@
         <v>58</v>
       </c>
       <c r="N5" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="O5" s="3" t="s">
         <v>247</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>248</v>
       </c>
       <c r="P5" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="242.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:16" ht="242.25" hidden="1" x14ac:dyDescent="0.45">
       <c r="A6" s="8" t="s">
         <v>59</v>
       </c>
@@ -2807,18 +2805,18 @@
         <v>69</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P6" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A7" s="8" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>70</v>
@@ -2857,16 +2855,16 @@
         <v>79</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P7" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:16" ht="370.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A8" s="8" t="s">
         <v>80</v>
       </c>
@@ -2907,16 +2905,16 @@
         <v>88</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P8" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A9" s="8" t="s">
         <v>89</v>
       </c>
@@ -2957,16 +2955,16 @@
         <v>97</v>
       </c>
       <c r="N9" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="O9" s="3" t="s">
         <v>252</v>
-      </c>
-      <c r="O9" s="3" t="s">
-        <v>253</v>
       </c>
       <c r="P9" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:16" ht="199.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A10" s="8" t="s">
         <v>98</v>
       </c>
@@ -3007,16 +3005,16 @@
         <v>106</v>
       </c>
       <c r="N10" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="O10" s="3" t="s">
         <v>244</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>245</v>
       </c>
       <c r="P10" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:16" ht="128.25" hidden="1" x14ac:dyDescent="0.45">
       <c r="A11" s="8" t="s">
         <v>107</v>
       </c>
@@ -3057,21 +3055,21 @@
         <v>115</v>
       </c>
       <c r="N11" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="O11" s="3" t="s">
         <v>254</v>
-      </c>
-      <c r="O11" s="3" t="s">
-        <v>255</v>
       </c>
       <c r="P11" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:16" ht="128.25" hidden="1" x14ac:dyDescent="0.45">
       <c r="A12" s="8" t="s">
+        <v>359</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>360</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>361</v>
       </c>
       <c r="C12" t="s">
         <v>61</v>
@@ -3092,7 +3090,7 @@
         <v>118</v>
       </c>
       <c r="I12" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="J12" t="s">
         <v>120</v>
@@ -3107,16 +3105,16 @@
         <v>123</v>
       </c>
       <c r="N12" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="O12" s="3" t="s">
         <v>242</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>243</v>
       </c>
       <c r="P12" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:16" ht="142.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A13" s="8" t="s">
         <v>116</v>
       </c>
@@ -3157,16 +3155,16 @@
         <v>123</v>
       </c>
       <c r="N13" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="O13" s="3" t="s">
         <v>242</v>
-      </c>
-      <c r="O13" s="3" t="s">
-        <v>243</v>
       </c>
       <c r="P13" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A14" s="8" t="s">
         <v>124</v>
       </c>
@@ -3207,18 +3205,18 @@
         <v>133</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="P14" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A15" s="8" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>134</v>
@@ -3254,18 +3252,18 @@
         <v>139</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P15" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="342" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:16" ht="342" hidden="1" x14ac:dyDescent="0.45">
       <c r="A16" s="8" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>140</v>
@@ -3304,18 +3302,18 @@
         <v>146</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P16" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="228" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:16" ht="228" hidden="1" x14ac:dyDescent="0.45">
       <c r="A17" s="8" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>147</v>
@@ -3354,18 +3352,18 @@
         <v>154</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A18" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>155</v>
@@ -3404,16 +3402,16 @@
         <v>161</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P18" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A19" s="8" t="s">
         <v>162</v>
       </c>
@@ -3454,16 +3452,16 @@
         <v>167</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P19" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.45">
       <c r="A20" s="8" t="s">
         <v>168</v>
       </c>
@@ -3504,16 +3502,16 @@
         <v>175</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="P20" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A21" s="8" t="s">
         <v>176</v>
       </c>
@@ -3554,16 +3552,16 @@
         <v>182</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P21" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="270.75" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:16" ht="270.75" hidden="1" x14ac:dyDescent="0.45">
       <c r="A22" s="8" t="s">
         <v>183</v>
       </c>
@@ -3604,16 +3602,16 @@
         <v>190</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="P22" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A23" s="8" t="s">
         <v>191</v>
       </c>
@@ -3654,18 +3652,18 @@
         <v>167</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P23" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:16" ht="199.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A24" s="8" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>197</v>
@@ -3704,16 +3702,16 @@
         <v>202</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P24" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="57" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:16" ht="57" hidden="1" x14ac:dyDescent="0.45">
       <c r="A25" s="8" t="s">
         <v>203</v>
       </c>
@@ -3754,18 +3752,18 @@
         <v>209</v>
       </c>
       <c r="N25" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="O25" s="3" t="s">
         <v>242</v>
-      </c>
-      <c r="O25" s="3" t="s">
-        <v>243</v>
       </c>
       <c r="P25" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="399" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:16" ht="399" hidden="1" x14ac:dyDescent="0.45">
       <c r="A26" s="8" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>210</v>
@@ -3804,16 +3802,16 @@
         <v>216</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P26" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:16" ht="370.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A27" s="8" t="s">
         <v>217</v>
       </c>
@@ -3854,10 +3852,10 @@
         <v>225</v>
       </c>
       <c r="N27" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="O27" s="3" t="s">
         <v>259</v>
-      </c>
-      <c r="O27" s="3" t="s">
-        <v>260</v>
       </c>
       <c r="P27" s="3" t="s">
         <v>27</v>
@@ -3865,10 +3863,10 @@
     </row>
     <row r="28" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A28" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="B28" s="9" t="s">
         <v>363</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>364</v>
       </c>
       <c r="C28" t="s">
         <v>30</v>
@@ -3883,31 +3881,31 @@
         <v>72</v>
       </c>
       <c r="G28" t="s">
+        <v>73</v>
+      </c>
+      <c r="H28" t="s">
         <v>226</v>
       </c>
-      <c r="H28" t="s">
-        <v>227</v>
-      </c>
       <c r="I28" s="8" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="K28" t="s">
         <v>86</v>
       </c>
       <c r="L28" t="s">
+        <v>228</v>
+      </c>
+      <c r="M28" t="s">
         <v>229</v>
       </c>
-      <c r="M28" t="s">
-        <v>230</v>
-      </c>
       <c r="N28" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P28" s="3" t="s">
         <v>27</v>
@@ -3915,10 +3913,10 @@
     </row>
     <row r="29" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A29" s="8" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C29" t="s">
         <v>30</v>
@@ -3933,42 +3931,42 @@
         <v>72</v>
       </c>
       <c r="G29" t="s">
+        <v>73</v>
+      </c>
+      <c r="H29" t="s">
         <v>226</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>227</v>
       </c>
-      <c r="I29" t="s">
-        <v>228</v>
-      </c>
       <c r="J29" s="8" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="K29" t="s">
         <v>86</v>
       </c>
       <c r="L29" t="s">
+        <v>228</v>
+      </c>
+      <c r="M29" t="s">
         <v>229</v>
       </c>
-      <c r="M29" t="s">
-        <v>230</v>
-      </c>
       <c r="N29" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P29" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A30" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>231</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>232</v>
       </c>
       <c r="C30" t="s">
         <v>30</v>
@@ -3983,42 +3981,42 @@
         <v>72</v>
       </c>
       <c r="G30" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="H30" t="s">
         <v>233</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>234</v>
       </c>
-      <c r="I30" t="s">
+      <c r="J30" t="s">
         <v>235</v>
       </c>
-      <c r="J30" t="s">
+      <c r="K30" t="s">
         <v>236</v>
       </c>
-      <c r="K30" t="s">
+      <c r="L30" t="s">
         <v>237</v>
       </c>
-      <c r="L30" t="s">
+      <c r="M30" t="s">
         <v>238</v>
       </c>
-      <c r="M30" t="s">
-        <v>239</v>
-      </c>
       <c r="N30" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="O30" s="3" t="s">
         <v>259</v>
-      </c>
-      <c r="O30" s="3" t="s">
-        <v>260</v>
       </c>
       <c r="P30" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="66" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:16" ht="66" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>42</v>
@@ -4033,42 +4031,42 @@
         <v>127</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H31" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="I31" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="J31" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="K31" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="J31" s="2" t="s">
+      <c r="L31" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="M31" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="K31" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="M31" s="2" t="s">
+      <c r="N31" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="N31" s="3" t="s">
+      <c r="O31" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="P31" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="O31" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="P31" s="3" t="s">
-        <v>265</v>
-      </c>
     </row>
-    <row r="32" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:16" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="6" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>42</v>
@@ -4080,45 +4078,45 @@
         <v>32</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H32" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="I32" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="J32" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="K32" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="J32" s="2" t="s">
+      <c r="L32" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="N32" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="K32" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="L32" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="N32" s="3" t="s">
+      <c r="O32" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="P32" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="O32" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="P32" s="3" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="6" t="s">
-        <v>269</v>
-      </c>
       <c r="B33" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>42</v>
@@ -4130,45 +4128,45 @@
         <v>32</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="H33" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="I33" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="I33" s="2" t="s">
-        <v>310</v>
-      </c>
       <c r="J33" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="K33" s="2" t="s">
         <v>95</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="P33" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="120" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:16" ht="120" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>16</v>
@@ -4180,10 +4178,10 @@
         <v>32</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>92</v>
@@ -4192,7 +4190,7 @@
         <v>93</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>95</v>
@@ -4201,24 +4199,24 @@
         <v>96</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N34" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="O34" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="O34" s="3" t="s">
-        <v>253</v>
-      </c>
       <c r="P34" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:16" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="6" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>30</v>
@@ -4230,45 +4228,45 @@
         <v>32</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G35" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H35" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="I35" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="I35" s="2" t="s">
-        <v>314</v>
-      </c>
       <c r="J35" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>86</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:16" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>30</v>
@@ -4280,43 +4278,43 @@
         <v>32</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="I36" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="I36" s="2" t="s">
-        <v>317</v>
-      </c>
       <c r="J36" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>86</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:16" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>42</v>
@@ -4328,42 +4326,42 @@
         <v>18</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H37" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="I37" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="I37" s="2" t="s">
+      <c r="J37" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="K37" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="J37" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="K37" s="2" t="s">
+      <c r="L37" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="L37" s="2" t="s">
-        <v>322</v>
-      </c>
       <c r="M37" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N37" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="O37" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="O37" s="3" t="s">
-        <v>253</v>
-      </c>
       <c r="P37" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:16" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="6" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>60</v>
@@ -4399,24 +4397,24 @@
         <v>68</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N38" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="O38" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P38" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="39" spans="1:16" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:16" ht="142.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A39" s="6" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>30</v>
@@ -4428,45 +4426,45 @@
         <v>32</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H39" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="I39" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="I39" s="2" t="s">
+      <c r="J39" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="L39" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="J39" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="K39" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="L39" s="2" t="s">
-        <v>325</v>
-      </c>
       <c r="M39" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="40" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:16" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>30</v>
@@ -4478,45 +4476,45 @@
         <v>32</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G40" s="6" t="s">
         <v>73</v>
       </c>
       <c r="H40" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="I40" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="I40" s="2" t="s">
-        <v>327</v>
-      </c>
       <c r="J40" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="K40" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P40" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="41" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:16" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>30</v>
@@ -4534,39 +4532,39 @@
         <v>73</v>
       </c>
       <c r="H41" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="I41" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="J41" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="K41" s="2" t="s">
         <v>330</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>331</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>139</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N41" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="O41" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="P41" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A42" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="O41" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="P41" s="3" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="6" t="s">
-        <v>280</v>
-      </c>
       <c r="B42" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>16</v>
@@ -4578,45 +4576,45 @@
         <v>63</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H42" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="I42" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="I42" s="2" t="s">
+      <c r="J42" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="K42" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="J42" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="K42" s="2" t="s">
+      <c r="L42" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="L42" s="2" t="s">
-        <v>335</v>
-      </c>
       <c r="M42" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="43" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:16" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>30</v>
@@ -4634,37 +4632,37 @@
         <v>109</v>
       </c>
       <c r="H43" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="I43" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="I43" s="2" t="s">
+      <c r="J43" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="K43" s="2" t="s">
         <v>337</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>338</v>
       </c>
       <c r="L43" s="2" t="s">
         <v>139</v>
       </c>
       <c r="M43" s="2"/>
       <c r="N43" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="O43" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="P43" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="O43" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="P43" s="3" t="s">
-        <v>265</v>
-      </c>
     </row>
-    <row r="44" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A44" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>42</v>
@@ -4682,36 +4680,36 @@
         <v>109</v>
       </c>
       <c r="H44" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="I44" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="I44" s="2" t="s">
-        <v>341</v>
-      </c>
       <c r="J44" s="2" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="K44" s="2" t="s">
         <v>113</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="N44" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="O44" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="P44" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="O44" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="P44" s="3" t="s">
-        <v>265</v>
-      </c>
     </row>
-    <row r="45" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A45" s="6" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>42</v>
@@ -4729,44 +4727,44 @@
         <v>109</v>
       </c>
       <c r="H45" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="I45" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="I45" s="2" t="s">
-        <v>345</v>
-      </c>
       <c r="J45" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="K45" s="2" t="s">
         <v>113</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="N45" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="O45" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="P45" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="O45" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="P45" s="3" t="s">
-        <v>265</v>
-      </c>
     </row>
-    <row r="46" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A46" s="6" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
-    <row r="47" spans="1:16" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.45">
       <c r="A47" s="8" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C47" t="s">
         <v>42</v>
@@ -4802,17 +4800,23 @@
         <v>146</v>
       </c>
       <c r="N47" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="O47" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P47" s="3" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P47" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:P47" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="Jour1_Sequence4"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>

</xml_diff>